<commit_message>
Add proposed base DIY assortment for the unattended store
184 items in 19 sections; 134 backed by store 1 sales data, 50 added
from hardware/garden and emergency needs outside the export. Adds a
sheet to the workbook, a CSV, the generating script and a README section.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01H9fdgZQbPRfobYczG68Y19
</commit_message>
<xml_diff>
--- a/analyzy/bezobsluzny-obchod/sortiment_24-7_analyza.xlsx
+++ b/analyzy/bezobsluzny-obchod/sortiment_24-7_analyza.xlsx
@@ -7,9 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Skupiny" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Kandidatni polozky" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Metodika" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Zakladni sortiment" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Skupiny" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Kandidatni polozky" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Metodika" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -415,6 +416,3810 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E185"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="55" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Sekce</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Položka</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Cena Kč</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Prodej Solnice ks/měs</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Poznámka</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Baterie</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>AA alkalická po kuse (Panasonic)</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D2" t="n">
+        <v>46</v>
+      </c>
+      <c r="E2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Baterie</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>AA alkalická 10 ks (GETI)</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>120</v>
+      </c>
+      <c r="D3" t="n">
+        <v>73</v>
+      </c>
+      <c r="E3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Baterie</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>AAA alkalická po kuse</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>25</v>
+      </c>
+      <c r="D4" t="n">
+        <v>43</v>
+      </c>
+      <c r="E4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Baterie</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>AAA alkalická 10 ks</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>120</v>
+      </c>
+      <c r="D5" t="n">
+        <v>41</v>
+      </c>
+      <c r="E5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Baterie</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>CR2032 knoflíková</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>45</v>
+      </c>
+      <c r="D6" t="n">
+        <v>38</v>
+      </c>
+      <c r="E6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Baterie</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>CR2025 knoflíková</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>39</v>
+      </c>
+      <c r="D7" t="n">
+        <v>6</v>
+      </c>
+      <c r="E7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Baterie</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>C / LR14 (2 ks)</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>39</v>
+      </c>
+      <c r="D8" t="n">
+        <v>14</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>zinkové R14 + alkalické LR14</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Baterie</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>D / LR20 (2 ks)</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>60</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>svítilny, plynové kotle</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Baterie</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>9V blok 6LR61</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>60</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>kouřové hlásiče</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Baterie</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>A23 12V</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>39</v>
+      </c>
+      <c r="D11" t="n">
+        <v>7</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>dálkové ovladače vrat</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Baterie</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>LR44 / A76</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>25</v>
+      </c>
+      <c r="D12" t="n">
+        <v>6</v>
+      </c>
+      <c r="E12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Baterie</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>PR312 do naslouchátek</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>18</v>
+      </c>
+      <c r="D13" t="n">
+        <v>6</v>
+      </c>
+      <c r="E13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Baterie</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Lithium AA (2 ks)</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>74</v>
+      </c>
+      <c r="D14" t="n">
+        <v>10</v>
+      </c>
+      <c r="E14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Žárovky a svítidla</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>LED E27 8–10 W teplá bílá</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>89</v>
+      </c>
+      <c r="D15" t="n">
+        <v>8</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>nahrazuje 60 W</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Žárovky a svítidla</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>LED E27 13–15 W teplá bílá</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>119</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>nahrazuje 100 W</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Žárovky a svítidla</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>LED E14 svíčka 5–6 W</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>79</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>klasické E14 25/40 W se prodávají 10 ks/měs</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Žárovky a svítidla</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Žárovka E27 40 W / 60 W (tes-lamp, klasik)</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>20</v>
+      </c>
+      <c r="D18" t="n">
+        <v>21</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>dokud je dostupná</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Žárovky a svítidla</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Žárovka E14 svíčka 25 W / 40 W</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>20</v>
+      </c>
+      <c r="D19" t="n">
+        <v>10</v>
+      </c>
+      <c r="E19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Žárovky a svítidla</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>GU10 LED 5 W</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>69</v>
+      </c>
+      <c r="D20" t="n">
+        <v>5</v>
+      </c>
+      <c r="E20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Žárovky a svítidla</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>G9 halogen / LED</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>39</v>
+      </c>
+      <c r="D21" t="n">
+        <v>14</v>
+      </c>
+      <c r="E21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Žárovky a svítidla</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Reflektor R50 E14 40 W</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>39</v>
+      </c>
+      <c r="D22" t="n">
+        <v>3</v>
+      </c>
+      <c r="E22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Žárovky a svítidla</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>LED trubice 120 cm T8</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>149</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>garáže, dílny</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Žárovky a svítidla</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Startér do zářivky S2/S10</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>15</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Žárovky a svítidla</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Svítilna / čelovka LED na AA/AAA</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>119</v>
+      </c>
+      <c r="D25" t="n">
+        <v>5</v>
+      </c>
+      <c r="E25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Elektroinstalace</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>WAGO 221-412 (2×4 mm) s páčkou</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>13</v>
+      </c>
+      <c r="D26" t="n">
+        <v>15</v>
+      </c>
+      <c r="E26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Elektroinstalace</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>WAGO 221-413 (3×4 mm) s páčkou</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>16</v>
+      </c>
+      <c r="D27" t="n">
+        <v>30</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>nejprodávanější</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Elektroinstalace</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>WAGO 221-415 (5×4 mm) s páčkou</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>20</v>
+      </c>
+      <c r="D28" t="n">
+        <v>5</v>
+      </c>
+      <c r="E28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Elektroinstalace</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>WAGO 2273-203 (3×2,5 mm)</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>6</v>
+      </c>
+      <c r="D29" t="n">
+        <v>21</v>
+      </c>
+      <c r="E29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Elektroinstalace</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>WAGO 2273-204 (4×2,5 mm)</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>8</v>
+      </c>
+      <c r="D30" t="n">
+        <v>20</v>
+      </c>
+      <c r="E30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Elektroinstalace</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Pojistky přístrojové 5×20 mm – sada hodnot</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>9</v>
+      </c>
+      <c r="D31" t="n">
+        <v>17</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>prodávat v sadě 10 ks</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Elektroinstalace</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Pojistka 16 A válcová</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>25</v>
+      </c>
+      <c r="D32" t="n">
+        <v>6</v>
+      </c>
+      <c r="E32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Elektroinstalace</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Vidlice úhlová bílá</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>53</v>
+      </c>
+      <c r="D33" t="n">
+        <v>7</v>
+      </c>
+      <c r="E33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Elektroinstalace</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Vidlice gumová IP44 černá</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>109</v>
+      </c>
+      <c r="D34" t="n">
+        <v>6</v>
+      </c>
+      <c r="E34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Elektroinstalace</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Zásuvka pohyblivá (na kabel) bílá / gumová</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>60</v>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Elektroinstalace</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Prodlužovací kabel 3 zásuvky, 3 m a 5 m</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>199</v>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>nejčastější nouzový nákup elektro</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Elektroinstalace</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Prodlužovací kabel 1 zásuvka 10 m (zahradní)</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>299</v>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Elektroinstalace</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Spínač jednopólový + zásuvka nástěnná (Tango/Classic)</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>91</v>
+      </c>
+      <c r="D38" t="n">
+        <v>4</v>
+      </c>
+      <c r="E38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Elektroinstalace</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Instalační krabice KU 68 (do zdi) a do SDK</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>8</v>
+      </c>
+      <c r="D39" t="n">
+        <v>15</v>
+      </c>
+      <c r="E39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Elektroinstalace</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Svorkovnice 12pól. 2,5 mm</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>25</v>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Elektroinstalace</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Husí krk 16 / 23 mm (návin 5 m)</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>80</v>
+      </c>
+      <c r="D41" t="n">
+        <v>26</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>v datech na metry</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Elektroinstalace</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Lišta vkládací 17×17 mm 2 m</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>66</v>
+      </c>
+      <c r="D42" t="n">
+        <v>5</v>
+      </c>
+      <c r="E42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Elektroinstalace</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Faston zdířky 6,3 mm (sáček 20 ks)</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>30</v>
+      </c>
+      <c r="D43" t="n">
+        <v>14</v>
+      </c>
+      <c r="E43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Elektroinstalace</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Zvonek bezdrátový / bateriový tlačítko</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>249</v>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Kabely (předbalené náviny)</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>CYSY 3G×1,5 návin 5 m a 10 m</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>160</v>
+      </c>
+      <c r="D45" t="n">
+        <v>72</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>v datech 72 m/měs po metrech</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Kabely (předbalené náviny)</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>CYKY 3×2,5 návin 10 m</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>380</v>
+      </c>
+      <c r="D46" t="n">
+        <v>49</v>
+      </c>
+      <c r="E46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Kabely (předbalené náviny)</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>CYKY 3×1,5 návin 10 m</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>280</v>
+      </c>
+      <c r="D47" t="n">
+        <v>30</v>
+      </c>
+      <c r="E47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Kabely (předbalené náviny)</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>CYSY 2×1 návin 5 m</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>85</v>
+      </c>
+      <c r="D48" t="n">
+        <v>33</v>
+      </c>
+      <c r="E48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Kabely (předbalené náviny)</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>CYSY 3G×1 návin 5 m</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>105</v>
+      </c>
+      <c r="D49" t="n">
+        <v>12</v>
+      </c>
+      <c r="E49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Kabely (předbalené náviny)</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Dvojlinka 2×0,75 návin 20 m</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>60</v>
+      </c>
+      <c r="D50" t="n">
+        <v>22</v>
+      </c>
+      <c r="E50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Pásky</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Maskovací páska TX 25 mm 50 m</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>59</v>
+      </c>
+      <c r="D51" t="n">
+        <v>72</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>marže 144 %</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Pásky</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Maskovací páska TX 30 / 38 / 48 mm</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>50</v>
+      </c>
+      <c r="D52" t="n">
+        <v>25</v>
+      </c>
+      <c r="E52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Pásky</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Krepová páska 50 mm 50 m (60 °C)</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>76</v>
+      </c>
+      <c r="D53" t="n">
+        <v>7</v>
+      </c>
+      <c r="E53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Pásky</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Izolační páska 15 mm černá + sada barev</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>12</v>
+      </c>
+      <c r="D54" t="n">
+        <v>14</v>
+      </c>
+      <c r="E54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Pásky</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Izolační páska 25 mm</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>22</v>
+      </c>
+      <c r="D55" t="n">
+        <v>6</v>
+      </c>
+      <c r="E55" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Pásky</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Teflonová páska 12 mm</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>22</v>
+      </c>
+      <c r="D56" t="n">
+        <v>6</v>
+      </c>
+      <c r="E56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Pásky</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Balicí páska 48 mm 66 m</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>55</v>
+      </c>
+      <c r="D57" t="n">
+        <v>6</v>
+      </c>
+      <c r="E57" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Pásky</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Univerzální textilní (duct) páska 50 mm</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>145</v>
+      </c>
+      <c r="D58" t="n">
+        <v>5</v>
+      </c>
+      <c r="E58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Pásky</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Oboustranná montážní páska</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>89</v>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Pásky</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Stahovací pásky 200 mm a 300 mm (50 ks)</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>50</v>
+      </c>
+      <c r="D60" t="n">
+        <v>8</v>
+      </c>
+      <c r="E60" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Lepidla, tmely, pěny</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Mamut Glue High tack 290 ml bílý</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>199</v>
+      </c>
+      <c r="D61" t="n">
+        <v>26</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>nosná položka</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Lepidla, tmely, pěny</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Mamut Glue Crystal transparent 290 ml</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>235</v>
+      </c>
+      <c r="D62" t="n">
+        <v>4</v>
+      </c>
+      <c r="E62" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Lepidla, tmely, pěny</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Mamut Glue 25 ml (tuba)</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>75</v>
+      </c>
+      <c r="D63" t="n">
+        <v>5</v>
+      </c>
+      <c r="E63" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Lepidla, tmely, pěny</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Sekundové lepidlo 3 g (Loctite)</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>53</v>
+      </c>
+      <c r="D64" t="n">
+        <v>3</v>
+      </c>
+      <c r="E64" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Lepidla, tmely, pěny</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Herkules / Chemoprén univerzál 50–120 g</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>60</v>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Lepidla, tmely, pěny</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Sanitární silikon 280 ml bílý a transparent</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>155</v>
+      </c>
+      <c r="D66" t="n">
+        <v>13</v>
+      </c>
+      <c r="E66" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Lepidla, tmely, pěny</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Akryl bílý 310 ml</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>95</v>
+      </c>
+      <c r="D67" t="n">
+        <v>5</v>
+      </c>
+      <c r="E67" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Lepidla, tmely, pěny</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Montážní pěna trubičková 750 ml</t>
+        </is>
+      </c>
+      <c r="C68" t="n">
+        <v>169</v>
+      </c>
+      <c r="D68" t="n">
+        <v>4</v>
+      </c>
+      <c r="E68" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Lepidla, tmely, pěny</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Pěna 500 ml s aplikátorem (Pattex Control)</t>
+        </is>
+      </c>
+      <c r="C69" t="n">
+        <v>169</v>
+      </c>
+      <c r="D69" t="n">
+        <v>6</v>
+      </c>
+      <c r="E69" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Lepidla, tmely, pěny</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Pistole na kartuše</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
+        <v>99</v>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>bez ní se silikon neprodá</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Lepidla, tmely, pěny</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Aplikační špičky na kartuše 5 ks</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>44</v>
+      </c>
+      <c r="D71" t="n">
+        <v>4</v>
+      </c>
+      <c r="E71" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Lepidla, tmely, pěny</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Tmel na dřevo 250 g (smrk, dub)</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>62</v>
+      </c>
+      <c r="D72" t="n">
+        <v>5</v>
+      </c>
+      <c r="E72" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Lepidla, tmely, pěny</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Sádra bílá 1 kg a 3 kg</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>45</v>
+      </c>
+      <c r="D73" t="n">
+        <v>10</v>
+      </c>
+      <c r="E73" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Lepidla, tmely, pěny</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Univerzální štukový tmel 400 g (Uniflex)</t>
+        </is>
+      </c>
+      <c r="C74" t="n">
+        <v>65</v>
+      </c>
+      <c r="D74" t="n">
+        <v>3</v>
+      </c>
+      <c r="E74" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Malířské potřeby</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Zakrývací fólie 4×5 m</t>
+        </is>
+      </c>
+      <c r="C75" t="n">
+        <v>25</v>
+      </c>
+      <c r="D75" t="n">
+        <v>63</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>nejprodávanější kus prodejny</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Malířské potřeby</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Zakrývací plachta 4×12,5 m</t>
+        </is>
+      </c>
+      <c r="C76" t="n">
+        <v>55</v>
+      </c>
+      <c r="D76" t="n">
+        <v>16</v>
+      </c>
+      <c r="E76" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Malířské potřeby</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Štětec plochý 40 / 50 / 70 mm</t>
+        </is>
+      </c>
+      <c r="C77" t="n">
+        <v>37</v>
+      </c>
+      <c r="D77" t="n">
+        <v>26</v>
+      </c>
+      <c r="E77" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Malířské potřeby</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Váleček velvet 10 cm + držadlo</t>
+        </is>
+      </c>
+      <c r="C78" t="n">
+        <v>22</v>
+      </c>
+      <c r="D78" t="n">
+        <v>10</v>
+      </c>
+      <c r="E78" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Malířské potřeby</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Váleček 18 / 25 cm + rukojeť</t>
+        </is>
+      </c>
+      <c r="C79" t="n">
+        <v>90</v>
+      </c>
+      <c r="D79" t="n">
+        <v>9</v>
+      </c>
+      <c r="E79" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Malířské potřeby</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Malířská mřížka / vanička</t>
+        </is>
+      </c>
+      <c r="C80" t="n">
+        <v>39</v>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Malířské potřeby</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Brusné plátno 60 / 80 / 120</t>
+        </is>
+      </c>
+      <c r="C81" t="n">
+        <v>17</v>
+      </c>
+      <c r="D81" t="n">
+        <v>35</v>
+      </c>
+      <c r="E81" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Malířské potřeby</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Brusný papír pod vodu 600 / 800</t>
+        </is>
+      </c>
+      <c r="C82" t="n">
+        <v>15</v>
+      </c>
+      <c r="D82" t="n">
+        <v>20</v>
+      </c>
+      <c r="E82" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Malířské potřeby</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Špachtle 60 mm a 100 mm</t>
+        </is>
+      </c>
+      <c r="C83" t="n">
+        <v>39</v>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Malířské potřeby</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Míchací pohár 385 ml</t>
+        </is>
+      </c>
+      <c r="C84" t="n">
+        <v>21</v>
+      </c>
+      <c r="D84" t="n">
+        <v>4</v>
+      </c>
+      <c r="E84" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Malířské potřeby</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Nopová fólie 0,5 m a 1 m × 20 m</t>
+        </is>
+      </c>
+      <c r="C85" t="n">
+        <v>38</v>
+      </c>
+      <c r="D85" t="n">
+        <v>40</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>izolace základů, silný prodej</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Malířské potřeby</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Bílá malířská barva 4 kg (Primalex/HET)</t>
+        </is>
+      </c>
+      <c r="C86" t="n">
+        <v>199</v>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>jediná barva, kterou bezobslužně držet</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Malířské potřeby</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Univerzální lazura 0,75 l ořech / teak</t>
+        </is>
+      </c>
+      <c r="C87" t="n">
+        <v>259</v>
+      </c>
+      <c r="D87" t="n">
+        <v>5</v>
+      </c>
+      <c r="E87" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Malířské potřeby</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Bochemit proti plísním 500 ml</t>
+        </is>
+      </c>
+      <c r="C88" t="n">
+        <v>99</v>
+      </c>
+      <c r="D88" t="n">
+        <v>6</v>
+      </c>
+      <c r="E88" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Vodoinstalace</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Hadicové spony 8–12 / 12–20 / 16–25 / 20–32 / 25–40 / 32–50</t>
+        </is>
+      </c>
+      <c r="C89" t="n">
+        <v>9</v>
+      </c>
+      <c r="D89" t="n">
+        <v>77</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>celá řada</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Vodoinstalace</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Objímka trubková 2-šroub 31–38 mm</t>
+        </is>
+      </c>
+      <c r="C90" t="n">
+        <v>16</v>
+      </c>
+      <c r="D90" t="n">
+        <v>25</v>
+      </c>
+      <c r="E90" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Vodoinstalace</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Objímka trubková 2-šroub 54–59 mm</t>
+        </is>
+      </c>
+      <c r="C91" t="n">
+        <v>22</v>
+      </c>
+      <c r="D91" t="n">
+        <v>14</v>
+      </c>
+      <c r="E91" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Vodoinstalace</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Příchytka na potrubí 20 / 25 mm</t>
+        </is>
+      </c>
+      <c r="C92" t="n">
+        <v>8</v>
+      </c>
+      <c r="D92" t="n">
+        <v>17</v>
+      </c>
+      <c r="E92" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Vodoinstalace</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>PPR koleno 90° 20 mm, T-kus 20, nátrubek 20</t>
+        </is>
+      </c>
+      <c r="C93" t="n">
+        <v>8</v>
+      </c>
+      <c r="D93" t="n">
+        <v>15</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>jen dimenze 20 a 25</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Vodoinstalace</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Mosazná vsuvka 3/4", 1/2"</t>
+        </is>
+      </c>
+      <c r="C94" t="n">
+        <v>48</v>
+      </c>
+      <c r="D94" t="n">
+        <v>9</v>
+      </c>
+      <c r="E94" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Vodoinstalace</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Tubex izolace 20×10 mm (2 m)</t>
+        </is>
+      </c>
+      <c r="C95" t="n">
+        <v>12</v>
+      </c>
+      <c r="D95" t="n">
+        <v>14</v>
+      </c>
+      <c r="E95" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Vodoinstalace</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Těsnění gumová sada 1/2"–3/4"</t>
+        </is>
+      </c>
+      <c r="C96" t="n">
+        <v>25</v>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>nejčastější havárie</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Vodoinstalace</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Flexi hadička 3/8" 30–50 cm</t>
+        </is>
+      </c>
+      <c r="C97" t="n">
+        <v>79</v>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Vodoinstalace</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Perlátor M22/M24</t>
+        </is>
+      </c>
+      <c r="C98" t="n">
+        <v>39</v>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Vodoinstalace</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Sprchová hadice 150 cm</t>
+        </is>
+      </c>
+      <c r="C99" t="n">
+        <v>245</v>
+      </c>
+      <c r="D99" t="n">
+        <v>3</v>
+      </c>
+      <c r="E99" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Vodoinstalace</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Sifon umyvadlový plast</t>
+        </is>
+      </c>
+      <c r="C100" t="n">
+        <v>89</v>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr"/>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Vodoinstalace</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Zahradní hadice 1/2" 20 m + rychlospojky</t>
+        </is>
+      </c>
+      <c r="C101" t="n">
+        <v>399</v>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>ověřit z dat prodejny 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Spojovací materiál (blistry)</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Hmoždinky 6 / 8 / 10 mm (sady)</t>
+        </is>
+      </c>
+      <c r="C102" t="n">
+        <v>39</v>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>v datech kusový prodej</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Spojovací materiál (blistry)</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Vruty univerzální 4×40, 4×50, 5×60 (sady)</t>
+        </is>
+      </c>
+      <c r="C103" t="n">
+        <v>59</v>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr"/>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Spojovací materiál (blistry)</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Šrouby do plechu 2,9×13 (sada 50 ks)</t>
+        </is>
+      </c>
+      <c r="C104" t="n">
+        <v>29</v>
+      </c>
+      <c r="D104" t="n">
+        <v>37</v>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>v datech 37 ks/měs po 0,40 Kč</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Spojovací materiál (blistry)</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Hřebíky 40 / 60 / 80 mm (sáček)</t>
+        </is>
+      </c>
+      <c r="C105" t="n">
+        <v>39</v>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr"/>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Spojovací materiál (blistry)</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Skoby, háčky, oka (sada)</t>
+        </is>
+      </c>
+      <c r="C106" t="n">
+        <v>39</v>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr"/>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Spojovací materiál (blistry)</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Hmoždinka rámová 10×100 (sada)</t>
+        </is>
+      </c>
+      <c r="C107" t="n">
+        <v>79</v>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr"/>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Spojovací materiál (blistry)</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Vázací drát pozink</t>
+        </is>
+      </c>
+      <c r="C108" t="n">
+        <v>49</v>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr"/>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Spojovací materiál (blistry)</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Zárohák (hák do zdi)</t>
+        </is>
+      </c>
+      <c r="C109" t="n">
+        <v>69</v>
+      </c>
+      <c r="D109" t="n">
+        <v>5</v>
+      </c>
+      <c r="E109" t="inlineStr"/>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Ruční nářadí</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Svinovací metr 5 m</t>
+        </is>
+      </c>
+      <c r="C110" t="n">
+        <v>99</v>
+      </c>
+      <c r="D110" t="n">
+        <v>9</v>
+      </c>
+      <c r="E110" t="inlineStr"/>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Ruční nářadí</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Odlamovací nůž 18 mm kovový</t>
+        </is>
+      </c>
+      <c r="C111" t="n">
+        <v>89</v>
+      </c>
+      <c r="D111" t="n">
+        <v>7</v>
+      </c>
+      <c r="E111" t="inlineStr"/>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Ruční nářadí</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Náhradní čepele 18 mm 10 ks</t>
+        </is>
+      </c>
+      <c r="C112" t="n">
+        <v>40</v>
+      </c>
+      <c r="D112" t="n">
+        <v>12</v>
+      </c>
+      <c r="E112" t="inlineStr"/>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Ruční nářadí</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Šroubovák s bity (ráčna + 20 bitů)</t>
+        </is>
+      </c>
+      <c r="C113" t="n">
+        <v>199</v>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Ruční nářadí</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Kleště kombinované 180 mm</t>
+        </is>
+      </c>
+      <c r="C114" t="n">
+        <v>149</v>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Ruční nářadí</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Kladivo 300 g</t>
+        </is>
+      </c>
+      <c r="C115" t="n">
+        <v>129</v>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr"/>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Ruční nářadí</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Ocelový kartáč 5řadý</t>
+        </is>
+      </c>
+      <c r="C116" t="n">
+        <v>68</v>
+      </c>
+      <c r="D116" t="n">
+        <v>5</v>
+      </c>
+      <c r="E116" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Ruční nářadí</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Pilka na kov / pilový list</t>
+        </is>
+      </c>
+      <c r="C117" t="n">
+        <v>99</v>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Ruční nářadí</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Vodováha 40 cm</t>
+        </is>
+      </c>
+      <c r="C118" t="n">
+        <v>99</v>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Ruční nářadí</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Sada imbus klíčů</t>
+        </is>
+      </c>
+      <c r="C119" t="n">
+        <v>89</v>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr"/>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>Ruční nářadí</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Zavírací nůž</t>
+        </is>
+      </c>
+      <c r="C120" t="n">
+        <v>163</v>
+      </c>
+      <c r="D120" t="n">
+        <v>4</v>
+      </c>
+      <c r="E120" t="inlineStr"/>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Ruční nářadí</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Vědro stavební 12 l</t>
+        </is>
+      </c>
+      <c r="C121" t="n">
+        <v>49</v>
+      </c>
+      <c r="D121" t="n">
+        <v>6</v>
+      </c>
+      <c r="E121" t="inlineStr"/>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>Ochranné pomůcky</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Pracovní rukavice vel. 8 / 9 / 10 / 11</t>
+        </is>
+      </c>
+      <c r="C122" t="n">
+        <v>59</v>
+      </c>
+      <c r="D122" t="n">
+        <v>30</v>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>celá řada velikostí</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Ochranné pomůcky</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Rukavice profi 1+1</t>
+        </is>
+      </c>
+      <c r="C123" t="n">
+        <v>28</v>
+      </c>
+      <c r="D123" t="n">
+        <v>5</v>
+      </c>
+      <c r="E123" t="inlineStr"/>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Ochranné pomůcky</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Jednorázové nitrilové rukavice (10 ks)</t>
+        </is>
+      </c>
+      <c r="C124" t="n">
+        <v>39</v>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr"/>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>Ochranné pomůcky</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Zátky do uší</t>
+        </is>
+      </c>
+      <c r="C125" t="n">
+        <v>10</v>
+      </c>
+      <c r="D125" t="n">
+        <v>3</v>
+      </c>
+      <c r="E125" t="inlineStr"/>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>Ochranné pomůcky</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Respirátor FFP2 (2 ks)</t>
+        </is>
+      </c>
+      <c r="C126" t="n">
+        <v>39</v>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>broušení, barvy</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>Ochranné pomůcky</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Ochranné brýle</t>
+        </is>
+      </c>
+      <c r="C127" t="n">
+        <v>49</v>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr"/>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>Technická chemie</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Ředidlo S6006 0,7 l</t>
+        </is>
+      </c>
+      <c r="C128" t="n">
+        <v>85</v>
+      </c>
+      <c r="D128" t="n">
+        <v>21</v>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>hořlavina – ověřit požární předpisy</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>Technická chemie</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Ředidlo S6005 0,7 l</t>
+        </is>
+      </c>
+      <c r="C129" t="n">
+        <v>95</v>
+      </c>
+      <c r="D129" t="n">
+        <v>12</v>
+      </c>
+      <c r="E129" t="inlineStr"/>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>Technická chemie</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Nitroředidlo C6000 0,7 l</t>
+        </is>
+      </c>
+      <c r="C130" t="n">
+        <v>95</v>
+      </c>
+      <c r="D130" t="n">
+        <v>9</v>
+      </c>
+      <c r="E130" t="inlineStr"/>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>Technická chemie</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Líh technický 0,7 l</t>
+        </is>
+      </c>
+      <c r="C131" t="n">
+        <v>98</v>
+      </c>
+      <c r="D131" t="n">
+        <v>7</v>
+      </c>
+      <c r="E131" t="inlineStr"/>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>Technická chemie</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Lakový benzín 0,7 l</t>
+        </is>
+      </c>
+      <c r="C132" t="n">
+        <v>109</v>
+      </c>
+      <c r="D132" t="n">
+        <v>4</v>
+      </c>
+      <c r="E132" t="inlineStr"/>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>Technická chemie</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>WD-40 / univerzální mazivo sprej 200 ml</t>
+        </is>
+      </c>
+      <c r="C133" t="n">
+        <v>129</v>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr"/>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>Technická chemie</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Odrezovač 0,5 l</t>
+        </is>
+      </c>
+      <c r="C134" t="n">
+        <v>112</v>
+      </c>
+      <c r="D134" t="n">
+        <v>3</v>
+      </c>
+      <c r="E134" t="inlineStr"/>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>Technická chemie</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Kyselina citronová 100 g</t>
+        </is>
+      </c>
+      <c r="C135" t="n">
+        <v>22</v>
+      </c>
+      <c r="D135" t="n">
+        <v>6</v>
+      </c>
+      <c r="E135" t="inlineStr"/>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>Technická chemie</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Vazelína bílá</t>
+        </is>
+      </c>
+      <c r="C136" t="n">
+        <v>195</v>
+      </c>
+      <c r="D136" t="n">
+        <v>4</v>
+      </c>
+      <c r="E136" t="inlineStr"/>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>Technická chemie</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Destilovaná voda 5 l</t>
+        </is>
+      </c>
+      <c r="C137" t="n">
+        <v>70</v>
+      </c>
+      <c r="D137" t="n">
+        <v>6</v>
+      </c>
+      <c r="E137" t="inlineStr"/>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>Technická chemie</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Nemrznoucí směs do ostřikovačů 3 l</t>
+        </is>
+      </c>
+      <c r="C138" t="n">
+        <v>99</v>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>sezónně</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>Úklid</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Savo Original 1,2 l</t>
+        </is>
+      </c>
+      <c r="C139" t="n">
+        <v>67</v>
+      </c>
+      <c r="D139" t="n">
+        <v>5</v>
+      </c>
+      <c r="E139" t="inlineStr"/>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>Úklid</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Savo proti plísni 500 ml</t>
+        </is>
+      </c>
+      <c r="C140" t="n">
+        <v>99</v>
+      </c>
+      <c r="D140" t="n">
+        <v>5</v>
+      </c>
+      <c r="E140" t="inlineStr"/>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>Úklid</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Domestos 750 ml / 2 l</t>
+        </is>
+      </c>
+      <c r="C141" t="n">
+        <v>59</v>
+      </c>
+      <c r="D141" t="n">
+        <v>10</v>
+      </c>
+      <c r="E141" t="inlineStr"/>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>Úklid</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Jar / prostředek na nádobí 900 ml</t>
+        </is>
+      </c>
+      <c r="C142" t="n">
+        <v>59</v>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr"/>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>Úklid</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>Univerzální čistič (Ajax, Cif)</t>
+        </is>
+      </c>
+      <c r="C143" t="n">
+        <v>59</v>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr"/>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>Úklid</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Pytle na odpad 60 l a 120 l</t>
+        </is>
+      </c>
+      <c r="C144" t="n">
+        <v>39</v>
+      </c>
+      <c r="D144" t="n">
+        <v>11</v>
+      </c>
+      <c r="E144" t="inlineStr"/>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>Úklid</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Houbičky na nádobí 5 ks</t>
+        </is>
+      </c>
+      <c r="C145" t="n">
+        <v>25</v>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr"/>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>Úklid</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Hadr podlahový</t>
+        </is>
+      </c>
+      <c r="C146" t="n">
+        <v>32</v>
+      </c>
+      <c r="D146" t="n">
+        <v>4</v>
+      </c>
+      <c r="E146" t="inlineStr"/>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>Úklid</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Osvěžovač vzduchu</t>
+        </is>
+      </c>
+      <c r="C147" t="n">
+        <v>29</v>
+      </c>
+      <c r="D147" t="n">
+        <v>9</v>
+      </c>
+      <c r="E147" t="inlineStr"/>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>Úklid</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Solvina / Praganda (mycí pasta na ruce)</t>
+        </is>
+      </c>
+      <c r="C148" t="n">
+        <v>20</v>
+      </c>
+      <c r="D148" t="n">
+        <v>15</v>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>typicky DIY</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>Úklid</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>WC blok</t>
+        </is>
+      </c>
+      <c r="C149" t="n">
+        <v>39</v>
+      </c>
+      <c r="D149" t="n">
+        <v>5</v>
+      </c>
+      <c r="E149" t="inlineStr"/>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>Úklid</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Lopatka + smetáček</t>
+        </is>
+      </c>
+      <c r="C150" t="n">
+        <v>49</v>
+      </c>
+      <c r="D150" t="n">
+        <v>6</v>
+      </c>
+      <c r="E150" t="inlineStr"/>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>Úklid</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Zamražovací / svačinové sáčky</t>
+        </is>
+      </c>
+      <c r="C151" t="n">
+        <v>39</v>
+      </c>
+      <c r="D151" t="n">
+        <v>4</v>
+      </c>
+      <c r="E151" t="inlineStr"/>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>Hygiena</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Toaletní papír Jumbo / 8 rolí</t>
+        </is>
+      </c>
+      <c r="C152" t="n">
+        <v>39</v>
+      </c>
+      <c r="D152" t="n">
+        <v>30</v>
+      </c>
+      <c r="E152" t="inlineStr"/>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>Hygiena</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>Papírové ručníky ZZ</t>
+        </is>
+      </c>
+      <c r="C153" t="n">
+        <v>45</v>
+      </c>
+      <c r="D153" t="n">
+        <v>15</v>
+      </c>
+      <c r="E153" t="inlineStr"/>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>Hygiena</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Kapesníky krabička 150 ks</t>
+        </is>
+      </c>
+      <c r="C154" t="n">
+        <v>38</v>
+      </c>
+      <c r="D154" t="n">
+        <v>3</v>
+      </c>
+      <c r="E154" t="inlineStr"/>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>Hygiena</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Kuchyňské utěrky 2 role</t>
+        </is>
+      </c>
+      <c r="C155" t="n">
+        <v>39</v>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr"/>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>Hubení škůdců</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Pastička na myši dřevo / kov</t>
+        </is>
+      </c>
+      <c r="C156" t="n">
+        <v>16</v>
+      </c>
+      <c r="D156" t="n">
+        <v>12</v>
+      </c>
+      <c r="E156" t="inlineStr"/>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>Hubení škůdců</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Nástraha na myši Ratimor 150 g</t>
+        </is>
+      </c>
+      <c r="C157" t="n">
+        <v>42</v>
+      </c>
+      <c r="D157" t="n">
+        <v>8</v>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>balení pro veřejnost</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>Hubení škůdců</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Lepová deska na myši</t>
+        </is>
+      </c>
+      <c r="C158" t="n">
+        <v>35</v>
+      </c>
+      <c r="D158" t="n">
+        <v>3</v>
+      </c>
+      <c r="E158" t="inlineStr"/>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>Hubení škůdců</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Mucholapka</t>
+        </is>
+      </c>
+      <c r="C159" t="n">
+        <v>7</v>
+      </c>
+      <c r="D159" t="n">
+        <v>4</v>
+      </c>
+      <c r="E159" t="inlineStr"/>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>Hubení škůdců</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Feroset – lapač moučných molů</t>
+        </is>
+      </c>
+      <c r="C160" t="n">
+        <v>16</v>
+      </c>
+      <c r="D160" t="n">
+        <v>8</v>
+      </c>
+      <c r="E160" t="inlineStr"/>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>Hubení škůdců</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Sprej na vosy / hmyz (Biolit)</t>
+        </is>
+      </c>
+      <c r="C161" t="n">
+        <v>119</v>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>léto</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>Hubení škůdců</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Proti mravencům (Bioformatox)</t>
+        </is>
+      </c>
+      <c r="C162" t="n">
+        <v>109</v>
+      </c>
+      <c r="D162" t="n">
+        <v>2</v>
+      </c>
+      <c r="E162" t="inlineStr"/>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>Topení a zapalování</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Pepo pevný podpalovač 40 ks</t>
+        </is>
+      </c>
+      <c r="C163" t="n">
+        <v>35</v>
+      </c>
+      <c r="D163" t="n">
+        <v>29</v>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>celoročně</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>Topení a zapalování</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>Tekutý podpalovač 1 l</t>
+        </is>
+      </c>
+      <c r="C164" t="n">
+        <v>96</v>
+      </c>
+      <c r="D164" t="n">
+        <v>3</v>
+      </c>
+      <c r="E164" t="inlineStr"/>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>Topení a zapalování</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>Zapalovač kuchyňský dlouhý</t>
+        </is>
+      </c>
+      <c r="C165" t="n">
+        <v>37</v>
+      </c>
+      <c r="D165" t="n">
+        <v>3</v>
+      </c>
+      <c r="E165" t="inlineStr"/>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>Topení a zapalování</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>Zapalovače turbo (2 ks)</t>
+        </is>
+      </c>
+      <c r="C166" t="n">
+        <v>15</v>
+      </c>
+      <c r="D166" t="n">
+        <v>4</v>
+      </c>
+      <c r="E166" t="inlineStr"/>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>Topení a zapalování</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>Zápalky (balení 10 krabiček)</t>
+        </is>
+      </c>
+      <c r="C167" t="n">
+        <v>25</v>
+      </c>
+      <c r="D167" t="n">
+        <v>2</v>
+      </c>
+      <c r="E167" t="inlineStr"/>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>Topení a zapalování</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>Dřevěné uhlí 2,5 kg</t>
+        </is>
+      </c>
+      <c r="C168" t="n">
+        <v>112</v>
+      </c>
+      <c r="D168" t="n">
+        <v>3</v>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>sezónně</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>Svíčky</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>Hřbitovní patrona 120 g a 180 g</t>
+        </is>
+      </c>
+      <c r="C169" t="n">
+        <v>28</v>
+      </c>
+      <c r="D169" t="n">
+        <v>18</v>
+      </c>
+      <c r="E169" t="inlineStr"/>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>Svíčky</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>Svíčka Theresia 4,5 dne</t>
+        </is>
+      </c>
+      <c r="C170" t="n">
+        <v>47</v>
+      </c>
+      <c r="D170" t="n">
+        <v>3</v>
+      </c>
+      <c r="E170" t="inlineStr"/>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>Svíčky</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>Iluminační svíčky 10 ks</t>
+        </is>
+      </c>
+      <c r="C171" t="n">
+        <v>59</v>
+      </c>
+      <c r="D171" t="n">
+        <v>3</v>
+      </c>
+      <c r="E171" t="inlineStr"/>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>Svíčky</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>Čajové svíčky 30 ks</t>
+        </is>
+      </c>
+      <c r="C172" t="n">
+        <v>49</v>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr"/>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>Domácnost</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>Skřipce záclonové</t>
+        </is>
+      </c>
+      <c r="C173" t="n">
+        <v>6</v>
+      </c>
+      <c r="D173" t="n">
+        <v>22</v>
+      </c>
+      <c r="E173" t="inlineStr"/>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>Domácnost</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>Háčky samolepicí</t>
+        </is>
+      </c>
+      <c r="C174" t="n">
+        <v>30</v>
+      </c>
+      <c r="D174" t="n">
+        <v>5</v>
+      </c>
+      <c r="E174" t="inlineStr"/>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>Domácnost</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>Věšák nástěnný chrom</t>
+        </is>
+      </c>
+      <c r="C175" t="n">
+        <v>62</v>
+      </c>
+      <c r="D175" t="n">
+        <v>10</v>
+      </c>
+      <c r="E175" t="inlineStr"/>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>Domácnost</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>Kolíčky na prádlo 24 ks</t>
+        </is>
+      </c>
+      <c r="C176" t="n">
+        <v>39</v>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr"/>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>Domácnost</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>Prádelní šňůra 20 m</t>
+        </is>
+      </c>
+      <c r="C177" t="n">
+        <v>49</v>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr"/>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>Domácnost</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>Provázek / polypropylenové lano 20 m</t>
+        </is>
+      </c>
+      <c r="C178" t="n">
+        <v>59</v>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr"/>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>Domácnost</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>Kroužky na klíče + rozlišovače</t>
+        </is>
+      </c>
+      <c r="C179" t="n">
+        <v>4</v>
+      </c>
+      <c r="D179" t="n">
+        <v>46</v>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>u pokladny</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>Domácnost</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>Visací zámek 30 / 40 mm</t>
+        </is>
+      </c>
+      <c r="C180" t="n">
+        <v>129</v>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr"/>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>Domácnost</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>Magnety 10 ks</t>
+        </is>
+      </c>
+      <c r="C181" t="n">
+        <v>50</v>
+      </c>
+      <c r="D181" t="n">
+        <v>3</v>
+      </c>
+      <c r="E181" t="inlineStr"/>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>Sezónní stojan (rotace)</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>Semena zeleniny a květin (stojan)</t>
+        </is>
+      </c>
+      <c r="C182" t="n">
+        <v>25</v>
+      </c>
+      <c r="D182" t="n">
+        <v>153</v>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>únor–květen, marže 40–100 %</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>Sezónní stojan (rotace)</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>Barvy na vejce, obtisky</t>
+        </is>
+      </c>
+      <c r="C183" t="n">
+        <v>12</v>
+      </c>
+      <c r="D183" t="n">
+        <v>15</v>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>březen–duben</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>Sezónní stojan (rotace)</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>Zavařovací víčka Twist, špejle, střeva</t>
+        </is>
+      </c>
+      <c r="C184" t="n">
+        <v>40</v>
+      </c>
+      <c r="D184" t="n">
+        <v>15</v>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>červenec–říjen</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>Sezónní stojan (rotace)</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>Posypová sůl 5 kg, škrabka na led</t>
+        </is>
+      </c>
+      <c r="C185" t="n">
+        <v>79</v>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>listopad–únor</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:P33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2123,8 +5928,6 @@
       <c r="L31" t="n">
         <v>0</v>
       </c>
-      <c r="M31" t="inlineStr"/>
-      <c r="N31" t="inlineStr"/>
       <c r="O31" t="n">
         <v>1</v>
       </c>
@@ -2173,8 +5976,6 @@
       <c r="L32" t="n">
         <v>0</v>
       </c>
-      <c r="M32" t="inlineStr"/>
-      <c r="N32" t="inlineStr"/>
       <c r="O32" t="n">
         <v>1</v>
       </c>
@@ -2243,7 +6044,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -23433,7 +27234,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Add turnover forecast model for the unattended store
Three scenarios with seasonality derived from 2023-2024 monthly sales,
ramp-up, shrinkage and fixed costs; break-even per scenario and a
variant as a 24/7 zone of the existing store. Adds a formula-driven
Predikce sheet to the workbook, the generating script and a README section.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01H9fdgZQbPRfobYczG68Y19
</commit_message>
<xml_diff>
--- a/analyzy/bezobsluzny-obchod/sortiment_24-7_analyza.xlsx
+++ b/analyzy/bezobsluzny-obchod/sortiment_24-7_analyza.xlsx
@@ -7,10 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Zakladni sortiment" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Skupiny" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Kandidatni polozky" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Metodika" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Predikce" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Zakladni sortiment" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Skupiny" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Kandidatni polozky" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Metodika" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,8 +20,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0%"/>
+  </numFmts>
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,13 +31,26 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -49,8 +65,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -416,6 +440,1745 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:J63"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Predikce obratu bezobslužné prodejny 24/7 (Kč bez DPH). Žluté buňky = parametry k úpravě.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Parametr</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Pesimistický</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Realistický</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Optimistický</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Základ: prodej základního sortimentu v Solnici, průměrný měsíc (Kč bez DPH)</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>119919</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>119919</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>119919</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Z listu Zakladni sortiment, 108 289 Kč v okně březen/duben, přepočteno sezónním indexem</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Faktor lokality (poptávka nového města vs. Solnice)</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Solnice = zavedená prodejna od 2012, 52 nákupů/den; nové město bez historie</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Uplift 24/7 (nákupy mimo běžnou otevírací dobu)</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="E6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Ztráty krádežemi a šlonky (% obratu)</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="E7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Obchodní marže</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="C8" s="5" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="D8" s="5" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Prodejna 1 podle exportu 38 %</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Poplatky za platby (% obratu)</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="E9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Nájem Kč/měs</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>12000</v>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>12000</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>12000</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>samostatná jednotka; při rozšíření stávající prodejny 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Energie Kč/měs</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>3000</v>
+      </c>
+      <c r="C11" s="3" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>3000</v>
+      </c>
+      <c r="E11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Technologie (vstup, samoobslužná pokladna, kamery, SW) Kč/měs</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>7000</v>
+      </c>
+      <c r="C12" s="3" t="n">
+        <v>7000</v>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>7000</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>amortizace + licence</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Doplňování zboží a úklid Kč/měs</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>8000</v>
+      </c>
+      <c r="C13" s="3" t="n">
+        <v>8000</v>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>8000</v>
+      </c>
+      <c r="E13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Pojištění Kč/měs</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C14" s="3" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E14" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>Sezónní index (tržby Drogerie 2023–24)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Měsíc</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Index</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Rozjezd rok 1</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Rozjezd: podíl plného prodeje v 1.–12. měsíci provozu (počítá se od ledna; start v jiném měsíci = posunout hodnoty)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>leden</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="C18" s="4" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>únor</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="C19" s="4" t="n">
+        <v>0.65</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>březen</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>0.843</v>
+      </c>
+      <c r="C20" s="4" t="n">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>duben</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>0.963</v>
+      </c>
+      <c r="C21" s="4" t="n">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>květen</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>1.242</v>
+      </c>
+      <c r="C22" s="4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>červen</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>1.212</v>
+      </c>
+      <c r="C23" s="4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>červenec</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>1.362</v>
+      </c>
+      <c r="C24" s="4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>srpen</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>1.284</v>
+      </c>
+      <c r="C25" s="4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>září</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>1.123</v>
+      </c>
+      <c r="C26" s="4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>říjen</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>1.036</v>
+      </c>
+      <c r="C27" s="4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>listopad</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="C28" s="4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>prosinec</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>0.918</v>
+      </c>
+      <c r="C29" s="4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="1" t="inlineStr">
+        <is>
+          <t>Měsíční predikce – ustálený rok (bez rozjezdu)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Měsíc</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Pesimistický – Obrat</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Pesimistický – Hrubý zisk po ztrátách a poplatcích</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Pesimistický – Výsledek po fixních nákladech</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Realistický – Obrat</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Realistický – Hrubý zisk po ztrátách a poplatcích</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>Realistický – Výsledek po fixních nákladech</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>Optimistický – Obrat</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>Optimistický – Hrubý zisk po ztrátách a poplatcích</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>Optimistický – Výsledek po fixních nákladech</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>leden</t>
+        </is>
+      </c>
+      <c r="B33" s="6">
+        <f>B$4*$B18*B$5*B$6</f>
+        <v/>
+      </c>
+      <c r="C33" s="6">
+        <f>B33*(B$8*(1-B$7)-B$9)</f>
+        <v/>
+      </c>
+      <c r="D33" s="6">
+        <f>C33-SUM(B$10:B$14)</f>
+        <v/>
+      </c>
+      <c r="E33" s="6">
+        <f>C$4*$B18*C$5*C$6</f>
+        <v/>
+      </c>
+      <c r="F33" s="6">
+        <f>E33*(C$8*(1-C$7)-C$9)</f>
+        <v/>
+      </c>
+      <c r="G33" s="6">
+        <f>F33-SUM(C$10:C$14)</f>
+        <v/>
+      </c>
+      <c r="H33" s="6">
+        <f>D$4*$B18*D$5*D$6</f>
+        <v/>
+      </c>
+      <c r="I33" s="6">
+        <f>H33*(D$8*(1-D$7)-D$9)</f>
+        <v/>
+      </c>
+      <c r="J33" s="6">
+        <f>I33-SUM(D$10:D$14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>únor</t>
+        </is>
+      </c>
+      <c r="B34" s="6">
+        <f>B$4*$B19*B$5*B$6</f>
+        <v/>
+      </c>
+      <c r="C34" s="6">
+        <f>B34*(B$8*(1-B$7)-B$9)</f>
+        <v/>
+      </c>
+      <c r="D34" s="6">
+        <f>C34-SUM(B$10:B$14)</f>
+        <v/>
+      </c>
+      <c r="E34" s="6">
+        <f>C$4*$B19*C$5*C$6</f>
+        <v/>
+      </c>
+      <c r="F34" s="6">
+        <f>E34*(C$8*(1-C$7)-C$9)</f>
+        <v/>
+      </c>
+      <c r="G34" s="6">
+        <f>F34-SUM(C$10:C$14)</f>
+        <v/>
+      </c>
+      <c r="H34" s="6">
+        <f>D$4*$B19*D$5*D$6</f>
+        <v/>
+      </c>
+      <c r="I34" s="6">
+        <f>H34*(D$8*(1-D$7)-D$9)</f>
+        <v/>
+      </c>
+      <c r="J34" s="6">
+        <f>I34-SUM(D$10:D$14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>březen</t>
+        </is>
+      </c>
+      <c r="B35" s="6">
+        <f>B$4*$B20*B$5*B$6</f>
+        <v/>
+      </c>
+      <c r="C35" s="6">
+        <f>B35*(B$8*(1-B$7)-B$9)</f>
+        <v/>
+      </c>
+      <c r="D35" s="6">
+        <f>C35-SUM(B$10:B$14)</f>
+        <v/>
+      </c>
+      <c r="E35" s="6">
+        <f>C$4*$B20*C$5*C$6</f>
+        <v/>
+      </c>
+      <c r="F35" s="6">
+        <f>E35*(C$8*(1-C$7)-C$9)</f>
+        <v/>
+      </c>
+      <c r="G35" s="6">
+        <f>F35-SUM(C$10:C$14)</f>
+        <v/>
+      </c>
+      <c r="H35" s="6">
+        <f>D$4*$B20*D$5*D$6</f>
+        <v/>
+      </c>
+      <c r="I35" s="6">
+        <f>H35*(D$8*(1-D$7)-D$9)</f>
+        <v/>
+      </c>
+      <c r="J35" s="6">
+        <f>I35-SUM(D$10:D$14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>duben</t>
+        </is>
+      </c>
+      <c r="B36" s="6">
+        <f>B$4*$B21*B$5*B$6</f>
+        <v/>
+      </c>
+      <c r="C36" s="6">
+        <f>B36*(B$8*(1-B$7)-B$9)</f>
+        <v/>
+      </c>
+      <c r="D36" s="6">
+        <f>C36-SUM(B$10:B$14)</f>
+        <v/>
+      </c>
+      <c r="E36" s="6">
+        <f>C$4*$B21*C$5*C$6</f>
+        <v/>
+      </c>
+      <c r="F36" s="6">
+        <f>E36*(C$8*(1-C$7)-C$9)</f>
+        <v/>
+      </c>
+      <c r="G36" s="6">
+        <f>F36-SUM(C$10:C$14)</f>
+        <v/>
+      </c>
+      <c r="H36" s="6">
+        <f>D$4*$B21*D$5*D$6</f>
+        <v/>
+      </c>
+      <c r="I36" s="6">
+        <f>H36*(D$8*(1-D$7)-D$9)</f>
+        <v/>
+      </c>
+      <c r="J36" s="6">
+        <f>I36-SUM(D$10:D$14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>květen</t>
+        </is>
+      </c>
+      <c r="B37" s="6">
+        <f>B$4*$B22*B$5*B$6</f>
+        <v/>
+      </c>
+      <c r="C37" s="6">
+        <f>B37*(B$8*(1-B$7)-B$9)</f>
+        <v/>
+      </c>
+      <c r="D37" s="6">
+        <f>C37-SUM(B$10:B$14)</f>
+        <v/>
+      </c>
+      <c r="E37" s="6">
+        <f>C$4*$B22*C$5*C$6</f>
+        <v/>
+      </c>
+      <c r="F37" s="6">
+        <f>E37*(C$8*(1-C$7)-C$9)</f>
+        <v/>
+      </c>
+      <c r="G37" s="6">
+        <f>F37-SUM(C$10:C$14)</f>
+        <v/>
+      </c>
+      <c r="H37" s="6">
+        <f>D$4*$B22*D$5*D$6</f>
+        <v/>
+      </c>
+      <c r="I37" s="6">
+        <f>H37*(D$8*(1-D$7)-D$9)</f>
+        <v/>
+      </c>
+      <c r="J37" s="6">
+        <f>I37-SUM(D$10:D$14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>červen</t>
+        </is>
+      </c>
+      <c r="B38" s="6">
+        <f>B$4*$B23*B$5*B$6</f>
+        <v/>
+      </c>
+      <c r="C38" s="6">
+        <f>B38*(B$8*(1-B$7)-B$9)</f>
+        <v/>
+      </c>
+      <c r="D38" s="6">
+        <f>C38-SUM(B$10:B$14)</f>
+        <v/>
+      </c>
+      <c r="E38" s="6">
+        <f>C$4*$B23*C$5*C$6</f>
+        <v/>
+      </c>
+      <c r="F38" s="6">
+        <f>E38*(C$8*(1-C$7)-C$9)</f>
+        <v/>
+      </c>
+      <c r="G38" s="6">
+        <f>F38-SUM(C$10:C$14)</f>
+        <v/>
+      </c>
+      <c r="H38" s="6">
+        <f>D$4*$B23*D$5*D$6</f>
+        <v/>
+      </c>
+      <c r="I38" s="6">
+        <f>H38*(D$8*(1-D$7)-D$9)</f>
+        <v/>
+      </c>
+      <c r="J38" s="6">
+        <f>I38-SUM(D$10:D$14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>červenec</t>
+        </is>
+      </c>
+      <c r="B39" s="6">
+        <f>B$4*$B24*B$5*B$6</f>
+        <v/>
+      </c>
+      <c r="C39" s="6">
+        <f>B39*(B$8*(1-B$7)-B$9)</f>
+        <v/>
+      </c>
+      <c r="D39" s="6">
+        <f>C39-SUM(B$10:B$14)</f>
+        <v/>
+      </c>
+      <c r="E39" s="6">
+        <f>C$4*$B24*C$5*C$6</f>
+        <v/>
+      </c>
+      <c r="F39" s="6">
+        <f>E39*(C$8*(1-C$7)-C$9)</f>
+        <v/>
+      </c>
+      <c r="G39" s="6">
+        <f>F39-SUM(C$10:C$14)</f>
+        <v/>
+      </c>
+      <c r="H39" s="6">
+        <f>D$4*$B24*D$5*D$6</f>
+        <v/>
+      </c>
+      <c r="I39" s="6">
+        <f>H39*(D$8*(1-D$7)-D$9)</f>
+        <v/>
+      </c>
+      <c r="J39" s="6">
+        <f>I39-SUM(D$10:D$14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>srpen</t>
+        </is>
+      </c>
+      <c r="B40" s="6">
+        <f>B$4*$B25*B$5*B$6</f>
+        <v/>
+      </c>
+      <c r="C40" s="6">
+        <f>B40*(B$8*(1-B$7)-B$9)</f>
+        <v/>
+      </c>
+      <c r="D40" s="6">
+        <f>C40-SUM(B$10:B$14)</f>
+        <v/>
+      </c>
+      <c r="E40" s="6">
+        <f>C$4*$B25*C$5*C$6</f>
+        <v/>
+      </c>
+      <c r="F40" s="6">
+        <f>E40*(C$8*(1-C$7)-C$9)</f>
+        <v/>
+      </c>
+      <c r="G40" s="6">
+        <f>F40-SUM(C$10:C$14)</f>
+        <v/>
+      </c>
+      <c r="H40" s="6">
+        <f>D$4*$B25*D$5*D$6</f>
+        <v/>
+      </c>
+      <c r="I40" s="6">
+        <f>H40*(D$8*(1-D$7)-D$9)</f>
+        <v/>
+      </c>
+      <c r="J40" s="6">
+        <f>I40-SUM(D$10:D$14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>září</t>
+        </is>
+      </c>
+      <c r="B41" s="6">
+        <f>B$4*$B26*B$5*B$6</f>
+        <v/>
+      </c>
+      <c r="C41" s="6">
+        <f>B41*(B$8*(1-B$7)-B$9)</f>
+        <v/>
+      </c>
+      <c r="D41" s="6">
+        <f>C41-SUM(B$10:B$14)</f>
+        <v/>
+      </c>
+      <c r="E41" s="6">
+        <f>C$4*$B26*C$5*C$6</f>
+        <v/>
+      </c>
+      <c r="F41" s="6">
+        <f>E41*(C$8*(1-C$7)-C$9)</f>
+        <v/>
+      </c>
+      <c r="G41" s="6">
+        <f>F41-SUM(C$10:C$14)</f>
+        <v/>
+      </c>
+      <c r="H41" s="6">
+        <f>D$4*$B26*D$5*D$6</f>
+        <v/>
+      </c>
+      <c r="I41" s="6">
+        <f>H41*(D$8*(1-D$7)-D$9)</f>
+        <v/>
+      </c>
+      <c r="J41" s="6">
+        <f>I41-SUM(D$10:D$14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>říjen</t>
+        </is>
+      </c>
+      <c r="B42" s="6">
+        <f>B$4*$B27*B$5*B$6</f>
+        <v/>
+      </c>
+      <c r="C42" s="6">
+        <f>B42*(B$8*(1-B$7)-B$9)</f>
+        <v/>
+      </c>
+      <c r="D42" s="6">
+        <f>C42-SUM(B$10:B$14)</f>
+        <v/>
+      </c>
+      <c r="E42" s="6">
+        <f>C$4*$B27*C$5*C$6</f>
+        <v/>
+      </c>
+      <c r="F42" s="6">
+        <f>E42*(C$8*(1-C$7)-C$9)</f>
+        <v/>
+      </c>
+      <c r="G42" s="6">
+        <f>F42-SUM(C$10:C$14)</f>
+        <v/>
+      </c>
+      <c r="H42" s="6">
+        <f>D$4*$B27*D$5*D$6</f>
+        <v/>
+      </c>
+      <c r="I42" s="6">
+        <f>H42*(D$8*(1-D$7)-D$9)</f>
+        <v/>
+      </c>
+      <c r="J42" s="6">
+        <f>I42-SUM(D$10:D$14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>listopad</t>
+        </is>
+      </c>
+      <c r="B43" s="6">
+        <f>B$4*$B28*B$5*B$6</f>
+        <v/>
+      </c>
+      <c r="C43" s="6">
+        <f>B43*(B$8*(1-B$7)-B$9)</f>
+        <v/>
+      </c>
+      <c r="D43" s="6">
+        <f>C43-SUM(B$10:B$14)</f>
+        <v/>
+      </c>
+      <c r="E43" s="6">
+        <f>C$4*$B28*C$5*C$6</f>
+        <v/>
+      </c>
+      <c r="F43" s="6">
+        <f>E43*(C$8*(1-C$7)-C$9)</f>
+        <v/>
+      </c>
+      <c r="G43" s="6">
+        <f>F43-SUM(C$10:C$14)</f>
+        <v/>
+      </c>
+      <c r="H43" s="6">
+        <f>D$4*$B28*D$5*D$6</f>
+        <v/>
+      </c>
+      <c r="I43" s="6">
+        <f>H43*(D$8*(1-D$7)-D$9)</f>
+        <v/>
+      </c>
+      <c r="J43" s="6">
+        <f>I43-SUM(D$10:D$14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>prosinec</t>
+        </is>
+      </c>
+      <c r="B44" s="6">
+        <f>B$4*$B29*B$5*B$6</f>
+        <v/>
+      </c>
+      <c r="C44" s="6">
+        <f>B44*(B$8*(1-B$7)-B$9)</f>
+        <v/>
+      </c>
+      <c r="D44" s="6">
+        <f>C44-SUM(B$10:B$14)</f>
+        <v/>
+      </c>
+      <c r="E44" s="6">
+        <f>C$4*$B29*C$5*C$6</f>
+        <v/>
+      </c>
+      <c r="F44" s="6">
+        <f>E44*(C$8*(1-C$7)-C$9)</f>
+        <v/>
+      </c>
+      <c r="G44" s="6">
+        <f>F44-SUM(C$10:C$14)</f>
+        <v/>
+      </c>
+      <c r="H44" s="6">
+        <f>D$4*$B29*D$5*D$6</f>
+        <v/>
+      </c>
+      <c r="I44" s="6">
+        <f>H44*(D$8*(1-D$7)-D$9)</f>
+        <v/>
+      </c>
+      <c r="J44" s="6">
+        <f>I44-SUM(D$10:D$14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="1" t="inlineStr">
+        <is>
+          <t>Celkem rok</t>
+        </is>
+      </c>
+      <c r="B45" s="7">
+        <f>SUM(B33:B44)</f>
+        <v/>
+      </c>
+      <c r="C45" s="7">
+        <f>SUM(C33:C44)</f>
+        <v/>
+      </c>
+      <c r="D45" s="7">
+        <f>SUM(D33:D44)</f>
+        <v/>
+      </c>
+      <c r="E45" s="7">
+        <f>SUM(E33:E44)</f>
+        <v/>
+      </c>
+      <c r="F45" s="7">
+        <f>SUM(F33:F44)</f>
+        <v/>
+      </c>
+      <c r="G45" s="7">
+        <f>SUM(G33:G44)</f>
+        <v/>
+      </c>
+      <c r="H45" s="7">
+        <f>SUM(H33:H44)</f>
+        <v/>
+      </c>
+      <c r="I45" s="7">
+        <f>SUM(I33:I44)</f>
+        <v/>
+      </c>
+      <c r="J45" s="7">
+        <f>SUM(J33:J44)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Break-even obrat/měs</t>
+        </is>
+      </c>
+      <c r="B46" s="6">
+        <f>SUM(B10:B14)/(B8*(1-B7)-B9)</f>
+        <v/>
+      </c>
+      <c r="C46" s="6" t="n"/>
+      <c r="D46" s="6" t="n"/>
+      <c r="E46" s="6">
+        <f>SUM(C10:C14)/(C8*(1-C7)-C9)</f>
+        <v/>
+      </c>
+      <c r="F46" s="6" t="n"/>
+      <c r="G46" s="6" t="n"/>
+      <c r="H46" s="6">
+        <f>SUM(D10:D14)/(D8*(1-D7)-D9)</f>
+        <v/>
+      </c>
+      <c r="I46" s="6" t="n"/>
+      <c r="J46" s="6" t="n"/>
+    </row>
+    <row r="47">
+      <c r="B47" s="6" t="n"/>
+      <c r="C47" s="6" t="n"/>
+      <c r="D47" s="6" t="n"/>
+      <c r="E47" s="6" t="n"/>
+      <c r="F47" s="6" t="n"/>
+      <c r="G47" s="6" t="n"/>
+      <c r="H47" s="6" t="n"/>
+      <c r="I47" s="6" t="n"/>
+      <c r="J47" s="6" t="n"/>
+    </row>
+    <row r="48">
+      <c r="B48" s="6" t="n"/>
+      <c r="C48" s="6" t="n"/>
+      <c r="D48" s="6" t="n"/>
+      <c r="E48" s="6" t="n"/>
+      <c r="F48" s="6" t="n"/>
+      <c r="G48" s="6" t="n"/>
+      <c r="H48" s="6" t="n"/>
+      <c r="I48" s="6" t="n"/>
+      <c r="J48" s="6" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="1" t="inlineStr">
+        <is>
+          <t>Rok 1 s rozjezdem (start v lednu; pro start v dubnu posuňte sloupec C17:C29)</t>
+        </is>
+      </c>
+      <c r="B49" s="6" t="n"/>
+      <c r="C49" s="6" t="n"/>
+      <c r="D49" s="6" t="n"/>
+      <c r="E49" s="6" t="n"/>
+      <c r="F49" s="6" t="n"/>
+      <c r="G49" s="6" t="n"/>
+      <c r="H49" s="6" t="n"/>
+      <c r="I49" s="6" t="n"/>
+      <c r="J49" s="6" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Měsíc</t>
+        </is>
+      </c>
+      <c r="B50" s="8" t="inlineStr">
+        <is>
+          <t>Pesimistický – Obrat</t>
+        </is>
+      </c>
+      <c r="C50" s="8" t="inlineStr">
+        <is>
+          <t>Pesimistický – Hrubý zisk po ztrátách a poplatcích</t>
+        </is>
+      </c>
+      <c r="D50" s="8" t="inlineStr">
+        <is>
+          <t>Pesimistický – Výsledek po fixních nákladech</t>
+        </is>
+      </c>
+      <c r="E50" s="8" t="inlineStr">
+        <is>
+          <t>Realistický – Obrat</t>
+        </is>
+      </c>
+      <c r="F50" s="8" t="inlineStr">
+        <is>
+          <t>Realistický – Hrubý zisk po ztrátách a poplatcích</t>
+        </is>
+      </c>
+      <c r="G50" s="8" t="inlineStr">
+        <is>
+          <t>Realistický – Výsledek po fixních nákladech</t>
+        </is>
+      </c>
+      <c r="H50" s="8" t="inlineStr">
+        <is>
+          <t>Optimistický – Obrat</t>
+        </is>
+      </c>
+      <c r="I50" s="8" t="inlineStr">
+        <is>
+          <t>Optimistický – Hrubý zisk po ztrátách a poplatcích</t>
+        </is>
+      </c>
+      <c r="J50" s="8" t="inlineStr">
+        <is>
+          <t>Optimistický – Výsledek po fixních nákladech</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>leden</t>
+        </is>
+      </c>
+      <c r="B51" s="6">
+        <f>B$4*$B18*$C18*B$5*B$6</f>
+        <v/>
+      </c>
+      <c r="C51" s="6">
+        <f>B51*(B$8*(1-B$7)-B$9)</f>
+        <v/>
+      </c>
+      <c r="D51" s="6">
+        <f>C51-SUM(B$10:B$14)</f>
+        <v/>
+      </c>
+      <c r="E51" s="6">
+        <f>C$4*$B18*$C18*C$5*C$6</f>
+        <v/>
+      </c>
+      <c r="F51" s="6">
+        <f>E51*(C$8*(1-C$7)-C$9)</f>
+        <v/>
+      </c>
+      <c r="G51" s="6">
+        <f>F51-SUM(C$10:C$14)</f>
+        <v/>
+      </c>
+      <c r="H51" s="6">
+        <f>D$4*$B18*$C18*D$5*D$6</f>
+        <v/>
+      </c>
+      <c r="I51" s="6">
+        <f>H51*(D$8*(1-D$7)-D$9)</f>
+        <v/>
+      </c>
+      <c r="J51" s="6">
+        <f>I51-SUM(D$10:D$14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>únor</t>
+        </is>
+      </c>
+      <c r="B52" s="6">
+        <f>B$4*$B19*$C19*B$5*B$6</f>
+        <v/>
+      </c>
+      <c r="C52" s="6">
+        <f>B52*(B$8*(1-B$7)-B$9)</f>
+        <v/>
+      </c>
+      <c r="D52" s="6">
+        <f>C52-SUM(B$10:B$14)</f>
+        <v/>
+      </c>
+      <c r="E52" s="6">
+        <f>C$4*$B19*$C19*C$5*C$6</f>
+        <v/>
+      </c>
+      <c r="F52" s="6">
+        <f>E52*(C$8*(1-C$7)-C$9)</f>
+        <v/>
+      </c>
+      <c r="G52" s="6">
+        <f>F52-SUM(C$10:C$14)</f>
+        <v/>
+      </c>
+      <c r="H52" s="6">
+        <f>D$4*$B19*$C19*D$5*D$6</f>
+        <v/>
+      </c>
+      <c r="I52" s="6">
+        <f>H52*(D$8*(1-D$7)-D$9)</f>
+        <v/>
+      </c>
+      <c r="J52" s="6">
+        <f>I52-SUM(D$10:D$14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>březen</t>
+        </is>
+      </c>
+      <c r="B53" s="6">
+        <f>B$4*$B20*$C20*B$5*B$6</f>
+        <v/>
+      </c>
+      <c r="C53" s="6">
+        <f>B53*(B$8*(1-B$7)-B$9)</f>
+        <v/>
+      </c>
+      <c r="D53" s="6">
+        <f>C53-SUM(B$10:B$14)</f>
+        <v/>
+      </c>
+      <c r="E53" s="6">
+        <f>C$4*$B20*$C20*C$5*C$6</f>
+        <v/>
+      </c>
+      <c r="F53" s="6">
+        <f>E53*(C$8*(1-C$7)-C$9)</f>
+        <v/>
+      </c>
+      <c r="G53" s="6">
+        <f>F53-SUM(C$10:C$14)</f>
+        <v/>
+      </c>
+      <c r="H53" s="6">
+        <f>D$4*$B20*$C20*D$5*D$6</f>
+        <v/>
+      </c>
+      <c r="I53" s="6">
+        <f>H53*(D$8*(1-D$7)-D$9)</f>
+        <v/>
+      </c>
+      <c r="J53" s="6">
+        <f>I53-SUM(D$10:D$14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>duben</t>
+        </is>
+      </c>
+      <c r="B54" s="6">
+        <f>B$4*$B21*$C21*B$5*B$6</f>
+        <v/>
+      </c>
+      <c r="C54" s="6">
+        <f>B54*(B$8*(1-B$7)-B$9)</f>
+        <v/>
+      </c>
+      <c r="D54" s="6">
+        <f>C54-SUM(B$10:B$14)</f>
+        <v/>
+      </c>
+      <c r="E54" s="6">
+        <f>C$4*$B21*$C21*C$5*C$6</f>
+        <v/>
+      </c>
+      <c r="F54" s="6">
+        <f>E54*(C$8*(1-C$7)-C$9)</f>
+        <v/>
+      </c>
+      <c r="G54" s="6">
+        <f>F54-SUM(C$10:C$14)</f>
+        <v/>
+      </c>
+      <c r="H54" s="6">
+        <f>D$4*$B21*$C21*D$5*D$6</f>
+        <v/>
+      </c>
+      <c r="I54" s="6">
+        <f>H54*(D$8*(1-D$7)-D$9)</f>
+        <v/>
+      </c>
+      <c r="J54" s="6">
+        <f>I54-SUM(D$10:D$14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>květen</t>
+        </is>
+      </c>
+      <c r="B55" s="6">
+        <f>B$4*$B22*$C22*B$5*B$6</f>
+        <v/>
+      </c>
+      <c r="C55" s="6">
+        <f>B55*(B$8*(1-B$7)-B$9)</f>
+        <v/>
+      </c>
+      <c r="D55" s="6">
+        <f>C55-SUM(B$10:B$14)</f>
+        <v/>
+      </c>
+      <c r="E55" s="6">
+        <f>C$4*$B22*$C22*C$5*C$6</f>
+        <v/>
+      </c>
+      <c r="F55" s="6">
+        <f>E55*(C$8*(1-C$7)-C$9)</f>
+        <v/>
+      </c>
+      <c r="G55" s="6">
+        <f>F55-SUM(C$10:C$14)</f>
+        <v/>
+      </c>
+      <c r="H55" s="6">
+        <f>D$4*$B22*$C22*D$5*D$6</f>
+        <v/>
+      </c>
+      <c r="I55" s="6">
+        <f>H55*(D$8*(1-D$7)-D$9)</f>
+        <v/>
+      </c>
+      <c r="J55" s="6">
+        <f>I55-SUM(D$10:D$14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>červen</t>
+        </is>
+      </c>
+      <c r="B56" s="6">
+        <f>B$4*$B23*$C23*B$5*B$6</f>
+        <v/>
+      </c>
+      <c r="C56" s="6">
+        <f>B56*(B$8*(1-B$7)-B$9)</f>
+        <v/>
+      </c>
+      <c r="D56" s="6">
+        <f>C56-SUM(B$10:B$14)</f>
+        <v/>
+      </c>
+      <c r="E56" s="6">
+        <f>C$4*$B23*$C23*C$5*C$6</f>
+        <v/>
+      </c>
+      <c r="F56" s="6">
+        <f>E56*(C$8*(1-C$7)-C$9)</f>
+        <v/>
+      </c>
+      <c r="G56" s="6">
+        <f>F56-SUM(C$10:C$14)</f>
+        <v/>
+      </c>
+      <c r="H56" s="6">
+        <f>D$4*$B23*$C23*D$5*D$6</f>
+        <v/>
+      </c>
+      <c r="I56" s="6">
+        <f>H56*(D$8*(1-D$7)-D$9)</f>
+        <v/>
+      </c>
+      <c r="J56" s="6">
+        <f>I56-SUM(D$10:D$14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>červenec</t>
+        </is>
+      </c>
+      <c r="B57" s="6">
+        <f>B$4*$B24*$C24*B$5*B$6</f>
+        <v/>
+      </c>
+      <c r="C57" s="6">
+        <f>B57*(B$8*(1-B$7)-B$9)</f>
+        <v/>
+      </c>
+      <c r="D57" s="6">
+        <f>C57-SUM(B$10:B$14)</f>
+        <v/>
+      </c>
+      <c r="E57" s="6">
+        <f>C$4*$B24*$C24*C$5*C$6</f>
+        <v/>
+      </c>
+      <c r="F57" s="6">
+        <f>E57*(C$8*(1-C$7)-C$9)</f>
+        <v/>
+      </c>
+      <c r="G57" s="6">
+        <f>F57-SUM(C$10:C$14)</f>
+        <v/>
+      </c>
+      <c r="H57" s="6">
+        <f>D$4*$B24*$C24*D$5*D$6</f>
+        <v/>
+      </c>
+      <c r="I57" s="6">
+        <f>H57*(D$8*(1-D$7)-D$9)</f>
+        <v/>
+      </c>
+      <c r="J57" s="6">
+        <f>I57-SUM(D$10:D$14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>srpen</t>
+        </is>
+      </c>
+      <c r="B58" s="6">
+        <f>B$4*$B25*$C25*B$5*B$6</f>
+        <v/>
+      </c>
+      <c r="C58" s="6">
+        <f>B58*(B$8*(1-B$7)-B$9)</f>
+        <v/>
+      </c>
+      <c r="D58" s="6">
+        <f>C58-SUM(B$10:B$14)</f>
+        <v/>
+      </c>
+      <c r="E58" s="6">
+        <f>C$4*$B25*$C25*C$5*C$6</f>
+        <v/>
+      </c>
+      <c r="F58" s="6">
+        <f>E58*(C$8*(1-C$7)-C$9)</f>
+        <v/>
+      </c>
+      <c r="G58" s="6">
+        <f>F58-SUM(C$10:C$14)</f>
+        <v/>
+      </c>
+      <c r="H58" s="6">
+        <f>D$4*$B25*$C25*D$5*D$6</f>
+        <v/>
+      </c>
+      <c r="I58" s="6">
+        <f>H58*(D$8*(1-D$7)-D$9)</f>
+        <v/>
+      </c>
+      <c r="J58" s="6">
+        <f>I58-SUM(D$10:D$14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>září</t>
+        </is>
+      </c>
+      <c r="B59" s="6">
+        <f>B$4*$B26*$C26*B$5*B$6</f>
+        <v/>
+      </c>
+      <c r="C59" s="6">
+        <f>B59*(B$8*(1-B$7)-B$9)</f>
+        <v/>
+      </c>
+      <c r="D59" s="6">
+        <f>C59-SUM(B$10:B$14)</f>
+        <v/>
+      </c>
+      <c r="E59" s="6">
+        <f>C$4*$B26*$C26*C$5*C$6</f>
+        <v/>
+      </c>
+      <c r="F59" s="6">
+        <f>E59*(C$8*(1-C$7)-C$9)</f>
+        <v/>
+      </c>
+      <c r="G59" s="6">
+        <f>F59-SUM(C$10:C$14)</f>
+        <v/>
+      </c>
+      <c r="H59" s="6">
+        <f>D$4*$B26*$C26*D$5*D$6</f>
+        <v/>
+      </c>
+      <c r="I59" s="6">
+        <f>H59*(D$8*(1-D$7)-D$9)</f>
+        <v/>
+      </c>
+      <c r="J59" s="6">
+        <f>I59-SUM(D$10:D$14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>říjen</t>
+        </is>
+      </c>
+      <c r="B60" s="6">
+        <f>B$4*$B27*$C27*B$5*B$6</f>
+        <v/>
+      </c>
+      <c r="C60" s="6">
+        <f>B60*(B$8*(1-B$7)-B$9)</f>
+        <v/>
+      </c>
+      <c r="D60" s="6">
+        <f>C60-SUM(B$10:B$14)</f>
+        <v/>
+      </c>
+      <c r="E60" s="6">
+        <f>C$4*$B27*$C27*C$5*C$6</f>
+        <v/>
+      </c>
+      <c r="F60" s="6">
+        <f>E60*(C$8*(1-C$7)-C$9)</f>
+        <v/>
+      </c>
+      <c r="G60" s="6">
+        <f>F60-SUM(C$10:C$14)</f>
+        <v/>
+      </c>
+      <c r="H60" s="6">
+        <f>D$4*$B27*$C27*D$5*D$6</f>
+        <v/>
+      </c>
+      <c r="I60" s="6">
+        <f>H60*(D$8*(1-D$7)-D$9)</f>
+        <v/>
+      </c>
+      <c r="J60" s="6">
+        <f>I60-SUM(D$10:D$14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>listopad</t>
+        </is>
+      </c>
+      <c r="B61" s="6">
+        <f>B$4*$B28*$C28*B$5*B$6</f>
+        <v/>
+      </c>
+      <c r="C61" s="6">
+        <f>B61*(B$8*(1-B$7)-B$9)</f>
+        <v/>
+      </c>
+      <c r="D61" s="6">
+        <f>C61-SUM(B$10:B$14)</f>
+        <v/>
+      </c>
+      <c r="E61" s="6">
+        <f>C$4*$B28*$C28*C$5*C$6</f>
+        <v/>
+      </c>
+      <c r="F61" s="6">
+        <f>E61*(C$8*(1-C$7)-C$9)</f>
+        <v/>
+      </c>
+      <c r="G61" s="6">
+        <f>F61-SUM(C$10:C$14)</f>
+        <v/>
+      </c>
+      <c r="H61" s="6">
+        <f>D$4*$B28*$C28*D$5*D$6</f>
+        <v/>
+      </c>
+      <c r="I61" s="6">
+        <f>H61*(D$8*(1-D$7)-D$9)</f>
+        <v/>
+      </c>
+      <c r="J61" s="6">
+        <f>I61-SUM(D$10:D$14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>prosinec</t>
+        </is>
+      </c>
+      <c r="B62" s="6">
+        <f>B$4*$B29*$C29*B$5*B$6</f>
+        <v/>
+      </c>
+      <c r="C62" s="6">
+        <f>B62*(B$8*(1-B$7)-B$9)</f>
+        <v/>
+      </c>
+      <c r="D62" s="6">
+        <f>C62-SUM(B$10:B$14)</f>
+        <v/>
+      </c>
+      <c r="E62" s="6">
+        <f>C$4*$B29*$C29*C$5*C$6</f>
+        <v/>
+      </c>
+      <c r="F62" s="6">
+        <f>E62*(C$8*(1-C$7)-C$9)</f>
+        <v/>
+      </c>
+      <c r="G62" s="6">
+        <f>F62-SUM(C$10:C$14)</f>
+        <v/>
+      </c>
+      <c r="H62" s="6">
+        <f>D$4*$B29*$C29*D$5*D$6</f>
+        <v/>
+      </c>
+      <c r="I62" s="6">
+        <f>H62*(D$8*(1-D$7)-D$9)</f>
+        <v/>
+      </c>
+      <c r="J62" s="6">
+        <f>I62-SUM(D$10:D$14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="1" t="inlineStr">
+        <is>
+          <t>Celkem rok 1</t>
+        </is>
+      </c>
+      <c r="B63" s="7">
+        <f>SUM(B51:B62)</f>
+        <v/>
+      </c>
+      <c r="C63" s="7">
+        <f>SUM(C51:C62)</f>
+        <v/>
+      </c>
+      <c r="D63" s="7">
+        <f>SUM(D51:D62)</f>
+        <v/>
+      </c>
+      <c r="E63" s="7">
+        <f>SUM(E51:E62)</f>
+        <v/>
+      </c>
+      <c r="F63" s="7">
+        <f>SUM(F51:F62)</f>
+        <v/>
+      </c>
+      <c r="G63" s="7">
+        <f>SUM(G51:G62)</f>
+        <v/>
+      </c>
+      <c r="H63" s="7">
+        <f>SUM(H51:H62)</f>
+        <v/>
+      </c>
+      <c r="I63" s="7">
+        <f>SUM(I51:I62)</f>
+        <v/>
+      </c>
+      <c r="J63" s="7">
+        <f>SUM(J51:J62)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E185"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -470,7 +2233,6 @@
       <c r="D2" t="n">
         <v>46</v>
       </c>
-      <c r="E2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -489,7 +2251,6 @@
       <c r="D3" t="n">
         <v>73</v>
       </c>
-      <c r="E3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -508,7 +2269,6 @@
       <c r="D4" t="n">
         <v>43</v>
       </c>
-      <c r="E4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -527,7 +2287,6 @@
       <c r="D5" t="n">
         <v>41</v>
       </c>
-      <c r="E5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -546,7 +2305,6 @@
       <c r="D6" t="n">
         <v>38</v>
       </c>
-      <c r="E6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -565,7 +2323,6 @@
       <c r="D7" t="n">
         <v>6</v>
       </c>
-      <c r="E7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -680,7 +2437,6 @@
       <c r="D12" t="n">
         <v>6</v>
       </c>
-      <c r="E12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -699,7 +2455,6 @@
       <c r="D13" t="n">
         <v>6</v>
       </c>
-      <c r="E13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -718,7 +2473,6 @@
       <c r="D14" t="n">
         <v>10</v>
       </c>
-      <c r="E14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -833,7 +2587,6 @@
       <c r="D19" t="n">
         <v>10</v>
       </c>
-      <c r="E19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -852,7 +2605,6 @@
       <c r="D20" t="n">
         <v>5</v>
       </c>
-      <c r="E20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -871,7 +2623,6 @@
       <c r="D21" t="n">
         <v>14</v>
       </c>
-      <c r="E21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -890,7 +2641,6 @@
       <c r="D22" t="n">
         <v>3</v>
       </c>
-      <c r="E22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -936,7 +2686,6 @@
           <t>doplnit</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -955,7 +2704,6 @@
       <c r="D25" t="n">
         <v>5</v>
       </c>
-      <c r="E25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -974,7 +2722,6 @@
       <c r="D26" t="n">
         <v>15</v>
       </c>
-      <c r="E26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1016,7 +2763,6 @@
       <c r="D28" t="n">
         <v>5</v>
       </c>
-      <c r="E28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1035,7 +2781,6 @@
       <c r="D29" t="n">
         <v>21</v>
       </c>
-      <c r="E29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1054,7 +2799,6 @@
       <c r="D30" t="n">
         <v>20</v>
       </c>
-      <c r="E30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1096,7 +2840,6 @@
       <c r="D32" t="n">
         <v>6</v>
       </c>
-      <c r="E32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1115,7 +2858,6 @@
       <c r="D33" t="n">
         <v>7</v>
       </c>
-      <c r="E33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1134,7 +2876,6 @@
       <c r="D34" t="n">
         <v>6</v>
       </c>
-      <c r="E34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1155,7 +2896,6 @@
           <t>doplnit</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1201,7 +2941,6 @@
           <t>doplnit</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1220,7 +2959,6 @@
       <c r="D38" t="n">
         <v>4</v>
       </c>
-      <c r="E38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1239,7 +2977,6 @@
       <c r="D39" t="n">
         <v>15</v>
       </c>
-      <c r="E39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1260,7 +2997,6 @@
           <t>doplnit</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1302,7 +3038,6 @@
       <c r="D42" t="n">
         <v>5</v>
       </c>
-      <c r="E42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1321,7 +3056,6 @@
       <c r="D43" t="n">
         <v>14</v>
       </c>
-      <c r="E43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1342,7 +3076,6 @@
           <t>doplnit</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1384,7 +3117,6 @@
       <c r="D46" t="n">
         <v>49</v>
       </c>
-      <c r="E46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -1403,7 +3135,6 @@
       <c r="D47" t="n">
         <v>30</v>
       </c>
-      <c r="E47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1422,7 +3153,6 @@
       <c r="D48" t="n">
         <v>33</v>
       </c>
-      <c r="E48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -1441,7 +3171,6 @@
       <c r="D49" t="n">
         <v>12</v>
       </c>
-      <c r="E49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -1460,7 +3189,6 @@
       <c r="D50" t="n">
         <v>22</v>
       </c>
-      <c r="E50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -1502,7 +3230,6 @@
       <c r="D52" t="n">
         <v>25</v>
       </c>
-      <c r="E52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -1521,7 +3248,6 @@
       <c r="D53" t="n">
         <v>7</v>
       </c>
-      <c r="E53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -1540,7 +3266,6 @@
       <c r="D54" t="n">
         <v>14</v>
       </c>
-      <c r="E54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -1559,7 +3284,6 @@
       <c r="D55" t="n">
         <v>6</v>
       </c>
-      <c r="E55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -1578,7 +3302,6 @@
       <c r="D56" t="n">
         <v>6</v>
       </c>
-      <c r="E56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -1597,7 +3320,6 @@
       <c r="D57" t="n">
         <v>6</v>
       </c>
-      <c r="E57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -1616,7 +3338,6 @@
       <c r="D58" t="n">
         <v>5</v>
       </c>
-      <c r="E58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -1637,7 +3358,6 @@
           <t>doplnit</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -1656,7 +3376,6 @@
       <c r="D60" t="n">
         <v>8</v>
       </c>
-      <c r="E60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -1698,7 +3417,6 @@
       <c r="D62" t="n">
         <v>4</v>
       </c>
-      <c r="E62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -1717,7 +3435,6 @@
       <c r="D63" t="n">
         <v>5</v>
       </c>
-      <c r="E63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -1736,7 +3453,6 @@
       <c r="D64" t="n">
         <v>3</v>
       </c>
-      <c r="E64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -1757,7 +3473,6 @@
           <t>doplnit</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -1776,7 +3491,6 @@
       <c r="D66" t="n">
         <v>13</v>
       </c>
-      <c r="E66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -1795,7 +3509,6 @@
       <c r="D67" t="n">
         <v>5</v>
       </c>
-      <c r="E67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -1814,7 +3527,6 @@
       <c r="D68" t="n">
         <v>4</v>
       </c>
-      <c r="E68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -1833,7 +3545,6 @@
       <c r="D69" t="n">
         <v>6</v>
       </c>
-      <c r="E69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -1877,7 +3588,6 @@
       <c r="D71" t="n">
         <v>4</v>
       </c>
-      <c r="E71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -1896,7 +3606,6 @@
       <c r="D72" t="n">
         <v>5</v>
       </c>
-      <c r="E72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -1915,7 +3624,6 @@
       <c r="D73" t="n">
         <v>10</v>
       </c>
-      <c r="E73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -1934,7 +3642,6 @@
       <c r="D74" t="n">
         <v>3</v>
       </c>
-      <c r="E74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -1976,7 +3683,6 @@
       <c r="D76" t="n">
         <v>16</v>
       </c>
-      <c r="E76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -1995,7 +3701,6 @@
       <c r="D77" t="n">
         <v>26</v>
       </c>
-      <c r="E77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -2014,7 +3719,6 @@
       <c r="D78" t="n">
         <v>10</v>
       </c>
-      <c r="E78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -2033,7 +3737,6 @@
       <c r="D79" t="n">
         <v>9</v>
       </c>
-      <c r="E79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -2054,7 +3757,6 @@
           <t>doplnit</t>
         </is>
       </c>
-      <c r="E80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -2073,7 +3775,6 @@
       <c r="D81" t="n">
         <v>35</v>
       </c>
-      <c r="E81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -2092,7 +3793,6 @@
       <c r="D82" t="n">
         <v>20</v>
       </c>
-      <c r="E82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -2113,7 +3813,6 @@
           <t>doplnit</t>
         </is>
       </c>
-      <c r="E83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -2132,7 +3831,6 @@
       <c r="D84" t="n">
         <v>4</v>
       </c>
-      <c r="E84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -2199,7 +3897,6 @@
       <c r="D87" t="n">
         <v>5</v>
       </c>
-      <c r="E87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -2218,7 +3915,6 @@
       <c r="D88" t="n">
         <v>6</v>
       </c>
-      <c r="E88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -2260,7 +3956,6 @@
       <c r="D90" t="n">
         <v>25</v>
       </c>
-      <c r="E90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -2279,7 +3974,6 @@
       <c r="D91" t="n">
         <v>14</v>
       </c>
-      <c r="E91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -2298,7 +3992,6 @@
       <c r="D92" t="n">
         <v>17</v>
       </c>
-      <c r="E92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -2340,7 +4033,6 @@
       <c r="D94" t="n">
         <v>9</v>
       </c>
-      <c r="E94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -2359,7 +4051,6 @@
       <c r="D95" t="n">
         <v>14</v>
       </c>
-      <c r="E95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -2405,7 +4096,6 @@
           <t>doplnit</t>
         </is>
       </c>
-      <c r="E97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -2426,7 +4116,6 @@
           <t>doplnit</t>
         </is>
       </c>
-      <c r="E98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -2445,7 +4134,6 @@
       <c r="D99" t="n">
         <v>3</v>
       </c>
-      <c r="E99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -2466,7 +4154,6 @@
           <t>doplnit</t>
         </is>
       </c>
-      <c r="E100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -2537,7 +4224,6 @@
           <t>doplnit</t>
         </is>
       </c>
-      <c r="E103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -2581,7 +4267,6 @@
           <t>doplnit</t>
         </is>
       </c>
-      <c r="E105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -2602,7 +4287,6 @@
           <t>doplnit</t>
         </is>
       </c>
-      <c r="E106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -2623,7 +4307,6 @@
           <t>doplnit</t>
         </is>
       </c>
-      <c r="E107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -2644,7 +4327,6 @@
           <t>doplnit</t>
         </is>
       </c>
-      <c r="E108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -2663,7 +4345,6 @@
       <c r="D109" t="n">
         <v>5</v>
       </c>
-      <c r="E109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -2682,7 +4363,6 @@
       <c r="D110" t="n">
         <v>9</v>
       </c>
-      <c r="E110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -2701,7 +4381,6 @@
       <c r="D111" t="n">
         <v>7</v>
       </c>
-      <c r="E111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -2720,7 +4399,6 @@
       <c r="D112" t="n">
         <v>12</v>
       </c>
-      <c r="E112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -2741,7 +4419,6 @@
           <t>doplnit</t>
         </is>
       </c>
-      <c r="E113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -2762,7 +4439,6 @@
           <t>doplnit</t>
         </is>
       </c>
-      <c r="E114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -2783,7 +4459,6 @@
           <t>doplnit</t>
         </is>
       </c>
-      <c r="E115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -2802,7 +4477,6 @@
       <c r="D116" t="n">
         <v>5</v>
       </c>
-      <c r="E116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -2823,7 +4497,6 @@
           <t>doplnit</t>
         </is>
       </c>
-      <c r="E117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -2844,7 +4517,6 @@
           <t>doplnit</t>
         </is>
       </c>
-      <c r="E118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -2865,7 +4537,6 @@
           <t>doplnit</t>
         </is>
       </c>
-      <c r="E119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -2884,7 +4555,6 @@
       <c r="D120" t="n">
         <v>4</v>
       </c>
-      <c r="E120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -2903,7 +4573,6 @@
       <c r="D121" t="n">
         <v>6</v>
       </c>
-      <c r="E121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -2945,7 +4614,6 @@
       <c r="D123" t="n">
         <v>5</v>
       </c>
-      <c r="E123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -2966,7 +4634,6 @@
           <t>doplnit</t>
         </is>
       </c>
-      <c r="E124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -2985,7 +4652,6 @@
       <c r="D125" t="n">
         <v>3</v>
       </c>
-      <c r="E125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -3031,7 +4697,6 @@
           <t>doplnit</t>
         </is>
       </c>
-      <c r="E127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -3073,7 +4738,6 @@
       <c r="D129" t="n">
         <v>12</v>
       </c>
-      <c r="E129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -3092,7 +4756,6 @@
       <c r="D130" t="n">
         <v>9</v>
       </c>
-      <c r="E130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -3111,7 +4774,6 @@
       <c r="D131" t="n">
         <v>7</v>
       </c>
-      <c r="E131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -3130,7 +4792,6 @@
       <c r="D132" t="n">
         <v>4</v>
       </c>
-      <c r="E132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -3151,7 +4812,6 @@
           <t>doplnit</t>
         </is>
       </c>
-      <c r="E133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -3170,7 +4830,6 @@
       <c r="D134" t="n">
         <v>3</v>
       </c>
-      <c r="E134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -3189,7 +4848,6 @@
       <c r="D135" t="n">
         <v>6</v>
       </c>
-      <c r="E135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -3208,7 +4866,6 @@
       <c r="D136" t="n">
         <v>4</v>
       </c>
-      <c r="E136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -3227,7 +4884,6 @@
       <c r="D137" t="n">
         <v>6</v>
       </c>
-      <c r="E137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -3271,7 +4927,6 @@
       <c r="D139" t="n">
         <v>5</v>
       </c>
-      <c r="E139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -3290,7 +4945,6 @@
       <c r="D140" t="n">
         <v>5</v>
       </c>
-      <c r="E140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -3309,7 +4963,6 @@
       <c r="D141" t="n">
         <v>10</v>
       </c>
-      <c r="E141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -3330,7 +4983,6 @@
           <t>doplnit</t>
         </is>
       </c>
-      <c r="E142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -3351,7 +5003,6 @@
           <t>doplnit</t>
         </is>
       </c>
-      <c r="E143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -3370,7 +5021,6 @@
       <c r="D144" t="n">
         <v>11</v>
       </c>
-      <c r="E144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -3391,7 +5041,6 @@
           <t>doplnit</t>
         </is>
       </c>
-      <c r="E145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -3410,7 +5059,6 @@
       <c r="D146" t="n">
         <v>4</v>
       </c>
-      <c r="E146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -3429,7 +5077,6 @@
       <c r="D147" t="n">
         <v>9</v>
       </c>
-      <c r="E147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -3471,7 +5118,6 @@
       <c r="D149" t="n">
         <v>5</v>
       </c>
-      <c r="E149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -3490,7 +5136,6 @@
       <c r="D150" t="n">
         <v>6</v>
       </c>
-      <c r="E150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -3509,7 +5154,6 @@
       <c r="D151" t="n">
         <v>4</v>
       </c>
-      <c r="E151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -3528,7 +5172,6 @@
       <c r="D152" t="n">
         <v>30</v>
       </c>
-      <c r="E152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -3547,7 +5190,6 @@
       <c r="D153" t="n">
         <v>15</v>
       </c>
-      <c r="E153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -3566,7 +5208,6 @@
       <c r="D154" t="n">
         <v>3</v>
       </c>
-      <c r="E154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -3587,7 +5228,6 @@
           <t>doplnit</t>
         </is>
       </c>
-      <c r="E155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -3606,7 +5246,6 @@
       <c r="D156" t="n">
         <v>12</v>
       </c>
-      <c r="E156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -3648,7 +5287,6 @@
       <c r="D158" t="n">
         <v>3</v>
       </c>
-      <c r="E158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -3667,7 +5305,6 @@
       <c r="D159" t="n">
         <v>4</v>
       </c>
-      <c r="E159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -3686,7 +5323,6 @@
       <c r="D160" t="n">
         <v>8</v>
       </c>
-      <c r="E160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -3730,7 +5366,6 @@
       <c r="D162" t="n">
         <v>2</v>
       </c>
-      <c r="E162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -3772,7 +5407,6 @@
       <c r="D164" t="n">
         <v>3</v>
       </c>
-      <c r="E164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -3791,7 +5425,6 @@
       <c r="D165" t="n">
         <v>3</v>
       </c>
-      <c r="E165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -3810,7 +5443,6 @@
       <c r="D166" t="n">
         <v>4</v>
       </c>
-      <c r="E166" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -3829,7 +5461,6 @@
       <c r="D167" t="n">
         <v>2</v>
       </c>
-      <c r="E167" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -3871,7 +5502,6 @@
       <c r="D169" t="n">
         <v>18</v>
       </c>
-      <c r="E169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -3890,7 +5520,6 @@
       <c r="D170" t="n">
         <v>3</v>
       </c>
-      <c r="E170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -3909,7 +5538,6 @@
       <c r="D171" t="n">
         <v>3</v>
       </c>
-      <c r="E171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -3930,7 +5558,6 @@
           <t>doplnit</t>
         </is>
       </c>
-      <c r="E172" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -3949,7 +5576,6 @@
       <c r="D173" t="n">
         <v>22</v>
       </c>
-      <c r="E173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -3968,7 +5594,6 @@
       <c r="D174" t="n">
         <v>5</v>
       </c>
-      <c r="E174" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -3987,7 +5612,6 @@
       <c r="D175" t="n">
         <v>10</v>
       </c>
-      <c r="E175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -4008,7 +5632,6 @@
           <t>doplnit</t>
         </is>
       </c>
-      <c r="E176" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -4029,7 +5652,6 @@
           <t>doplnit</t>
         </is>
       </c>
-      <c r="E177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -4050,7 +5672,6 @@
           <t>doplnit</t>
         </is>
       </c>
-      <c r="E178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -4094,7 +5715,6 @@
           <t>doplnit</t>
         </is>
       </c>
-      <c r="E180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -4113,7 +5733,6 @@
       <c r="D181" t="n">
         <v>3</v>
       </c>
-      <c r="E181" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -4214,7 +5833,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6044,7 +7663,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -27234,7 +28853,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Expand fasteners and wall paint, add off-hours demand estimate
Base assortment grows from 184 to 220 items: 28 fastener items in blisters
(store 1 sells them loose per piece, main stock is in store 2) and a new
19-item wall paint section led by Het Klasik 15+3 kg, the strongest item
under 1000 CZK. Base turnover in Solnice rises to 145k CZK/month, so the
forecast is recomputed (realistic scenario now 906k CZK/year, -49k result).

Adds an off-hours demand estimate scored by urgency and weekend-project
character, since the stock export holds only 30-day totals and cannot be
broken down by weekday.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01H9fdgZQbPRfobYczG68Y19
</commit_message>
<xml_diff>
--- a/analyzy/bezobsluzny-obchod/sortiment_24-7_analyza.xlsx
+++ b/analyzy/bezobsluzny-obchod/sortiment_24-7_analyza.xlsx
@@ -9,9 +9,10 @@
   <sheets>
     <sheet name="Predikce" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Zakladni sortiment" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Skupiny" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Kandidatni polozky" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Metodika" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Mimo pracovni dobu" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Skupiny" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Kandidatni polozky" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Metodika" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -491,17 +492,17 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>119919</v>
+        <v>160897</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>119919</v>
+        <v>160897</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>119919</v>
+        <v>160897</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Z listu Zakladni sortiment, 108 289 Kč v okně březen/duben, přepočteno sezónním indexem</t>
+          <t>Z listu Zakladni sortiment, 145 293 Kč v okně březen/duben, přepočteno sezónním indexem</t>
         </is>
       </c>
     </row>
@@ -2179,7 +2180,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E185"/>
+  <dimension ref="A1:E221"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -3858,62 +3859,60 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Malířské potřeby</t>
+          <t>Vodoinstalace</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Bílá malířská barva 4 kg (Primalex/HET)</t>
+          <t>Hadicové spony 8–12 / 12–20 / 16–25 / 20–32 / 25–40 / 32–50</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>199</v>
-      </c>
-      <c r="D86" t="inlineStr">
-        <is>
-          <t>doplnit</t>
-        </is>
+        <v>9</v>
+      </c>
+      <c r="D86" t="n">
+        <v>77</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>jediná barva, kterou bezobslužně držet</t>
+          <t>celá řada</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Malířské potřeby</t>
+          <t>Vodoinstalace</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Univerzální lazura 0,75 l ořech / teak</t>
+          <t>Objímka trubková 2-šroub 31–38 mm</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>259</v>
+        <v>16</v>
       </c>
       <c r="D87" t="n">
-        <v>5</v>
+        <v>25</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Malířské potřeby</t>
+          <t>Vodoinstalace</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Bochemit proti plísním 500 ml</t>
+          <t>Objímka trubková 2-šroub 54–59 mm</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>99</v>
+        <v>22</v>
       </c>
       <c r="D88" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
     </row>
     <row r="89">
@@ -3924,19 +3923,14 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Hadicové spony 8–12 / 12–20 / 16–25 / 20–32 / 25–40 / 32–50</t>
+          <t>Příchytka na potrubí 20 / 25 mm</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D89" t="n">
-        <v>77</v>
-      </c>
-      <c r="E89" t="inlineStr">
-        <is>
-          <t>celá řada</t>
-        </is>
+        <v>17</v>
       </c>
     </row>
     <row r="90">
@@ -3947,14 +3941,19 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Objímka trubková 2-šroub 31–38 mm</t>
+          <t>PPR koleno 90° 20 mm, T-kus 20, nátrubek 20</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="D90" t="n">
-        <v>25</v>
+        <v>15</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>jen dimenze 20 a 25</t>
+        </is>
       </c>
     </row>
     <row r="91">
@@ -3965,14 +3964,14 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Objímka trubková 2-šroub 54–59 mm</t>
+          <t>Mosazná vsuvka 3/4", 1/2"</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>22</v>
+        <v>48</v>
       </c>
       <c r="D91" t="n">
-        <v>14</v>
+        <v>9</v>
       </c>
     </row>
     <row r="92">
@@ -3983,14 +3982,14 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Příchytka na potrubí 20 / 25 mm</t>
+          <t>Tubex izolace 20×10 mm (2 m)</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="D92" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="93">
@@ -4001,18 +4000,20 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>PPR koleno 90° 20 mm, T-kus 20, nátrubek 20</t>
+          <t>Těsnění gumová sada 1/2"–3/4"</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>8</v>
-      </c>
-      <c r="D93" t="n">
-        <v>15</v>
+        <v>25</v>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>jen dimenze 20 a 25</t>
+          <t>nejčastější havárie</t>
         </is>
       </c>
     </row>
@@ -4024,14 +4025,16 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Mosazná vsuvka 3/4", 1/2"</t>
+          <t>Flexi hadička 3/8" 30–50 cm</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>48</v>
-      </c>
-      <c r="D94" t="n">
-        <v>9</v>
+        <v>79</v>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
       </c>
     </row>
     <row r="95">
@@ -4042,14 +4045,16 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Tubex izolace 20×10 mm (2 m)</t>
+          <t>Perlátor M22/M24</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>12</v>
-      </c>
-      <c r="D95" t="n">
-        <v>14</v>
+        <v>39</v>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
       </c>
     </row>
     <row r="96">
@@ -4060,21 +4065,14 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Těsnění gumová sada 1/2"–3/4"</t>
+          <t>Sprchová hadice 150 cm</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>25</v>
-      </c>
-      <c r="D96" t="inlineStr">
-        <is>
-          <t>doplnit</t>
-        </is>
-      </c>
-      <c r="E96" t="inlineStr">
-        <is>
-          <t>nejčastější havárie</t>
-        </is>
+        <v>245</v>
+      </c>
+      <c r="D96" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="97">
@@ -4085,11 +4083,11 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Flexi hadička 3/8" 30–50 cm</t>
+          <t>Sifon umyvadlový plast</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="D97" t="inlineStr">
         <is>
@@ -4105,49 +4103,61 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Perlátor M22/M24</t>
+          <t>Zahradní hadice 1/2" 20 m + rychlospojky</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>39</v>
+        <v>399</v>
       </c>
       <c r="D98" t="inlineStr">
         <is>
           <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>ověřit z dat prodejny 2</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Vodoinstalace</t>
+          <t>Spojovací materiál (blistry)</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Sprchová hadice 150 cm</t>
+          <t>Vruty do dřeva 3,5×30 (100 ks)</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>245</v>
-      </c>
-      <c r="D99" t="n">
-        <v>3</v>
+        <v>59</v>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>nejmenší běžná velikost</t>
+        </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Vodoinstalace</t>
+          <t>Spojovací materiál (blistry)</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Sifon umyvadlový plast</t>
+          <t>Vruty do dřeva 4×40 (100 ks)</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>89</v>
+        <v>69</v>
       </c>
       <c r="D100" t="inlineStr">
         <is>
@@ -4158,25 +4168,20 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Vodoinstalace</t>
+          <t>Spojovací materiál (blistry)</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Zahradní hadice 1/2" 20 m + rychlospojky</t>
+          <t>Vruty do dřeva 4×50 (100 ks)</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>399</v>
+        <v>79</v>
       </c>
       <c r="D101" t="inlineStr">
         <is>
           <t>doplnit</t>
-        </is>
-      </c>
-      <c r="E101" t="inlineStr">
-        <is>
-          <t>ověřit z dat prodejny 2</t>
         </is>
       </c>
     </row>
@@ -4188,20 +4193,15 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Hmoždinky 6 / 8 / 10 mm (sady)</t>
+          <t>Vruty do dřeva 4,5×60 (50 ks)</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>39</v>
+        <v>79</v>
       </c>
       <c r="D102" t="inlineStr">
         <is>
           <t>doplnit</t>
-        </is>
-      </c>
-      <c r="E102" t="inlineStr">
-        <is>
-          <t>v datech kusový prodej</t>
         </is>
       </c>
     </row>
@@ -4213,11 +4213,11 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Vruty univerzální 4×40, 4×50, 5×60 (sady)</t>
+          <t>Vruty do dřeva 5×70 (50 ks)</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>59</v>
+        <v>89</v>
       </c>
       <c r="D103" t="inlineStr">
         <is>
@@ -4233,18 +4233,20 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Šrouby do plechu 2,9×13 (sada 50 ks)</t>
+          <t>Vruty do dřeva 6×80 / 6×100 (25 ks)</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>29</v>
-      </c>
-      <c r="D104" t="n">
-        <v>37</v>
+        <v>99</v>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>v datech 37 ks/měs po 0,40 Kč</t>
+          <t>terasy, konstrukce</t>
         </is>
       </c>
     </row>
@@ -4256,11 +4258,11 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Hřebíky 40 / 60 / 80 mm (sáček)</t>
+          <t>Vruty do sádrokartonu 3,5×25 a 3,5×35 (200 ks)</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>39</v>
+        <v>79</v>
       </c>
       <c r="D105" t="inlineStr">
         <is>
@@ -4276,15 +4278,18 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Skoby, háčky, oka (sada)</t>
+          <t>Šrouby do plechu 2,9×13 a 2,9×9,5 (50 ks)</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>39</v>
-      </c>
-      <c r="D106" t="inlineStr">
-        <is>
-          <t>doplnit</t>
+        <v>29</v>
+      </c>
+      <c r="D106" t="n">
+        <v>37</v>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>v datech 37 ks/měs po 0,30–0,40 Kč</t>
         </is>
       </c>
     </row>
@@ -4296,11 +4301,11 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Hmoždinka rámová 10×100 (sada)</t>
+          <t>Hmoždinky nylon 5 mm (50 ks)</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>79</v>
+        <v>39</v>
       </c>
       <c r="D107" t="inlineStr">
         <is>
@@ -4316,15 +4321,20 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Vázací drát pozink</t>
+          <t>Hmoždinky nylon 6 mm (50 ks)</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="D108" t="inlineStr">
         <is>
           <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>nejžádanější rozměr</t>
         </is>
       </c>
     </row>
@@ -4336,83 +4346,101 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Zárohák (hák do zdi)</t>
+          <t>Hmoždinky nylon 8 mm (50 ks)</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>69</v>
-      </c>
-      <c r="D109" t="n">
-        <v>5</v>
+        <v>55</v>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Ruční nářadí</t>
+          <t>Spojovací materiál (blistry)</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Svinovací metr 5 m</t>
+          <t>Hmoždinky nylon 10 mm (25 ks)</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>99</v>
-      </c>
-      <c r="D110" t="n">
-        <v>9</v>
+        <v>59</v>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Ruční nářadí</t>
+          <t>Spojovací materiál (blistry)</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Odlamovací nůž 18 mm kovový</t>
+          <t>Hmoždinka s vrutem 6×40 a 8×60 (20 ks)</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>89</v>
-      </c>
-      <c r="D111" t="n">
-        <v>7</v>
+        <v>79</v>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>natloukací, na lišty</t>
+        </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Ruční nářadí</t>
+          <t>Spojovací materiál (blistry)</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Náhradní čepele 18 mm 10 ks</t>
+          <t>Hmoždinka rámová 10×100 / 10×135 (10 ks)</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>40</v>
-      </c>
-      <c r="D112" t="n">
-        <v>12</v>
+        <v>89</v>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>okna, zárubně</t>
+        </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Ruční nářadí</t>
+          <t>Spojovací materiál (blistry)</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Šroubovák s bity (ráčna + 20 bitů)</t>
+          <t>Hmoždinka do dutin (sádrokarton) sada</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>199</v>
+        <v>79</v>
       </c>
       <c r="D113" t="inlineStr">
         <is>
@@ -4423,16 +4451,16 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Ruční nářadí</t>
+          <t>Spojovací materiál (blistry)</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Kleště kombinované 180 mm</t>
+          <t>Šrouby M6 a M8 s maticí a podložkou (sada)</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>149</v>
+        <v>69</v>
       </c>
       <c r="D114" t="inlineStr">
         <is>
@@ -4443,16 +4471,16 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Ruční nářadí</t>
+          <t>Spojovací materiál (blistry)</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Kladivo 300 g</t>
+          <t>Matice M6/M8/M10 (sada)</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>129</v>
+        <v>39</v>
       </c>
       <c r="D115" t="inlineStr">
         <is>
@@ -4463,34 +4491,36 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Ruční nářadí</t>
+          <t>Spojovací materiál (blistry)</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Ocelový kartáč 5řadý</t>
+          <t>Podložky ploché a pružné (sada mix)</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>68</v>
-      </c>
-      <c r="D116" t="n">
-        <v>5</v>
+        <v>39</v>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Ruční nářadí</t>
+          <t>Spojovací materiál (blistry)</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Pilka na kov / pilový list</t>
+          <t>Hřebíky 40 / 60 / 80 mm (sáček 0,5 kg)</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>99</v>
+        <v>49</v>
       </c>
       <c r="D117" t="inlineStr">
         <is>
@@ -4501,16 +4531,16 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Ruční nářadí</t>
+          <t>Spojovací materiál (blistry)</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Vodováha 40 cm</t>
+          <t>Hřebíčky čalounické a lepenkové (sáček)</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>99</v>
+        <v>29</v>
       </c>
       <c r="D118" t="inlineStr">
         <is>
@@ -4521,12 +4551,12 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Ruční nářadí</t>
+          <t>Spojovací materiál (blistry)</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Sada imbus klíčů</t>
+          <t>Závitová tyč M8 1 m</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -4541,93 +4571,100 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Ruční nářadí</t>
+          <t>Spojovací materiál (blistry)</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Zavírací nůž</t>
+          <t>Skoby, háky do zdi, oka (sada)</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>163</v>
-      </c>
-      <c r="D120" t="n">
-        <v>4</v>
+        <v>39</v>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Ruční nářadí</t>
+          <t>Spojovací materiál (blistry)</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Vědro stavební 12 l</t>
+          <t>Zárohák (hák do zdi)</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>49</v>
+        <v>69</v>
       </c>
       <c r="D121" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>Ochranné pomůcky</t>
+          <t>Spojovací materiál (blistry)</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Pracovní rukavice vel. 8 / 9 / 10 / 11</t>
+          <t>Chemická kotva 165 / 300 ml</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>59</v>
+        <v>190</v>
       </c>
       <c r="D122" t="n">
-        <v>30</v>
+        <v>7</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>celá řada velikostí</t>
+          <t>prodává se 7 ks/měs</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Ochranné pomůcky</t>
+          <t>Spojovací materiál (blistry)</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Rukavice profi 1+1</t>
+          <t>Vázací pásky 200 / 300 / 500 mm (50 ks)</t>
         </is>
       </c>
       <c r="C123" t="n">
-        <v>28</v>
+        <v>59</v>
       </c>
       <c r="D123" t="n">
-        <v>5</v>
+        <v>42</v>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>42 ks/měs, marže 70–190 %</t>
+        </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Ochranné pomůcky</t>
+          <t>Spojovací materiál (blistry)</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>Jednorázové nitrilové rukavice (10 ks)</t>
+          <t>Vázací drát pozink 50 m</t>
         </is>
       </c>
       <c r="C124" t="n">
-        <v>39</v>
+        <v>49</v>
       </c>
       <c r="D124" t="inlineStr">
         <is>
@@ -4638,590 +4675,620 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Ochranné pomůcky</t>
+          <t>Spojovací materiál (blistry)</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Zátky do uší</t>
+          <t>Karabiny a řetěz po 1 m</t>
         </is>
       </c>
       <c r="C125" t="n">
-        <v>10</v>
-      </c>
-      <c r="D125" t="n">
-        <v>3</v>
+        <v>59</v>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Ochranné pomůcky</t>
+          <t>Spojovací materiál (blistry)</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Respirátor FFP2 (2 ks)</t>
+          <t>Trhací nýty 4×10 (50 ks)</t>
         </is>
       </c>
       <c r="C126" t="n">
-        <v>39</v>
+        <v>59</v>
       </c>
       <c r="D126" t="inlineStr">
         <is>
           <t>doplnit</t>
-        </is>
-      </c>
-      <c r="E126" t="inlineStr">
-        <is>
-          <t>broušení, barvy</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>Ochranné pomůcky</t>
+          <t>Barvy na zeď a nátěry</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Ochranné brýle</t>
+          <t>Het Klasik otěruvzdorný 15+3 kg</t>
         </is>
       </c>
       <c r="C127" t="n">
-        <v>49</v>
-      </c>
-      <c r="D127" t="inlineStr">
-        <is>
-          <t>doplnit</t>
+        <v>799</v>
+      </c>
+      <c r="D127" t="n">
+        <v>15</v>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>nejsilnější položka do 1 000 Kč</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>Technická chemie</t>
+          <t>Barvy na zeď a nátěry</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Ředidlo S6006 0,7 l</t>
+          <t>Het Klasik otěruvzdorný 7+1 kg</t>
         </is>
       </c>
       <c r="C128" t="n">
-        <v>85</v>
+        <v>459</v>
       </c>
       <c r="D128" t="n">
-        <v>21</v>
-      </c>
-      <c r="E128" t="inlineStr">
-        <is>
-          <t>hořlavina – ověřit požární předpisy</t>
-        </is>
+        <v>3</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Technická chemie</t>
+          <t>Barvy na zeď a nátěry</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Ředidlo S6005 0,7 l</t>
+          <t>Het Klasik otěruvzdorný 4 kg</t>
         </is>
       </c>
       <c r="C129" t="n">
-        <v>95</v>
+        <v>319</v>
       </c>
       <c r="D129" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>Technická chemie</t>
+          <t>Barvy na zeď a nátěry</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>Nitroředidlo C6000 0,7 l</t>
+          <t>Het Klasik 1,5 kg</t>
         </is>
       </c>
       <c r="C130" t="n">
-        <v>95</v>
+        <v>150</v>
       </c>
       <c r="D130" t="n">
-        <v>9</v>
+        <v>5</v>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>malá oprava, nejnižší cena</t>
+        </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>Technická chemie</t>
+          <t>Barvy na zeď a nátěry</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>Líh technický 0,7 l</t>
+          <t>Primalex Polar 15+3 kg</t>
         </is>
       </c>
       <c r="C131" t="n">
-        <v>98</v>
+        <v>999</v>
       </c>
       <c r="D131" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>Technická chemie</t>
+          <t>Barvy na zeď a nátěry</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>Lakový benzín 0,7 l</t>
+          <t>Primalex Polar / Standard 7,5 kg</t>
         </is>
       </c>
       <c r="C132" t="n">
-        <v>109</v>
+        <v>500</v>
       </c>
       <c r="D132" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>Technická chemie</t>
+          <t>Barvy na zeď a nátěry</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>WD-40 / univerzální mazivo sprej 200 ml</t>
+          <t>Malířské vápno 11 kg / bílení 6 kg</t>
         </is>
       </c>
       <c r="C133" t="n">
-        <v>129</v>
-      </c>
-      <c r="D133" t="inlineStr">
-        <is>
-          <t>doplnit</t>
+        <v>250</v>
+      </c>
+      <c r="D133" t="n">
+        <v>4</v>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>sklepy, hospodářské budovy</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>Technická chemie</t>
+          <t>Barvy na zeď a nátěry</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>Odrezovač 0,5 l</t>
+          <t>Penetrace akrylátová 1 l</t>
         </is>
       </c>
       <c r="C134" t="n">
-        <v>112</v>
+        <v>69</v>
       </c>
       <c r="D134" t="n">
-        <v>3</v>
+        <v>2</v>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>patří k barvě, prodávat vedle</t>
+        </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>Technická chemie</t>
+          <t>Barvy na zeď a nátěry</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>Kyselina citronová 100 g</t>
+          <t>Protiplísňový nátěr / Remal 7,5 kg</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>22</v>
+        <v>533</v>
       </c>
       <c r="D135" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>Technická chemie</t>
+          <t>Barvy na zeď a nátěry</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>Vazelína bílá</t>
+          <t>Bochemit proti plísním 500 ml rozprašovač</t>
         </is>
       </c>
       <c r="C136" t="n">
-        <v>195</v>
+        <v>99</v>
       </c>
       <c r="D136" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>Technická chemie</t>
+          <t>Barvy na zeď a nátěry</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>Destilovaná voda 5 l</t>
+          <t>Eternal IN STOP izolační 1 kg</t>
         </is>
       </c>
       <c r="C137" t="n">
-        <v>70</v>
+        <v>309</v>
       </c>
       <c r="D137" t="n">
-        <v>6</v>
+        <v>2</v>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>na skvrny a fleky</t>
+        </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>Technická chemie</t>
+          <t>Barvy na zeď a nátěry</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>Nemrznoucí směs do ostřikovačů 3 l</t>
+          <t>Fasádní barva Remal 7,5 kg</t>
         </is>
       </c>
       <c r="C138" t="n">
-        <v>99</v>
-      </c>
-      <c r="D138" t="inlineStr">
-        <is>
-          <t>doplnit</t>
-        </is>
+        <v>639</v>
+      </c>
+      <c r="D138" t="n">
+        <v>1</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>sezónně</t>
+          <t>jen jedna velikost</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>Úklid</t>
+          <t>Barvy na zeď a nátěry</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>Savo Original 1,2 l</t>
+          <t>Lazura na dřevo 0,75 l (palisandr, ořech, teak)</t>
         </is>
       </c>
       <c r="C139" t="n">
-        <v>67</v>
+        <v>199</v>
       </c>
       <c r="D139" t="n">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>Luxol Originál</t>
+        </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>Úklid</t>
+          <t>Barvy na zeď a nátěry</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>Savo proti plísni 500 ml</t>
+          <t>Lak interiérový vodouředitelný 0,6 l mat a lesk</t>
         </is>
       </c>
       <c r="C140" t="n">
-        <v>99</v>
+        <v>275</v>
       </c>
       <c r="D140" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>Úklid</t>
+          <t>Barvy na zeď a nátěry</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>Domestos 750 ml / 2 l</t>
+          <t>Syntetický email bílý 0,6 l</t>
         </is>
       </c>
       <c r="C141" t="n">
-        <v>59</v>
+        <v>229</v>
       </c>
       <c r="D141" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>Úklid</t>
+          <t>Barvy na zeď a nátěry</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>Jar / prostředek na nádobí 900 ml</t>
+          <t>Základní barva na kov 0,6–0,75 l</t>
         </is>
       </c>
       <c r="C142" t="n">
-        <v>59</v>
-      </c>
-      <c r="D142" t="inlineStr">
-        <is>
-          <t>doplnit</t>
+        <v>200</v>
+      </c>
+      <c r="D142" t="n">
+        <v>10</v>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>Komaprim, syntetika primer</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>Úklid</t>
+          <t>Barvy na zeď a nátěry</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>Univerzální čistič (Ajax, Cif)</t>
+          <t>Alkyton 0,7–1 l přímo na rez</t>
         </is>
       </c>
       <c r="C143" t="n">
-        <v>59</v>
-      </c>
-      <c r="D143" t="inlineStr">
-        <is>
-          <t>doplnit</t>
+        <v>549</v>
+      </c>
+      <c r="D143" t="n">
+        <v>20</v>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>20 ks/měs, silná položka</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>Úklid</t>
+          <t>Barvy na zeď a nátěry</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>Pytle na odpad 60 l a 120 l</t>
+          <t>Laksil bezbarvý 0,7 kg</t>
         </is>
       </c>
       <c r="C144" t="n">
-        <v>39</v>
+        <v>499</v>
       </c>
       <c r="D144" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>Úklid</t>
+          <t>Barvy na zeď a nátěry</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>Houbičky na nádobí 5 ks</t>
+          <t>Míchací tyčka, sítko na lak, krycí papír</t>
         </is>
       </c>
       <c r="C145" t="n">
-        <v>25</v>
-      </c>
-      <c r="D145" t="inlineStr">
-        <is>
-          <t>doplnit</t>
+        <v>15</v>
+      </c>
+      <c r="D145" t="n">
+        <v>11</v>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>drobnost k barvě, marže 110–180 %</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>Úklid</t>
+          <t>Ruční nářadí</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>Hadr podlahový</t>
+          <t>Svinovací metr 5 m</t>
         </is>
       </c>
       <c r="C146" t="n">
-        <v>32</v>
+        <v>99</v>
       </c>
       <c r="D146" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>Úklid</t>
+          <t>Ruční nářadí</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>Osvěžovač vzduchu</t>
+          <t>Odlamovací nůž 18 mm kovový</t>
         </is>
       </c>
       <c r="C147" t="n">
-        <v>29</v>
+        <v>89</v>
       </c>
       <c r="D147" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>Úklid</t>
+          <t>Ruční nářadí</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>Solvina / Praganda (mycí pasta na ruce)</t>
+          <t>Náhradní čepele 18 mm 10 ks</t>
         </is>
       </c>
       <c r="C148" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="D148" t="n">
-        <v>15</v>
-      </c>
-      <c r="E148" t="inlineStr">
-        <is>
-          <t>typicky DIY</t>
-        </is>
+        <v>12</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>Úklid</t>
+          <t>Ruční nářadí</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>WC blok</t>
+          <t>Šroubovák s bity (ráčna + 20 bitů)</t>
         </is>
       </c>
       <c r="C149" t="n">
-        <v>39</v>
-      </c>
-      <c r="D149" t="n">
-        <v>5</v>
+        <v>199</v>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>Úklid</t>
+          <t>Ruční nářadí</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>Lopatka + smetáček</t>
+          <t>Kleště kombinované 180 mm</t>
         </is>
       </c>
       <c r="C150" t="n">
-        <v>49</v>
-      </c>
-      <c r="D150" t="n">
-        <v>6</v>
+        <v>149</v>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>Úklid</t>
+          <t>Ruční nářadí</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>Zamražovací / svačinové sáčky</t>
+          <t>Kladivo 300 g</t>
         </is>
       </c>
       <c r="C151" t="n">
-        <v>39</v>
-      </c>
-      <c r="D151" t="n">
-        <v>4</v>
+        <v>129</v>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>Hygiena</t>
+          <t>Ruční nářadí</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>Toaletní papír Jumbo / 8 rolí</t>
+          <t>Ocelový kartáč 5řadý</t>
         </is>
       </c>
       <c r="C152" t="n">
-        <v>39</v>
+        <v>68</v>
       </c>
       <c r="D152" t="n">
-        <v>30</v>
+        <v>5</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>Hygiena</t>
+          <t>Ruční nářadí</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>Papírové ručníky ZZ</t>
+          <t>Pilka na kov / pilový list</t>
         </is>
       </c>
       <c r="C153" t="n">
-        <v>45</v>
-      </c>
-      <c r="D153" t="n">
-        <v>15</v>
+        <v>99</v>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>Hygiena</t>
+          <t>Ruční nářadí</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>Kapesníky krabička 150 ks</t>
+          <t>Vodováha 40 cm</t>
         </is>
       </c>
       <c r="C154" t="n">
-        <v>38</v>
-      </c>
-      <c r="D154" t="n">
-        <v>3</v>
+        <v>99</v>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>Hygiena</t>
+          <t>Ruční nářadí</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>Kuchyňské utěrky 2 role</t>
+          <t>Sada imbus klíčů</t>
         </is>
       </c>
       <c r="C155" t="n">
-        <v>39</v>
+        <v>89</v>
       </c>
       <c r="D155" t="inlineStr">
         <is>
@@ -5232,290 +5299,291 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>Hubení škůdců</t>
+          <t>Ruční nářadí</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>Pastička na myši dřevo / kov</t>
+          <t>Zavírací nůž</t>
         </is>
       </c>
       <c r="C156" t="n">
-        <v>16</v>
+        <v>163</v>
       </c>
       <c r="D156" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>Hubení škůdců</t>
+          <t>Ruční nářadí</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>Nástraha na myši Ratimor 150 g</t>
+          <t>Vědro stavební 12 l</t>
         </is>
       </c>
       <c r="C157" t="n">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="D157" t="n">
-        <v>8</v>
-      </c>
-      <c r="E157" t="inlineStr">
-        <is>
-          <t>balení pro veřejnost</t>
-        </is>
+        <v>6</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>Hubení škůdců</t>
+          <t>Ochranné pomůcky</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>Lepová deska na myši</t>
+          <t>Pracovní rukavice vel. 8 / 9 / 10 / 11</t>
         </is>
       </c>
       <c r="C158" t="n">
-        <v>35</v>
+        <v>59</v>
       </c>
       <c r="D158" t="n">
-        <v>3</v>
+        <v>30</v>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>celá řada velikostí</t>
+        </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>Hubení škůdců</t>
+          <t>Ochranné pomůcky</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>Mucholapka</t>
+          <t>Rukavice profi 1+1</t>
         </is>
       </c>
       <c r="C159" t="n">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="D159" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>Hubení škůdců</t>
+          <t>Ochranné pomůcky</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>Feroset – lapač moučných molů</t>
+          <t>Jednorázové nitrilové rukavice (10 ks)</t>
         </is>
       </c>
       <c r="C160" t="n">
-        <v>16</v>
-      </c>
-      <c r="D160" t="n">
-        <v>8</v>
+        <v>39</v>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>Hubení škůdců</t>
+          <t>Ochranné pomůcky</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>Sprej na vosy / hmyz (Biolit)</t>
+          <t>Zátky do uší</t>
         </is>
       </c>
       <c r="C161" t="n">
-        <v>119</v>
-      </c>
-      <c r="D161" t="inlineStr">
-        <is>
-          <t>doplnit</t>
-        </is>
-      </c>
-      <c r="E161" t="inlineStr">
-        <is>
-          <t>léto</t>
-        </is>
+        <v>10</v>
+      </c>
+      <c r="D161" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>Hubení škůdců</t>
+          <t>Ochranné pomůcky</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>Proti mravencům (Bioformatox)</t>
+          <t>Respirátor FFP2 (2 ks)</t>
         </is>
       </c>
       <c r="C162" t="n">
-        <v>109</v>
-      </c>
-      <c r="D162" t="n">
-        <v>2</v>
+        <v>39</v>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>broušení, barvy</t>
+        </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>Topení a zapalování</t>
+          <t>Ochranné pomůcky</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>Pepo pevný podpalovač 40 ks</t>
+          <t>Ochranné brýle</t>
         </is>
       </c>
       <c r="C163" t="n">
-        <v>35</v>
-      </c>
-      <c r="D163" t="n">
-        <v>29</v>
-      </c>
-      <c r="E163" t="inlineStr">
-        <is>
-          <t>celoročně</t>
+        <v>49</v>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>doplnit</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>Topení a zapalování</t>
+          <t>Technická chemie</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>Tekutý podpalovač 1 l</t>
+          <t>Ředidlo S6006 0,7 l</t>
         </is>
       </c>
       <c r="C164" t="n">
-        <v>96</v>
+        <v>85</v>
       </c>
       <c r="D164" t="n">
-        <v>3</v>
+        <v>21</v>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>hořlavina – ověřit požární předpisy</t>
+        </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>Topení a zapalování</t>
+          <t>Technická chemie</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>Zapalovač kuchyňský dlouhý</t>
+          <t>Ředidlo S6005 0,7 l</t>
         </is>
       </c>
       <c r="C165" t="n">
-        <v>37</v>
+        <v>95</v>
       </c>
       <c r="D165" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>Topení a zapalování</t>
+          <t>Technická chemie</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>Zapalovače turbo (2 ks)</t>
+          <t>Nitroředidlo C6000 0,7 l</t>
         </is>
       </c>
       <c r="C166" t="n">
-        <v>15</v>
+        <v>95</v>
       </c>
       <c r="D166" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>Topení a zapalování</t>
+          <t>Technická chemie</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>Zápalky (balení 10 krabiček)</t>
+          <t>Líh technický 0,7 l</t>
         </is>
       </c>
       <c r="C167" t="n">
-        <v>25</v>
+        <v>98</v>
       </c>
       <c r="D167" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>Topení a zapalování</t>
+          <t>Technická chemie</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>Dřevěné uhlí 2,5 kg</t>
+          <t>Lakový benzín 0,7 l</t>
         </is>
       </c>
       <c r="C168" t="n">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="D168" t="n">
-        <v>3</v>
-      </c>
-      <c r="E168" t="inlineStr">
-        <is>
-          <t>sezónně</t>
-        </is>
+        <v>4</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>Svíčky</t>
+          <t>Technická chemie</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>Hřbitovní patrona 120 g a 180 g</t>
+          <t>WD-40 / univerzální mazivo sprej 200 ml</t>
         </is>
       </c>
       <c r="C169" t="n">
-        <v>28</v>
-      </c>
-      <c r="D169" t="n">
-        <v>18</v>
+        <v>129</v>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>Svíčky</t>
+          <t>Technická chemie</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>Svíčka Theresia 4,5 dne</t>
+          <t>Odrezovač 0,5 l</t>
         </is>
       </c>
       <c r="C170" t="n">
-        <v>47</v>
+        <v>112</v>
       </c>
       <c r="D170" t="n">
         <v>3</v>
@@ -5524,144 +5592,145 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>Svíčky</t>
+          <t>Technická chemie</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>Iluminační svíčky 10 ks</t>
+          <t>Kyselina citronová 100 g</t>
         </is>
       </c>
       <c r="C171" t="n">
-        <v>59</v>
+        <v>22</v>
       </c>
       <c r="D171" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>Svíčky</t>
+          <t>Technická chemie</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>Čajové svíčky 30 ks</t>
+          <t>Vazelína bílá</t>
         </is>
       </c>
       <c r="C172" t="n">
-        <v>49</v>
-      </c>
-      <c r="D172" t="inlineStr">
-        <is>
-          <t>doplnit</t>
-        </is>
+        <v>195</v>
+      </c>
+      <c r="D172" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>Domácnost</t>
+          <t>Technická chemie</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>Skřipce záclonové</t>
+          <t>Destilovaná voda 5 l</t>
         </is>
       </c>
       <c r="C173" t="n">
+        <v>70</v>
+      </c>
+      <c r="D173" t="n">
         <v>6</v>
-      </c>
-      <c r="D173" t="n">
-        <v>22</v>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>Domácnost</t>
+          <t>Technická chemie</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>Háčky samolepicí</t>
+          <t>Nemrznoucí směs do ostřikovačů 3 l</t>
         </is>
       </c>
       <c r="C174" t="n">
-        <v>30</v>
-      </c>
-      <c r="D174" t="n">
-        <v>5</v>
+        <v>99</v>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>sezónně</t>
+        </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>Domácnost</t>
+          <t>Úklid</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>Věšák nástěnný chrom</t>
+          <t>Savo Original 1,2 l</t>
         </is>
       </c>
       <c r="C175" t="n">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="D175" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>Domácnost</t>
+          <t>Úklid</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>Kolíčky na prádlo 24 ks</t>
+          <t>Savo proti plísni 500 ml</t>
         </is>
       </c>
       <c r="C176" t="n">
-        <v>39</v>
-      </c>
-      <c r="D176" t="inlineStr">
-        <is>
-          <t>doplnit</t>
-        </is>
+        <v>99</v>
+      </c>
+      <c r="D176" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>Domácnost</t>
+          <t>Úklid</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>Prádelní šňůra 20 m</t>
+          <t>Domestos 750 ml / 2 l</t>
         </is>
       </c>
       <c r="C177" t="n">
-        <v>49</v>
-      </c>
-      <c r="D177" t="inlineStr">
-        <is>
-          <t>doplnit</t>
-        </is>
+        <v>59</v>
+      </c>
+      <c r="D177" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>Domácnost</t>
+          <t>Úklid</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>Provázek / polypropylenové lano 20 m</t>
+          <t>Jar / prostředek na nádobí 900 ml</t>
         </is>
       </c>
       <c r="C178" t="n">
@@ -5676,153 +5745,842 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>Domácnost</t>
+          <t>Úklid</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>Kroužky na klíče + rozlišovače</t>
+          <t>Univerzální čistič (Ajax, Cif)</t>
         </is>
       </c>
       <c r="C179" t="n">
-        <v>4</v>
-      </c>
-      <c r="D179" t="n">
-        <v>46</v>
-      </c>
-      <c r="E179" t="inlineStr">
-        <is>
-          <t>u pokladny</t>
+        <v>59</v>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>doplnit</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>Domácnost</t>
+          <t>Úklid</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>Visací zámek 30 / 40 mm</t>
+          <t>Pytle na odpad 60 l a 120 l</t>
         </is>
       </c>
       <c r="C180" t="n">
-        <v>129</v>
-      </c>
-      <c r="D180" t="inlineStr">
-        <is>
-          <t>doplnit</t>
-        </is>
+        <v>39</v>
+      </c>
+      <c r="D180" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>Domácnost</t>
+          <t>Úklid</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>Magnety 10 ks</t>
+          <t>Houbičky na nádobí 5 ks</t>
         </is>
       </c>
       <c r="C181" t="n">
-        <v>50</v>
-      </c>
-      <c r="D181" t="n">
-        <v>3</v>
+        <v>25</v>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>Sezónní stojan (rotace)</t>
+          <t>Úklid</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>Semena zeleniny a květin (stojan)</t>
+          <t>Hadr podlahový</t>
         </is>
       </c>
       <c r="C182" t="n">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="D182" t="n">
-        <v>153</v>
-      </c>
-      <c r="E182" t="inlineStr">
-        <is>
-          <t>únor–květen, marže 40–100 %</t>
-        </is>
+        <v>4</v>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>Sezónní stojan (rotace)</t>
+          <t>Úklid</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>Barvy na vejce, obtisky</t>
+          <t>Osvěžovač vzduchu</t>
         </is>
       </c>
       <c r="C183" t="n">
-        <v>12</v>
+        <v>29</v>
       </c>
       <c r="D183" t="n">
-        <v>15</v>
-      </c>
-      <c r="E183" t="inlineStr">
-        <is>
-          <t>březen–duben</t>
-        </is>
+        <v>9</v>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>Sezónní stojan (rotace)</t>
+          <t>Úklid</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>Zavařovací víčka Twist, špejle, střeva</t>
+          <t>Solvina / Praganda (mycí pasta na ruce)</t>
         </is>
       </c>
       <c r="C184" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="D184" t="n">
         <v>15</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>červenec–říjen</t>
+          <t>typicky DIY</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
+          <t>Úklid</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>WC blok</t>
+        </is>
+      </c>
+      <c r="C185" t="n">
+        <v>39</v>
+      </c>
+      <c r="D185" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>Úklid</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>Lopatka + smetáček</t>
+        </is>
+      </c>
+      <c r="C186" t="n">
+        <v>49</v>
+      </c>
+      <c r="D186" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>Úklid</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>Zamražovací / svačinové sáčky</t>
+        </is>
+      </c>
+      <c r="C187" t="n">
+        <v>39</v>
+      </c>
+      <c r="D187" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>Hygiena</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>Toaletní papír Jumbo / 8 rolí</t>
+        </is>
+      </c>
+      <c r="C188" t="n">
+        <v>39</v>
+      </c>
+      <c r="D188" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>Hygiena</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>Papírové ručníky ZZ</t>
+        </is>
+      </c>
+      <c r="C189" t="n">
+        <v>45</v>
+      </c>
+      <c r="D189" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>Hygiena</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>Kapesníky krabička 150 ks</t>
+        </is>
+      </c>
+      <c r="C190" t="n">
+        <v>38</v>
+      </c>
+      <c r="D190" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>Hygiena</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>Kuchyňské utěrky 2 role</t>
+        </is>
+      </c>
+      <c r="C191" t="n">
+        <v>39</v>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>Hubení škůdců</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>Pastička na myši dřevo / kov</t>
+        </is>
+      </c>
+      <c r="C192" t="n">
+        <v>16</v>
+      </c>
+      <c r="D192" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>Hubení škůdců</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>Nástraha na myši Ratimor 150 g</t>
+        </is>
+      </c>
+      <c r="C193" t="n">
+        <v>42</v>
+      </c>
+      <c r="D193" t="n">
+        <v>8</v>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>balení pro veřejnost</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>Hubení škůdců</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>Lepová deska na myši</t>
+        </is>
+      </c>
+      <c r="C194" t="n">
+        <v>35</v>
+      </c>
+      <c r="D194" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>Hubení škůdců</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>Mucholapka</t>
+        </is>
+      </c>
+      <c r="C195" t="n">
+        <v>7</v>
+      </c>
+      <c r="D195" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>Hubení škůdců</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>Feroset – lapač moučných molů</t>
+        </is>
+      </c>
+      <c r="C196" t="n">
+        <v>16</v>
+      </c>
+      <c r="D196" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>Hubení škůdců</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>Sprej na vosy / hmyz (Biolit)</t>
+        </is>
+      </c>
+      <c r="C197" t="n">
+        <v>119</v>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>léto</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>Hubení škůdců</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>Proti mravencům (Bioformatox)</t>
+        </is>
+      </c>
+      <c r="C198" t="n">
+        <v>109</v>
+      </c>
+      <c r="D198" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>Topení a zapalování</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>Pepo pevný podpalovač 40 ks</t>
+        </is>
+      </c>
+      <c r="C199" t="n">
+        <v>35</v>
+      </c>
+      <c r="D199" t="n">
+        <v>29</v>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>celoročně</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>Topení a zapalování</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>Tekutý podpalovač 1 l</t>
+        </is>
+      </c>
+      <c r="C200" t="n">
+        <v>96</v>
+      </c>
+      <c r="D200" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>Topení a zapalování</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>Zapalovač kuchyňský dlouhý</t>
+        </is>
+      </c>
+      <c r="C201" t="n">
+        <v>37</v>
+      </c>
+      <c r="D201" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>Topení a zapalování</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>Zapalovače turbo (2 ks)</t>
+        </is>
+      </c>
+      <c r="C202" t="n">
+        <v>15</v>
+      </c>
+      <c r="D202" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>Topení a zapalování</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>Zápalky (balení 10 krabiček)</t>
+        </is>
+      </c>
+      <c r="C203" t="n">
+        <v>25</v>
+      </c>
+      <c r="D203" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>Topení a zapalování</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>Dřevěné uhlí 2,5 kg</t>
+        </is>
+      </c>
+      <c r="C204" t="n">
+        <v>112</v>
+      </c>
+      <c r="D204" t="n">
+        <v>3</v>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>sezónně</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>Svíčky</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>Hřbitovní patrona 120 g a 180 g</t>
+        </is>
+      </c>
+      <c r="C205" t="n">
+        <v>28</v>
+      </c>
+      <c r="D205" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>Svíčky</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>Svíčka Theresia 4,5 dne</t>
+        </is>
+      </c>
+      <c r="C206" t="n">
+        <v>47</v>
+      </c>
+      <c r="D206" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>Svíčky</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>Iluminační svíčky 10 ks</t>
+        </is>
+      </c>
+      <c r="C207" t="n">
+        <v>59</v>
+      </c>
+      <c r="D207" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>Svíčky</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>Čajové svíčky 30 ks</t>
+        </is>
+      </c>
+      <c r="C208" t="n">
+        <v>49</v>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>Domácnost</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>Skřipce záclonové</t>
+        </is>
+      </c>
+      <c r="C209" t="n">
+        <v>6</v>
+      </c>
+      <c r="D209" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>Domácnost</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>Háčky samolepicí</t>
+        </is>
+      </c>
+      <c r="C210" t="n">
+        <v>30</v>
+      </c>
+      <c r="D210" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>Domácnost</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>Věšák nástěnný chrom</t>
+        </is>
+      </c>
+      <c r="C211" t="n">
+        <v>62</v>
+      </c>
+      <c r="D211" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>Domácnost</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>Kolíčky na prádlo 24 ks</t>
+        </is>
+      </c>
+      <c r="C212" t="n">
+        <v>39</v>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>Domácnost</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>Prádelní šňůra 20 m</t>
+        </is>
+      </c>
+      <c r="C213" t="n">
+        <v>49</v>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>Domácnost</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>Provázek / polypropylenové lano 20 m</t>
+        </is>
+      </c>
+      <c r="C214" t="n">
+        <v>59</v>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>Domácnost</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>Kroužky na klíče + rozlišovače</t>
+        </is>
+      </c>
+      <c r="C215" t="n">
+        <v>4</v>
+      </c>
+      <c r="D215" t="n">
+        <v>46</v>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>u pokladny</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>Domácnost</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>Visací zámek 30 / 40 mm</t>
+        </is>
+      </c>
+      <c r="C216" t="n">
+        <v>129</v>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>Domácnost</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>Magnety 10 ks</t>
+        </is>
+      </c>
+      <c r="C217" t="n">
+        <v>50</v>
+      </c>
+      <c r="D217" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
           <t>Sezónní stojan (rotace)</t>
         </is>
       </c>
-      <c r="B185" t="inlineStr">
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>Semena zeleniny a květin (stojan)</t>
+        </is>
+      </c>
+      <c r="C218" t="n">
+        <v>25</v>
+      </c>
+      <c r="D218" t="n">
+        <v>153</v>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>únor–květen, marže 40–100 %</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>Sezónní stojan (rotace)</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>Barvy na vejce, obtisky</t>
+        </is>
+      </c>
+      <c r="C219" t="n">
+        <v>12</v>
+      </c>
+      <c r="D219" t="n">
+        <v>15</v>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>březen–duben</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>Sezónní stojan (rotace)</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>Zavařovací víčka Twist, špejle, střeva</t>
+        </is>
+      </c>
+      <c r="C220" t="n">
+        <v>40</v>
+      </c>
+      <c r="D220" t="n">
+        <v>15</v>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>červenec–říjen</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>Sezónní stojan (rotace)</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
         <is>
           <t>Posypová sůl 5 kg, škrabka na led</t>
         </is>
       </c>
-      <c r="C185" t="n">
+      <c r="C221" t="n">
         <v>79</v>
       </c>
-      <c r="D185" t="inlineStr">
+      <c r="D221" t="inlineStr">
         <is>
           <t>doplnit</t>
         </is>
       </c>
-      <c r="E185" t="inlineStr">
+      <c r="E221" t="inlineStr">
         <is>
           <t>listopad–únor</t>
         </is>
@@ -5834,6 +6592,739 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="80" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Odhad poptávky mimo otevírací dobu (Po–Pá 7–17, So 8–11). Skóre je expertní, ne z dat – účtenkový export by ho nahradil skutečností.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Skupina</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Naléhavost</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Víkend</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Podíl mimo dobu</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>ks/měs Solnice</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>ks/měs mimo dobu</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Obrat mimo dobu Kč bez DPH</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Proč</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Lepidla, tmely, silikony, PU pěny</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>4</v>
+      </c>
+      <c r="C4" t="n">
+        <v>4</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E4" t="n">
+        <v>358</v>
+      </c>
+      <c r="F4" t="n">
+        <v>179</v>
+      </c>
+      <c r="G4" t="n">
+        <v>17900</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Rozbité, odlepené, zatéká. Zároveň nutné pro víkendovou opravu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Malířské potřeby</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C5" t="n">
+        <v>5</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="E5" t="n">
+        <v>771</v>
+      </c>
+      <c r="F5" t="n">
+        <v>324</v>
+      </c>
+      <c r="G5" t="n">
+        <v>11240</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Fólie, štětce, brusivo, válečky. Kupuje se v pátek večer a v sobotu ráno před malováním.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Vodoinstalace a hadice</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="E6" t="n">
+        <v>420</v>
+      </c>
+      <c r="F6" t="n">
+        <v>218</v>
+      </c>
+      <c r="G6" t="n">
+        <v>8844</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Prasklá hadice, teče spoj. Havárie nečeká do pondělí.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Úklid a čisticí prostředky</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>3</v>
+      </c>
+      <c r="C7" t="n">
+        <v>3</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E7" t="n">
+        <v>314</v>
+      </c>
+      <c r="F7" t="n">
+        <v>126</v>
+      </c>
+      <c r="G7" t="n">
+        <v>6955</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Došlo Savo, pytle, houbičky. Uklízí se hlavně o víkendu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Nátěrové hmoty (barvy na zeď)</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>2</v>
+      </c>
+      <c r="C8" t="n">
+        <v>5</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="E8" t="n">
+        <v>54</v>
+      </c>
+      <c r="F8" t="n">
+        <v>23</v>
+      </c>
+      <c r="G8" t="n">
+        <v>6767</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Malování je víkendová akce. Chybí-li barva v sobotu, projekt stojí.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Ředidla a technická chemie</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>2</v>
+      </c>
+      <c r="C9" t="n">
+        <v>4</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="E9" t="n">
+        <v>190</v>
+      </c>
+      <c r="F9" t="n">
+        <v>72</v>
+      </c>
+      <c r="G9" t="n">
+        <v>6444</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Ředidlo a líh k víkendovému natírání a čištění.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Elektroinstalační drobný materiál</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>4</v>
+      </c>
+      <c r="C10" t="n">
+        <v>3</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="E10" t="n">
+        <v>328</v>
+      </c>
+      <c r="F10" t="n">
+        <v>151</v>
+      </c>
+      <c r="G10" t="n">
+        <v>6235</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Vyhozená pojistka, utržená vidlice, prodlužovačka.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Lepicí a maskovací pásky</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>3</v>
+      </c>
+      <c r="C11" t="n">
+        <v>5</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="E11" t="n">
+        <v>256</v>
+      </c>
+      <c r="F11" t="n">
+        <v>123</v>
+      </c>
+      <c r="G11" t="n">
+        <v>5382</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Bez maskovací pásky se nedá malovat, bez izolepy dodělat oprava.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Ruční nářadí a měřidla</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>3</v>
+      </c>
+      <c r="C12" t="n">
+        <v>4</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="E12" t="n">
+        <v>125</v>
+      </c>
+      <c r="F12" t="n">
+        <v>55</v>
+      </c>
+      <c r="G12" t="n">
+        <v>4818</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Zlomená čepel, ztracený metr, chybí šroubovák.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Baterie</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>5</v>
+      </c>
+      <c r="C13" t="n">
+        <v>2</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="E13" t="n">
+        <v>389</v>
+      </c>
+      <c r="F13" t="n">
+        <v>187</v>
+      </c>
+      <c r="G13" t="n">
+        <v>3549</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Vybité ovladače, hlásiče, hračky, svítilny. Klasický večerní a nedělní nákup.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Ochranné pomůcky</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>3</v>
+      </c>
+      <c r="C14" t="n">
+        <v>4</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="E14" t="n">
+        <v>88</v>
+      </c>
+      <c r="F14" t="n">
+        <v>39</v>
+      </c>
+      <c r="G14" t="n">
+        <v>3520</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Rukavice, brýle, respirátor k víkendové práci.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Stavební chemie a sádra</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>2</v>
+      </c>
+      <c r="C15" t="n">
+        <v>4</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="E15" t="n">
+        <v>67</v>
+      </c>
+      <c r="F15" t="n">
+        <v>25</v>
+      </c>
+      <c r="G15" t="n">
+        <v>3303</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Sádra k zaplácnutí díry, lepidlo na obklady.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Kabely a vodiče</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>3</v>
+      </c>
+      <c r="C16" t="n">
+        <v>3</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E16" t="n">
+        <v>300</v>
+      </c>
+      <c r="F16" t="n">
+        <v>120</v>
+      </c>
+      <c r="G16" t="n">
+        <v>3273</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Prodlužovačka a kabel k opravě.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Žárovky a světelné zdroje</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>5</v>
+      </c>
+      <c r="C17" t="n">
+        <v>2</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="E17" t="n">
+        <v>142</v>
+      </c>
+      <c r="F17" t="n">
+        <v>68</v>
+      </c>
+      <c r="G17" t="n">
+        <v>2929</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Přestane svítit večer. Nákup nesnese odklad a nedá se odložit na pracovní den.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Spojovací materiál</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>3</v>
+      </c>
+      <c r="C18" t="n">
+        <v>5</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="E18" t="n">
+        <v>174</v>
+      </c>
+      <c r="F18" t="n">
+        <v>84</v>
+      </c>
+      <c r="G18" t="n">
+        <v>2761</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Došly vruty nebo hmoždinky uprostřed víkendové práce. Typický dokup.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Semena a ochrana rostlin</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>1</v>
+      </c>
+      <c r="C19" t="n">
+        <v>5</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="E19" t="n">
+        <v>190</v>
+      </c>
+      <c r="F19" t="n">
+        <v>68</v>
+      </c>
+      <c r="G19" t="n">
+        <v>2035</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Sází se o víkendu, sezónní špička únor–květen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Domácnost (věšáky, šňůry, háčky)</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>2</v>
+      </c>
+      <c r="C20" t="n">
+        <v>3</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="E20" t="n">
+        <v>138</v>
+      </c>
+      <c r="F20" t="n">
+        <v>47</v>
+      </c>
+      <c r="G20" t="n">
+        <v>1745</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Drobné doplňky k úklidu a zabydlení.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Podpalovače, topení, zapalování</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>4</v>
+      </c>
+      <c r="C21" t="n">
+        <v>3</v>
+      </c>
+      <c r="D21" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="E21" t="n">
+        <v>65</v>
+      </c>
+      <c r="F21" t="n">
+        <v>30</v>
+      </c>
+      <c r="G21" t="n">
+        <v>1236</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Podpalovač a zapalovač dojdou v sobotu večer, topí se i v neděli.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Hubení škůdců</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>4</v>
+      </c>
+      <c r="C22" t="n">
+        <v>2</v>
+      </c>
+      <c r="D22" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="E22" t="n">
+        <v>68</v>
+      </c>
+      <c r="F22" t="n">
+        <v>29</v>
+      </c>
+      <c r="G22" t="n">
+        <v>1157</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Myš v domě nebo vosy se neřeší za tři dny.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Hygiena a papírové zboží</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>4</v>
+      </c>
+      <c r="C23" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="E23" t="n">
+        <v>101</v>
+      </c>
+      <c r="F23" t="n">
+        <v>38</v>
+      </c>
+      <c r="G23" t="n">
+        <v>1047</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Došel toaletní papír. Nejbanálnější nouzový nákup.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Papírnictví</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>2</v>
+      </c>
+      <c r="C24" t="n">
+        <v>2</v>
+      </c>
+      <c r="D24" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E24" t="n">
+        <v>82</v>
+      </c>
+      <c r="F24" t="n">
+        <v>25</v>
+      </c>
+      <c r="G24" t="n">
+        <v>813</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Popisovač, sáčky. Doplňkový nákup.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Svíčky a hřbitovní zboží</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>2</v>
+      </c>
+      <c r="C25" t="n">
+        <v>4</v>
+      </c>
+      <c r="D25" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="E25" t="n">
+        <v>42</v>
+      </c>
+      <c r="F25" t="n">
+        <v>16</v>
+      </c>
+      <c r="G25" t="n">
+        <v>514</v>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Návštěva hřbitova je nedělní a svátek (Dušičky, Vánoce), kdy je zavřeno.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7663,7 +9154,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -28853,7 +30344,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Rework assortment and add market and security research
Assortment: drop everyday cleaning products and leave fishing out, add a
12-item spray section and a 16-item building-materials section (tile
adhesive, cement, post concrete, render, penetration), expand fasteners to
41 items and Den Braven goods to 24. Now 258 items, 162k CZK/month in
Solnice, so the forecast is recomputed: realistic scenario 1,012k CZK/year
and only 11k short of covering fixed costs.

Research: koncepty-a-zabezpeceni.md covers unattended-store concepts abroad
and in Czechia (including the ALTARA 24/7 self-service hardware store in
Decin), Czech legal requirements, anti-theft technology with prices and a
recommended lean and full stack. Corrosives are excluded from the
assortment on the strength of it.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01H9fdgZQbPRfobYczG68Y19
</commit_message>
<xml_diff>
--- a/analyzy/bezobsluzny-obchod/sortiment_24-7_analyza.xlsx
+++ b/analyzy/bezobsluzny-obchod/sortiment_24-7_analyza.xlsx
@@ -492,17 +492,17 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>160897</v>
+        <v>179767</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>160897</v>
+        <v>179767</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>160897</v>
+        <v>179767</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Z listu Zakladni sortiment, 145 293 Kč v okně březen/duben, přepočteno sezónním indexem</t>
+          <t>Z listu Zakladni sortiment, 162 333 Kč v okně březen/duben, přepočteno sezónním indexem</t>
         </is>
       </c>
     </row>
@@ -2180,7 +2180,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E221"/>
+  <dimension ref="A1:E259"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -3647,190 +3647,201 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Malířské potřeby</t>
+          <t>Lepidla, tmely, pěny</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Zakrývací fólie 4×5 m</t>
+          <t>MAMUT GLUE MULTI 290 ml šedý</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>25</v>
+        <v>221</v>
       </c>
       <c r="D75" t="n">
-        <v>63</v>
-      </c>
-      <c r="E75" t="inlineStr">
-        <is>
-          <t>nejprodávanější kus prodejny</t>
-        </is>
+        <v>4</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Malířské potřeby</t>
+          <t>Lepidla, tmely, pěny</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Zakrývací plachta 4×12,5 m</t>
+          <t>MAMUT GLUE TOTAL 290 ml bílý</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>55</v>
+        <v>249</v>
       </c>
       <c r="D76" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Malířské potřeby</t>
+          <t>Lepidla, tmely, pěny</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Štětec plochý 40 / 50 / 70 mm</t>
+          <t>MAMUT GLUE CRYSTAL 290 ml transparentní</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>37</v>
+        <v>235</v>
       </c>
       <c r="D77" t="n">
-        <v>26</v>
+        <v>4</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Malířské potřeby</t>
+          <t>Lepidla, tmely, pěny</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Váleček velvet 10 cm + držadlo</t>
+          <t>Akrylový tmel 310 ml bílý</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>22</v>
+        <v>73</v>
       </c>
       <c r="D78" t="n">
-        <v>10</v>
+        <v>4</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>nejlevnější tmel do spár</t>
+        </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Malířské potřeby</t>
+          <t>Lepidla, tmely, pěny</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Váleček 18 / 25 cm + rukojeť</t>
+          <t>Akrylový štukový tmel 310 ml bílý</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>90</v>
+        <v>125</v>
       </c>
       <c r="D79" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Malířské potřeby</t>
+          <t>Lepidla, tmely, pěny</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Malířská mřížka / vanička</t>
+          <t>Lehčený brousitelný tmel Qualy Fill 500 ml</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>39</v>
-      </c>
-      <c r="D80" t="inlineStr">
-        <is>
-          <t>doplnit</t>
-        </is>
+        <v>149</v>
+      </c>
+      <c r="D80" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Malířské potřeby</t>
+          <t>Lepidla, tmely, pěny</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Brusné plátno 60 / 80 / 120</t>
+          <t>Lepidlo ve spreji butylové 400 ml</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>17</v>
+        <v>289</v>
       </c>
       <c r="D81" t="n">
-        <v>35</v>
+        <v>4</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Malířské potřeby</t>
+          <t>Lepidla, tmely, pěny</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Brusný papír pod vodu 600 / 800</t>
+          <t>Těsnicí guma K a D profil 9 mm × 6 m</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>15</v>
+        <v>95</v>
       </c>
       <c r="D82" t="n">
-        <v>20</v>
+        <v>7</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>okna a dveře, podzim</t>
+        </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Malířské potřeby</t>
+          <t>Lepidla, tmely, pěny</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Špachtle 60 mm a 100 mm</t>
+          <t>Zakrývací fólie stavební 4×5 m 40 µm</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>39</v>
-      </c>
-      <c r="D83" t="inlineStr">
-        <is>
-          <t>doplnit</t>
+        <v>99</v>
+      </c>
+      <c r="D83" t="n">
+        <v>4</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>silnější než malířská</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Malířské potřeby</t>
+          <t>Lepidla, tmely, pěny</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Míchací pohár 385 ml</t>
+          <t>Stretch fólie ruční 50 cm</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>21</v>
+        <v>249</v>
       </c>
       <c r="D84" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>marže 208 %</t>
+        </is>
       </c>
     </row>
     <row r="85">
@@ -3841,1376 +3852,1349 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Nopová fólie 0,5 m a 1 m × 20 m</t>
+          <t>Zakrývací fólie 4×5 m</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>38</v>
+        <v>25</v>
       </c>
       <c r="D85" t="n">
-        <v>40</v>
+        <v>63</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>izolace základů, silný prodej</t>
+          <t>nejprodávanější kus prodejny</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Vodoinstalace</t>
+          <t>Malířské potřeby</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Hadicové spony 8–12 / 12–20 / 16–25 / 20–32 / 25–40 / 32–50</t>
+          <t>Zakrývací plachta 4×12,5 m</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>9</v>
+        <v>55</v>
       </c>
       <c r="D86" t="n">
-        <v>77</v>
-      </c>
-      <c r="E86" t="inlineStr">
-        <is>
-          <t>celá řada</t>
-        </is>
+        <v>16</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Vodoinstalace</t>
+          <t>Malířské potřeby</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Objímka trubková 2-šroub 31–38 mm</t>
+          <t>Štětec plochý 40 / 50 / 70 mm</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>16</v>
+        <v>37</v>
       </c>
       <c r="D87" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Vodoinstalace</t>
+          <t>Malířské potřeby</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Objímka trubková 2-šroub 54–59 mm</t>
+          <t>Váleček velvet 10 cm + držadlo</t>
         </is>
       </c>
       <c r="C88" t="n">
         <v>22</v>
       </c>
       <c r="D88" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Vodoinstalace</t>
+          <t>Malířské potřeby</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Příchytka na potrubí 20 / 25 mm</t>
+          <t>Váleček 18 / 25 cm + rukojeť</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>8</v>
+        <v>90</v>
       </c>
       <c r="D89" t="n">
-        <v>17</v>
+        <v>9</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Vodoinstalace</t>
+          <t>Malířské potřeby</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>PPR koleno 90° 20 mm, T-kus 20, nátrubek 20</t>
+          <t>Malířská mřížka / vanička</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>8</v>
-      </c>
-      <c r="D90" t="n">
-        <v>15</v>
-      </c>
-      <c r="E90" t="inlineStr">
-        <is>
-          <t>jen dimenze 20 a 25</t>
+        <v>39</v>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>doplnit</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Vodoinstalace</t>
+          <t>Malířské potřeby</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Mosazná vsuvka 3/4", 1/2"</t>
+          <t>Brusné plátno 60 / 80 / 120</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>48</v>
+        <v>17</v>
       </c>
       <c r="D91" t="n">
-        <v>9</v>
+        <v>35</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Vodoinstalace</t>
+          <t>Malířské potřeby</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Tubex izolace 20×10 mm (2 m)</t>
+          <t>Brusný papír pod vodu 600 / 800</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D92" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Vodoinstalace</t>
+          <t>Malířské potřeby</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Těsnění gumová sada 1/2"–3/4"</t>
+          <t>Špachtle 60 mm a 100 mm</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>25</v>
+        <v>39</v>
       </c>
       <c r="D93" t="inlineStr">
         <is>
           <t>doplnit</t>
-        </is>
-      </c>
-      <c r="E93" t="inlineStr">
-        <is>
-          <t>nejčastější havárie</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Vodoinstalace</t>
+          <t>Malířské potřeby</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Flexi hadička 3/8" 30–50 cm</t>
+          <t>Míchací pohár 385 ml</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>79</v>
-      </c>
-      <c r="D94" t="inlineStr">
-        <is>
-          <t>doplnit</t>
-        </is>
+        <v>21</v>
+      </c>
+      <c r="D94" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Vodoinstalace</t>
+          <t>Malířské potřeby</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Perlátor M22/M24</t>
+          <t>Nopová fólie 0,5 m a 1 m × 20 m</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>39</v>
-      </c>
-      <c r="D95" t="inlineStr">
-        <is>
-          <t>doplnit</t>
+        <v>38</v>
+      </c>
+      <c r="D95" t="n">
+        <v>40</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>izolace základů, silný prodej</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Vodoinstalace</t>
+          <t>Barvy na zeď a nátěry</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Sprchová hadice 150 cm</t>
+          <t>Het Klasik otěruvzdorný 15+3 kg</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>245</v>
+        <v>799</v>
       </c>
       <c r="D96" t="n">
-        <v>3</v>
+        <v>15</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>nejsilnější položka do 1 000 Kč</t>
+        </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Vodoinstalace</t>
+          <t>Barvy na zeď a nátěry</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Sifon umyvadlový plast</t>
+          <t>Het Klasik otěruvzdorný 7+1 kg</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>89</v>
-      </c>
-      <c r="D97" t="inlineStr">
-        <is>
-          <t>doplnit</t>
-        </is>
+        <v>459</v>
+      </c>
+      <c r="D97" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Vodoinstalace</t>
+          <t>Barvy na zeď a nátěry</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Zahradní hadice 1/2" 20 m + rychlospojky</t>
+          <t>Het Klasik otěruvzdorný 4 kg</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>399</v>
-      </c>
-      <c r="D98" t="inlineStr">
-        <is>
-          <t>doplnit</t>
-        </is>
-      </c>
-      <c r="E98" t="inlineStr">
-        <is>
-          <t>ověřit z dat prodejny 2</t>
-        </is>
+        <v>319</v>
+      </c>
+      <c r="D98" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Spojovací materiál (blistry)</t>
+          <t>Barvy na zeď a nátěry</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Vruty do dřeva 3,5×30 (100 ks)</t>
+          <t>Het Klasik 1,5 kg</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>59</v>
-      </c>
-      <c r="D99" t="inlineStr">
-        <is>
-          <t>doplnit</t>
-        </is>
+        <v>150</v>
+      </c>
+      <c r="D99" t="n">
+        <v>5</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>nejmenší běžná velikost</t>
+          <t>malá oprava, nejnižší cena</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Spojovací materiál (blistry)</t>
+          <t>Barvy na zeď a nátěry</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Vruty do dřeva 4×40 (100 ks)</t>
+          <t>Primalex Polar 15+3 kg</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>69</v>
-      </c>
-      <c r="D100" t="inlineStr">
-        <is>
-          <t>doplnit</t>
-        </is>
+        <v>999</v>
+      </c>
+      <c r="D100" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Spojovací materiál (blistry)</t>
+          <t>Barvy na zeď a nátěry</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Vruty do dřeva 4×50 (100 ks)</t>
+          <t>Primalex Polar / Standard 7,5 kg</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>79</v>
-      </c>
-      <c r="D101" t="inlineStr">
-        <is>
-          <t>doplnit</t>
-        </is>
+        <v>500</v>
+      </c>
+      <c r="D101" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Spojovací materiál (blistry)</t>
+          <t>Barvy na zeď a nátěry</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Vruty do dřeva 4,5×60 (50 ks)</t>
+          <t>Malířské vápno 11 kg / bílení 6 kg</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>79</v>
-      </c>
-      <c r="D102" t="inlineStr">
-        <is>
-          <t>doplnit</t>
+        <v>250</v>
+      </c>
+      <c r="D102" t="n">
+        <v>4</v>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>sklepy, hospodářské budovy</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Spojovací materiál (blistry)</t>
+          <t>Barvy na zeď a nátěry</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Vruty do dřeva 5×70 (50 ks)</t>
+          <t>Penetrace akrylátová 1 l</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>89</v>
-      </c>
-      <c r="D103" t="inlineStr">
-        <is>
-          <t>doplnit</t>
+        <v>69</v>
+      </c>
+      <c r="D103" t="n">
+        <v>2</v>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>patří k barvě, prodávat vedle</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Spojovací materiál (blistry)</t>
+          <t>Barvy na zeď a nátěry</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Vruty do dřeva 6×80 / 6×100 (25 ks)</t>
+          <t>Protiplísňový nátěr / Remal 7,5 kg</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>99</v>
-      </c>
-      <c r="D104" t="inlineStr">
-        <is>
-          <t>doplnit</t>
-        </is>
-      </c>
-      <c r="E104" t="inlineStr">
-        <is>
-          <t>terasy, konstrukce</t>
-        </is>
+        <v>533</v>
+      </c>
+      <c r="D104" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Spojovací materiál (blistry)</t>
+          <t>Barvy na zeď a nátěry</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Vruty do sádrokartonu 3,5×25 a 3,5×35 (200 ks)</t>
+          <t>Bochemit proti plísním 500 ml rozprašovač</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>79</v>
-      </c>
-      <c r="D105" t="inlineStr">
-        <is>
-          <t>doplnit</t>
-        </is>
+        <v>99</v>
+      </c>
+      <c r="D105" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Spojovací materiál (blistry)</t>
+          <t>Barvy na zeď a nátěry</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Šrouby do plechu 2,9×13 a 2,9×9,5 (50 ks)</t>
+          <t>Eternal IN STOP izolační 1 kg</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>29</v>
+        <v>309</v>
       </c>
       <c r="D106" t="n">
-        <v>37</v>
+        <v>2</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>v datech 37 ks/měs po 0,30–0,40 Kč</t>
+          <t>na skvrny a fleky</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Spojovací materiál (blistry)</t>
+          <t>Barvy na zeď a nátěry</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Hmoždinky nylon 5 mm (50 ks)</t>
+          <t>Fasádní barva Remal 7,5 kg</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>39</v>
-      </c>
-      <c r="D107" t="inlineStr">
-        <is>
-          <t>doplnit</t>
+        <v>639</v>
+      </c>
+      <c r="D107" t="n">
+        <v>1</v>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>jen jedna velikost</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Spojovací materiál (blistry)</t>
+          <t>Barvy na zeď a nátěry</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Hmoždinky nylon 6 mm (50 ks)</t>
+          <t>Lazura na dřevo 0,75 l (palisandr, ořech, teak)</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>45</v>
-      </c>
-      <c r="D108" t="inlineStr">
-        <is>
-          <t>doplnit</t>
-        </is>
+        <v>199</v>
+      </c>
+      <c r="D108" t="n">
+        <v>6</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>nejžádanější rozměr</t>
+          <t>Luxol Originál</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Spojovací materiál (blistry)</t>
+          <t>Barvy na zeď a nátěry</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Hmoždinky nylon 8 mm (50 ks)</t>
+          <t>Lak interiérový vodouředitelný 0,6 l mat a lesk</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>55</v>
-      </c>
-      <c r="D109" t="inlineStr">
-        <is>
-          <t>doplnit</t>
-        </is>
+        <v>275</v>
+      </c>
+      <c r="D109" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Spojovací materiál (blistry)</t>
+          <t>Barvy na zeď a nátěry</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Hmoždinky nylon 10 mm (25 ks)</t>
+          <t>Syntetický email bílý 0,6 l</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>59</v>
-      </c>
-      <c r="D110" t="inlineStr">
-        <is>
-          <t>doplnit</t>
-        </is>
+        <v>229</v>
+      </c>
+      <c r="D110" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Spojovací materiál (blistry)</t>
+          <t>Barvy na zeď a nátěry</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Hmoždinka s vrutem 6×40 a 8×60 (20 ks)</t>
+          <t>Základní barva na kov 0,6–0,75 l</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>79</v>
-      </c>
-      <c r="D111" t="inlineStr">
-        <is>
-          <t>doplnit</t>
-        </is>
+        <v>200</v>
+      </c>
+      <c r="D111" t="n">
+        <v>10</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>natloukací, na lišty</t>
+          <t>Komaprim, syntetika primer</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Spojovací materiál (blistry)</t>
+          <t>Barvy na zeď a nátěry</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Hmoždinka rámová 10×100 / 10×135 (10 ks)</t>
+          <t>Alkyton 0,7–1 l přímo na rez</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>89</v>
-      </c>
-      <c r="D112" t="inlineStr">
-        <is>
-          <t>doplnit</t>
-        </is>
+        <v>549</v>
+      </c>
+      <c r="D112" t="n">
+        <v>20</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>okna, zárubně</t>
+          <t>20 ks/měs, silná položka</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Spojovací materiál (blistry)</t>
+          <t>Barvy na zeď a nátěry</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Hmoždinka do dutin (sádrokarton) sada</t>
+          <t>Laksil bezbarvý 0,7 kg</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>79</v>
-      </c>
-      <c r="D113" t="inlineStr">
-        <is>
-          <t>doplnit</t>
-        </is>
+        <v>499</v>
+      </c>
+      <c r="D113" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Spojovací materiál (blistry)</t>
+          <t>Barvy na zeď a nátěry</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Šrouby M6 a M8 s maticí a podložkou (sada)</t>
+          <t>Míchací tyčka, sítko na lak, krycí papír</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>69</v>
-      </c>
-      <c r="D114" t="inlineStr">
-        <is>
-          <t>doplnit</t>
+        <v>15</v>
+      </c>
+      <c r="D114" t="n">
+        <v>11</v>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>drobnost k barvě, marže 110–180 %</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Spojovací materiál (blistry)</t>
+          <t>Spreje</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Matice M6/M8/M10 (sada)</t>
+          <t>Značkovací sprej FLUO oranžový</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>39</v>
-      </c>
-      <c r="D115" t="inlineStr">
-        <is>
-          <t>doplnit</t>
+        <v>215</v>
+      </c>
+      <c r="D115" t="n">
+        <v>18</v>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>nejprodávanější sprej, 18 ks/měs</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Spojovací materiál (blistry)</t>
+          <t>Spreje</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Podložky ploché a pružné (sada mix)</t>
+          <t>Sprej RAL 9005 černý mat a lesk</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>39</v>
-      </c>
-      <c r="D116" t="inlineStr">
-        <is>
-          <t>doplnit</t>
-        </is>
+        <v>119</v>
+      </c>
+      <c r="D116" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Spojovací materiál (blistry)</t>
+          <t>Spreje</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Hřebíky 40 / 60 / 80 mm (sáček 0,5 kg)</t>
+          <t>Sprej RAL 9010 bílý mat</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>49</v>
-      </c>
-      <c r="D117" t="inlineStr">
-        <is>
-          <t>doplnit</t>
-        </is>
+        <v>119</v>
+      </c>
+      <c r="D117" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Spojovací materiál (blistry)</t>
+          <t>Spreje</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Hřebíčky čalounické a lepenkové (sáček)</t>
+          <t>Sprej RAL 3002 červený</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>29</v>
-      </c>
-      <c r="D118" t="inlineStr">
-        <is>
-          <t>doplnit</t>
-        </is>
+        <v>119</v>
+      </c>
+      <c r="D118" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Spojovací materiál (blistry)</t>
+          <t>Spreje</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Závitová tyč M8 1 m</t>
+          <t>Sprej RAL 5010 modrý</t>
         </is>
       </c>
       <c r="C119" t="n">
-        <v>89</v>
-      </c>
-      <c r="D119" t="inlineStr">
-        <is>
-          <t>doplnit</t>
-        </is>
+        <v>119</v>
+      </c>
+      <c r="D119" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Spojovací materiál (blistry)</t>
+          <t>Spreje</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Skoby, háky do zdi, oka (sada)</t>
+          <t>Sprej zinek ALU (pozinkování)</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>39</v>
-      </c>
-      <c r="D120" t="inlineStr">
-        <is>
-          <t>doplnit</t>
+        <v>189</v>
+      </c>
+      <c r="D120" t="n">
+        <v>4</v>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>opravy plotů a okapů</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Spojovací materiál (blistry)</t>
+          <t>Spreje</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Zárohák (hák do zdi)</t>
+          <t>Antikorozní základ ve spreji šedý</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>69</v>
+        <v>145</v>
       </c>
       <c r="D121" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>Spojovací materiál (blistry)</t>
+          <t>Spreje</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Chemická kotva 165 / 300 ml</t>
+          <t>Žáruvzdorný sprej do 600 °C černý</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="D122" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>prodává se 7 ks/měs</t>
+          <t>kamna, komíny</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Spojovací materiál (blistry)</t>
+          <t>Spreje</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Vázací pásky 200 / 300 / 500 mm (50 ks)</t>
+          <t>Akrylový sprej profi 600 ml černý</t>
         </is>
       </c>
       <c r="C123" t="n">
-        <v>59</v>
+        <v>249</v>
       </c>
       <c r="D123" t="n">
-        <v>42</v>
-      </c>
-      <c r="E123" t="inlineStr">
-        <is>
-          <t>42 ks/měs, marže 70–190 %</t>
-        </is>
+        <v>8</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Spojovací materiál (blistry)</t>
+          <t>Spreje</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>Vázací drát pozink 50 m</t>
+          <t>Uvolňovač šroubů a rzi 400 ml</t>
         </is>
       </c>
       <c r="C124" t="n">
-        <v>49</v>
-      </c>
-      <c r="D124" t="inlineStr">
-        <is>
-          <t>doplnit</t>
-        </is>
+        <v>153</v>
+      </c>
+      <c r="D124" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Spojovací materiál (blistry)</t>
+          <t>Spreje</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Karabiny a řetěz po 1 m</t>
+          <t>Multi sprej 6 v 1 400 ml</t>
         </is>
       </c>
       <c r="C125" t="n">
-        <v>59</v>
-      </c>
-      <c r="D125" t="inlineStr">
-        <is>
-          <t>doplnit</t>
+        <v>219</v>
+      </c>
+      <c r="D125" t="n">
+        <v>2</v>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>marže 141 %</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Spojovací materiál (blistry)</t>
+          <t>Spreje</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Trhací nýty 4×10 (50 ks)</t>
+          <t>Oživovač plastů 300 ml</t>
         </is>
       </c>
       <c r="C126" t="n">
-        <v>59</v>
-      </c>
-      <c r="D126" t="inlineStr">
-        <is>
-          <t>doplnit</t>
-        </is>
+        <v>99</v>
+      </c>
+      <c r="D126" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>Barvy na zeď a nátěry</t>
+          <t>Stavebniny a suché směsi</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Het Klasik otěruvzdorný 15+3 kg</t>
+          <t>Flexibilní lepidlo na obklady a dlažbu 25 kg</t>
         </is>
       </c>
       <c r="C127" t="n">
-        <v>799</v>
+        <v>429</v>
       </c>
       <c r="D127" t="n">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>nejsilnější položka do 1 000 Kč</t>
+          <t>v datech 4 ks/měs, marže 73 %</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>Barvy na zeď a nátěry</t>
+          <t>Stavebniny a suché směsi</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Het Klasik otěruvzdorný 7+1 kg</t>
+          <t>Cement 25 kg</t>
         </is>
       </c>
       <c r="C128" t="n">
-        <v>459</v>
-      </c>
-      <c r="D128" t="n">
-        <v>3</v>
+        <v>189</v>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>sklad prodejny 2</t>
+        </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Barvy na zeď a nátěry</t>
+          <t>Stavebniny a suché směsi</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Het Klasik otěruvzdorný 4 kg</t>
+          <t>Betonová směs / pískobeton 25 kg</t>
         </is>
       </c>
       <c r="C129" t="n">
-        <v>319</v>
-      </c>
-      <c r="D129" t="n">
-        <v>2</v>
+        <v>129</v>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>Barvy na zeď a nátěry</t>
+          <t>Stavebniny a suché směsi</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>Het Klasik 1,5 kg</t>
+          <t>Sloupkobeton rychletuhnoucí 20–25 kg</t>
         </is>
       </c>
       <c r="C130" t="n">
-        <v>150</v>
-      </c>
-      <c r="D130" t="n">
-        <v>5</v>
+        <v>149</v>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>malá oprava, nejnižší cena</t>
+          <t>plotové sloupky, sušáky, vývěsky</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>Barvy na zeď a nátěry</t>
+          <t>Stavebniny a suché směsi</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>Primalex Polar 15+3 kg</t>
+          <t>Zdicí malta 25 kg</t>
         </is>
       </c>
       <c r="C131" t="n">
-        <v>999</v>
-      </c>
-      <c r="D131" t="n">
-        <v>3</v>
+        <v>129</v>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>Barvy na zeď a nátěry</t>
+          <t>Stavebniny a suché směsi</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>Primalex Polar / Standard 7,5 kg</t>
+          <t>Jádrová omítka 25 kg</t>
         </is>
       </c>
       <c r="C132" t="n">
-        <v>500</v>
+        <v>155</v>
       </c>
       <c r="D132" t="n">
-        <v>2</v>
+        <v>5</v>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>v datech 5 ks/měs</t>
+        </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>Barvy na zeď a nátěry</t>
+          <t>Stavebniny a suché směsi</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>Malířské vápno 11 kg / bílení 6 kg</t>
+          <t>Sádrová omítka G300 20 kg</t>
         </is>
       </c>
       <c r="C133" t="n">
-        <v>250</v>
+        <v>257</v>
       </c>
       <c r="D133" t="n">
-        <v>4</v>
-      </c>
-      <c r="E133" t="inlineStr">
-        <is>
-          <t>sklepy, hospodářské budovy</t>
-        </is>
+        <v>2</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>Barvy na zeď a nátěry</t>
+          <t>Stavebniny a suché směsi</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>Penetrace akrylátová 1 l</t>
+          <t>Lepicí a stěrkový tmel fasáda 25 kg</t>
         </is>
       </c>
       <c r="C134" t="n">
-        <v>69</v>
+        <v>229</v>
       </c>
       <c r="D134" t="n">
-        <v>2</v>
-      </c>
-      <c r="E134" t="inlineStr">
-        <is>
-          <t>patří k barvě, prodávat vedle</t>
-        </is>
+        <v>4</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>Barvy na zeď a nátěry</t>
+          <t>Stavebniny a suché směsi</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>Protiplísňový nátěr / Remal 7,5 kg</t>
+          <t>Spárovací hmota 5 kg (bílá, šedá)</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>533</v>
-      </c>
-      <c r="D135" t="n">
-        <v>1</v>
+        <v>189</v>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>Barvy na zeď a nátěry</t>
+          <t>Stavebniny a suché směsi</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>Bochemit proti plísním 500 ml rozprašovač</t>
+          <t>Finish tmel na sádrokarton 5 kg</t>
         </is>
       </c>
       <c r="C136" t="n">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="D136" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>Barvy na zeď a nátěry</t>
+          <t>Stavebniny a suché směsi</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>Eternal IN STOP izolační 1 kg</t>
+          <t>Uniflex štukový a akrylátový 400 g</t>
         </is>
       </c>
       <c r="C137" t="n">
-        <v>309</v>
+        <v>65</v>
       </c>
       <c r="D137" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>na skvrny a fleky</t>
+          <t>malá oprava zdi</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>Barvy na zeď a nátěry</t>
+          <t>Stavebniny a suché směsi</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>Fasádní barva Remal 7,5 kg</t>
+          <t>Penetrace 1 kg a hloubková 5 l</t>
         </is>
       </c>
       <c r="C138" t="n">
-        <v>639</v>
+        <v>84</v>
       </c>
       <c r="D138" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>jen jedna velikost</t>
+          <t>patří k omítce i k barvě</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>Barvy na zeď a nátěry</t>
+          <t>Stavebniny a suché směsi</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>Lazura na dřevo 0,75 l (palisandr, ořech, teak)</t>
+          <t>Krabice a víčka do sádrokartonu</t>
         </is>
       </c>
       <c r="C139" t="n">
-        <v>199</v>
+        <v>40</v>
       </c>
       <c r="D139" t="n">
-        <v>6</v>
-      </c>
-      <c r="E139" t="inlineStr">
-        <is>
-          <t>Luxol Originál</t>
-        </is>
+        <v>7</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>Barvy na zeď a nátěry</t>
+          <t>Stavebniny a suché směsi</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>Lak interiérový vodouředitelný 0,6 l mat a lesk</t>
+          <t>Perlinka 50 m a rohová lišta</t>
         </is>
       </c>
       <c r="C140" t="n">
-        <v>275</v>
-      </c>
-      <c r="D140" t="n">
-        <v>6</v>
+        <v>299</v>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>Barvy na zeď a nátěry</t>
+          <t>Stavebniny a suché směsi</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>Syntetický email bílý 0,6 l</t>
+          <t>Pytle na suť 120 l (3 ks)</t>
         </is>
       </c>
       <c r="C141" t="n">
-        <v>229</v>
+        <v>89</v>
       </c>
       <c r="D141" t="n">
-        <v>7</v>
+        <v>3</v>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>marže 148 %</t>
+        </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>Barvy na zeď a nátěry</t>
+          <t>Stavebniny a suché směsi</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>Základní barva na kov 0,6–0,75 l</t>
+          <t>Stavební kolečko / zednická lžíce a hladítko</t>
         </is>
       </c>
       <c r="C142" t="n">
-        <v>200</v>
-      </c>
-      <c r="D142" t="n">
-        <v>10</v>
-      </c>
-      <c r="E142" t="inlineStr">
-        <is>
-          <t>Komaprim, syntetika primer</t>
+        <v>199</v>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>doplnit</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>Barvy na zeď a nátěry</t>
+          <t>Vodoinstalace</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>Alkyton 0,7–1 l přímo na rez</t>
+          <t>Hadicové spony 8–12 / 12–20 / 16–25 / 20–32 / 25–40 / 32–50</t>
         </is>
       </c>
       <c r="C143" t="n">
-        <v>549</v>
+        <v>9</v>
       </c>
       <c r="D143" t="n">
-        <v>20</v>
+        <v>77</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>20 ks/měs, silná položka</t>
+          <t>celá řada</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>Barvy na zeď a nátěry</t>
+          <t>Vodoinstalace</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>Laksil bezbarvý 0,7 kg</t>
+          <t>Objímka trubková 2-šroub 31–38 mm</t>
         </is>
       </c>
       <c r="C144" t="n">
-        <v>499</v>
+        <v>16</v>
       </c>
       <c r="D144" t="n">
-        <v>6</v>
+        <v>25</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>Barvy na zeď a nátěry</t>
+          <t>Vodoinstalace</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>Míchací tyčka, sítko na lak, krycí papír</t>
+          <t>Objímka trubková 2-šroub 54–59 mm</t>
         </is>
       </c>
       <c r="C145" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="D145" t="n">
-        <v>11</v>
-      </c>
-      <c r="E145" t="inlineStr">
-        <is>
-          <t>drobnost k barvě, marže 110–180 %</t>
-        </is>
+        <v>14</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>Ruční nářadí</t>
+          <t>Vodoinstalace</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>Svinovací metr 5 m</t>
+          <t>Příchytka na potrubí 20 / 25 mm</t>
         </is>
       </c>
       <c r="C146" t="n">
-        <v>99</v>
+        <v>8</v>
       </c>
       <c r="D146" t="n">
-        <v>9</v>
+        <v>17</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>Ruční nářadí</t>
+          <t>Vodoinstalace</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>Odlamovací nůž 18 mm kovový</t>
+          <t>PPR koleno 90° 20 mm, T-kus 20, nátrubek 20</t>
         </is>
       </c>
       <c r="C147" t="n">
-        <v>89</v>
+        <v>8</v>
       </c>
       <c r="D147" t="n">
-        <v>7</v>
+        <v>15</v>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>jen dimenze 20 a 25</t>
+        </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>Ruční nářadí</t>
+          <t>Vodoinstalace</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>Náhradní čepele 18 mm 10 ks</t>
+          <t>Mosazná vsuvka 3/4", 1/2"</t>
         </is>
       </c>
       <c r="C148" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="D148" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>Ruční nářadí</t>
+          <t>Vodoinstalace</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Šroubovák s bity (ráčna + 20 bitů)</t>
+          <t>Tubex izolace 20×10 mm (2 m)</t>
         </is>
       </c>
       <c r="C149" t="n">
-        <v>199</v>
-      </c>
-      <c r="D149" t="inlineStr">
-        <is>
-          <t>doplnit</t>
-        </is>
+        <v>12</v>
+      </c>
+      <c r="D149" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>Ruční nářadí</t>
+          <t>Vodoinstalace</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>Kleště kombinované 180 mm</t>
+          <t>Těsnění gumová sada 1/2"–3/4"</t>
         </is>
       </c>
       <c r="C150" t="n">
-        <v>149</v>
+        <v>25</v>
       </c>
       <c r="D150" t="inlineStr">
         <is>
           <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>nejčastější havárie</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>Ruční nářadí</t>
+          <t>Vodoinstalace</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>Kladivo 300 g</t>
+          <t>Flexi hadička 3/8" 30–50 cm</t>
         </is>
       </c>
       <c r="C151" t="n">
-        <v>129</v>
+        <v>79</v>
       </c>
       <c r="D151" t="inlineStr">
         <is>
@@ -5221,54 +5205,54 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>Ruční nářadí</t>
+          <t>Vodoinstalace</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>Ocelový kartáč 5řadý</t>
+          <t>Perlátor M22/M24</t>
         </is>
       </c>
       <c r="C152" t="n">
-        <v>68</v>
-      </c>
-      <c r="D152" t="n">
-        <v>5</v>
+        <v>39</v>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>Ruční nářadí</t>
+          <t>Vodoinstalace</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>Pilka na kov / pilový list</t>
+          <t>Sprchová hadice 150 cm</t>
         </is>
       </c>
       <c r="C153" t="n">
-        <v>99</v>
-      </c>
-      <c r="D153" t="inlineStr">
-        <is>
-          <t>doplnit</t>
-        </is>
+        <v>245</v>
+      </c>
+      <c r="D153" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>Ruční nářadí</t>
+          <t>Vodoinstalace</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>Vodováha 40 cm</t>
+          <t>Sifon umyvadlový plast</t>
         </is>
       </c>
       <c r="C154" t="n">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="D154" t="inlineStr">
         <is>
@@ -5279,113 +5263,126 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>Ruční nářadí</t>
+          <t>Vodoinstalace</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>Sada imbus klíčů</t>
+          <t>Zahradní hadice 1/2" 20 m + rychlospojky</t>
         </is>
       </c>
       <c r="C155" t="n">
-        <v>89</v>
+        <v>399</v>
       </c>
       <c r="D155" t="inlineStr">
         <is>
           <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>ověřit z dat prodejny 2</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>Ruční nářadí</t>
+          <t>Spojovací materiál (blistry)</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>Zavírací nůž</t>
+          <t>Vruty do dřeva 3,5×30 (100 ks)</t>
         </is>
       </c>
       <c r="C156" t="n">
-        <v>163</v>
-      </c>
-      <c r="D156" t="n">
-        <v>4</v>
+        <v>59</v>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>nejmenší běžná velikost</t>
+        </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>Ruční nářadí</t>
+          <t>Spojovací materiál (blistry)</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>Vědro stavební 12 l</t>
+          <t>Vruty do dřeva 4×40 (100 ks)</t>
         </is>
       </c>
       <c r="C157" t="n">
-        <v>49</v>
-      </c>
-      <c r="D157" t="n">
-        <v>6</v>
+        <v>69</v>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>Ochranné pomůcky</t>
+          <t>Spojovací materiál (blistry)</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>Pracovní rukavice vel. 8 / 9 / 10 / 11</t>
+          <t>Vruty do dřeva 4×50 (100 ks)</t>
         </is>
       </c>
       <c r="C158" t="n">
-        <v>59</v>
-      </c>
-      <c r="D158" t="n">
-        <v>30</v>
-      </c>
-      <c r="E158" t="inlineStr">
-        <is>
-          <t>celá řada velikostí</t>
+        <v>79</v>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>doplnit</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>Ochranné pomůcky</t>
+          <t>Spojovací materiál (blistry)</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>Rukavice profi 1+1</t>
+          <t>Vruty do dřeva 4,5×60 (50 ks)</t>
         </is>
       </c>
       <c r="C159" t="n">
-        <v>28</v>
-      </c>
-      <c r="D159" t="n">
-        <v>5</v>
+        <v>79</v>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>Ochranné pomůcky</t>
+          <t>Spojovací materiál (blistry)</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>Jednorázové nitrilové rukavice (10 ks)</t>
+          <t>Vruty do dřeva 5×70 (50 ks)</t>
         </is>
       </c>
       <c r="C160" t="n">
-        <v>39</v>
+        <v>89</v>
       </c>
       <c r="D160" t="inlineStr">
         <is>
@@ -5396,403 +5393,443 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>Ochranné pomůcky</t>
+          <t>Spojovací materiál (blistry)</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>Zátky do uší</t>
+          <t>Vruty do dřeva 6×80 / 6×100 (25 ks)</t>
         </is>
       </c>
       <c r="C161" t="n">
-        <v>10</v>
-      </c>
-      <c r="D161" t="n">
-        <v>3</v>
+        <v>99</v>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>terasy, konstrukce</t>
+        </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>Ochranné pomůcky</t>
+          <t>Spojovací materiál (blistry)</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>Respirátor FFP2 (2 ks)</t>
+          <t>Vruty do sádrokartonu 3,5×25 a 3,5×35 (200 ks)</t>
         </is>
       </c>
       <c r="C162" t="n">
-        <v>39</v>
+        <v>79</v>
       </c>
       <c r="D162" t="inlineStr">
         <is>
           <t>doplnit</t>
-        </is>
-      </c>
-      <c r="E162" t="inlineStr">
-        <is>
-          <t>broušení, barvy</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>Ochranné pomůcky</t>
+          <t>Spojovací materiál (blistry)</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>Ochranné brýle</t>
+          <t>Šrouby do plechu 2,9×13 a 2,9×9,5 (50 ks)</t>
         </is>
       </c>
       <c r="C163" t="n">
-        <v>49</v>
-      </c>
-      <c r="D163" t="inlineStr">
-        <is>
-          <t>doplnit</t>
+        <v>29</v>
+      </c>
+      <c r="D163" t="n">
+        <v>37</v>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>v datech 37 ks/měs po 0,30–0,40 Kč</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>Technická chemie</t>
+          <t>Spojovací materiál (blistry)</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>Ředidlo S6006 0,7 l</t>
+          <t>Hmoždinky nylon 5 mm (50 ks)</t>
         </is>
       </c>
       <c r="C164" t="n">
-        <v>85</v>
-      </c>
-      <c r="D164" t="n">
-        <v>21</v>
-      </c>
-      <c r="E164" t="inlineStr">
-        <is>
-          <t>hořlavina – ověřit požární předpisy</t>
+        <v>39</v>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>doplnit</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>Technická chemie</t>
+          <t>Spojovací materiál (blistry)</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>Ředidlo S6005 0,7 l</t>
+          <t>Hmoždinky nylon 6 mm (50 ks)</t>
         </is>
       </c>
       <c r="C165" t="n">
-        <v>95</v>
-      </c>
-      <c r="D165" t="n">
-        <v>12</v>
+        <v>45</v>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>nejžádanější rozměr</t>
+        </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>Technická chemie</t>
+          <t>Spojovací materiál (blistry)</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>Nitroředidlo C6000 0,7 l</t>
+          <t>Hmoždinky nylon 8 mm (50 ks)</t>
         </is>
       </c>
       <c r="C166" t="n">
-        <v>95</v>
-      </c>
-      <c r="D166" t="n">
-        <v>9</v>
+        <v>55</v>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>Technická chemie</t>
+          <t>Spojovací materiál (blistry)</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>Líh technický 0,7 l</t>
+          <t>Hmoždinky nylon 10 mm (25 ks)</t>
         </is>
       </c>
       <c r="C167" t="n">
-        <v>98</v>
-      </c>
-      <c r="D167" t="n">
-        <v>7</v>
+        <v>59</v>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>Technická chemie</t>
+          <t>Spojovací materiál (blistry)</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>Lakový benzín 0,7 l</t>
+          <t>Hmoždinka s vrutem 6×40 a 8×60 (20 ks)</t>
         </is>
       </c>
       <c r="C168" t="n">
-        <v>109</v>
-      </c>
-      <c r="D168" t="n">
-        <v>4</v>
+        <v>79</v>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>natloukací, na lišty</t>
+        </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>Technická chemie</t>
+          <t>Spojovací materiál (blistry)</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>WD-40 / univerzální mazivo sprej 200 ml</t>
+          <t>Hmoždinka rámová 10×100 / 10×135 (10 ks)</t>
         </is>
       </c>
       <c r="C169" t="n">
-        <v>129</v>
+        <v>89</v>
       </c>
       <c r="D169" t="inlineStr">
         <is>
           <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>okna, zárubně</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>Technická chemie</t>
+          <t>Spojovací materiál (blistry)</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>Odrezovač 0,5 l</t>
+          <t>Hmoždinka do dutin (sádrokarton) sada</t>
         </is>
       </c>
       <c r="C170" t="n">
-        <v>112</v>
-      </c>
-      <c r="D170" t="n">
-        <v>3</v>
+        <v>79</v>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>Technická chemie</t>
+          <t>Spojovací materiál (blistry)</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>Kyselina citronová 100 g</t>
+          <t>Šrouby M6 a M8 s maticí a podložkou (sada)</t>
         </is>
       </c>
       <c r="C171" t="n">
-        <v>22</v>
-      </c>
-      <c r="D171" t="n">
-        <v>6</v>
+        <v>69</v>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>Technická chemie</t>
+          <t>Spojovací materiál (blistry)</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>Vazelína bílá</t>
+          <t>Matice M6/M8/M10 (sada)</t>
         </is>
       </c>
       <c r="C172" t="n">
-        <v>195</v>
-      </c>
-      <c r="D172" t="n">
-        <v>4</v>
+        <v>39</v>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>Technická chemie</t>
+          <t>Spojovací materiál (blistry)</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>Destilovaná voda 5 l</t>
+          <t>Podložky ploché a pružné (sada mix)</t>
         </is>
       </c>
       <c r="C173" t="n">
-        <v>70</v>
-      </c>
-      <c r="D173" t="n">
-        <v>6</v>
+        <v>39</v>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>Technická chemie</t>
+          <t>Spojovací materiál (blistry)</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>Nemrznoucí směs do ostřikovačů 3 l</t>
+          <t>Hřebíky 40 / 60 / 80 mm (sáček 0,5 kg)</t>
         </is>
       </c>
       <c r="C174" t="n">
-        <v>99</v>
+        <v>49</v>
       </c>
       <c r="D174" t="inlineStr">
         <is>
           <t>doplnit</t>
-        </is>
-      </c>
-      <c r="E174" t="inlineStr">
-        <is>
-          <t>sezónně</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>Úklid</t>
+          <t>Spojovací materiál (blistry)</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>Savo Original 1,2 l</t>
+          <t>Hřebíčky čalounické a lepenkové (sáček)</t>
         </is>
       </c>
       <c r="C175" t="n">
-        <v>67</v>
-      </c>
-      <c r="D175" t="n">
-        <v>5</v>
+        <v>29</v>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>Úklid</t>
+          <t>Spojovací materiál (blistry)</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>Savo proti plísni 500 ml</t>
+          <t>Závitová tyč M8 1 m</t>
         </is>
       </c>
       <c r="C176" t="n">
-        <v>99</v>
-      </c>
-      <c r="D176" t="n">
-        <v>5</v>
+        <v>89</v>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>Úklid</t>
+          <t>Spojovací materiál (blistry)</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>Domestos 750 ml / 2 l</t>
+          <t>Skoby, háky do zdi, oka (sada)</t>
         </is>
       </c>
       <c r="C177" t="n">
-        <v>59</v>
-      </c>
-      <c r="D177" t="n">
-        <v>10</v>
+        <v>39</v>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>Úklid</t>
+          <t>Spojovací materiál (blistry)</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>Jar / prostředek na nádobí 900 ml</t>
+          <t>Zárohák (hák do zdi)</t>
         </is>
       </c>
       <c r="C178" t="n">
-        <v>59</v>
-      </c>
-      <c r="D178" t="inlineStr">
-        <is>
-          <t>doplnit</t>
-        </is>
+        <v>69</v>
+      </c>
+      <c r="D178" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>Úklid</t>
+          <t>Spojovací materiál (blistry)</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>Univerzální čistič (Ajax, Cif)</t>
+          <t>Chemická kotva 165 / 300 ml</t>
         </is>
       </c>
       <c r="C179" t="n">
-        <v>59</v>
-      </c>
-      <c r="D179" t="inlineStr">
-        <is>
-          <t>doplnit</t>
+        <v>190</v>
+      </c>
+      <c r="D179" t="n">
+        <v>7</v>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>prodává se 7 ks/měs</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>Úklid</t>
+          <t>Spojovací materiál (blistry)</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>Pytle na odpad 60 l a 120 l</t>
+          <t>Vázací pásky 200 / 300 / 500 mm (50 ks)</t>
         </is>
       </c>
       <c r="C180" t="n">
-        <v>39</v>
+        <v>59</v>
       </c>
       <c r="D180" t="n">
-        <v>11</v>
+        <v>42</v>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>42 ks/měs, marže 70–190 %</t>
+        </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>Úklid</t>
+          <t>Spojovací materiál (blistry)</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>Houbičky na nádobí 5 ks</t>
+          <t>Vázací drát pozink 50 m</t>
         </is>
       </c>
       <c r="C181" t="n">
-        <v>25</v>
+        <v>49</v>
       </c>
       <c r="D181" t="inlineStr">
         <is>
@@ -5803,183 +5840,226 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>Úklid</t>
+          <t>Spojovací materiál (blistry)</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>Hadr podlahový</t>
+          <t>Karabiny a řetěz po 1 m</t>
         </is>
       </c>
       <c r="C182" t="n">
-        <v>32</v>
-      </c>
-      <c r="D182" t="n">
-        <v>4</v>
+        <v>59</v>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>Úklid</t>
+          <t>Spojovací materiál (blistry)</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>Osvěžovač vzduchu</t>
+          <t>Trhací nýty 4×10 (50 ks)</t>
         </is>
       </c>
       <c r="C183" t="n">
-        <v>29</v>
-      </c>
-      <c r="D183" t="n">
-        <v>9</v>
+        <v>59</v>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>Úklid</t>
+          <t>Spojovací materiál (blistry)</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>Solvina / Praganda (mycí pasta na ruce)</t>
+          <t>Turbošrouby do betonu 7,5×60 a 7,5×100 (10 ks)</t>
         </is>
       </c>
       <c r="C184" t="n">
-        <v>20</v>
-      </c>
-      <c r="D184" t="n">
-        <v>15</v>
+        <v>99</v>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>typicky DIY</t>
+          <t>bez hmoždinky, rychlé kotvení</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>Úklid</t>
+          <t>Spojovací materiál (blistry)</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>WC blok</t>
+          <t>Natloukací hmoždinky 6×40 a 8×60 (50 ks)</t>
         </is>
       </c>
       <c r="C185" t="n">
-        <v>39</v>
-      </c>
-      <c r="D185" t="n">
-        <v>5</v>
+        <v>79</v>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>lišty, latě</t>
+        </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>Úklid</t>
+          <t>Spojovací materiál (blistry)</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>Lopatka + smetáček</t>
+          <t>Hřebíky do betonu (sáček)</t>
         </is>
       </c>
       <c r="C186" t="n">
         <v>49</v>
       </c>
-      <c r="D186" t="n">
-        <v>6</v>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>Úklid</t>
+          <t>Spojovací materiál (blistry)</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>Zamražovací / svačinové sáčky</t>
+          <t>Tesařské úhelníky 40, 70, 90 mm</t>
         </is>
       </c>
       <c r="C187" t="n">
-        <v>39</v>
-      </c>
-      <c r="D187" t="n">
-        <v>4</v>
+        <v>25</v>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>k vrutům, časté u altánů a plotů</t>
+        </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>Hygiena</t>
+          <t>Spojovací materiál (blistry)</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>Toaletní papír Jumbo / 8 rolí</t>
+          <t>Spojka a patka sloupku 70/90 mm</t>
         </is>
       </c>
       <c r="C188" t="n">
-        <v>39</v>
-      </c>
-      <c r="D188" t="n">
-        <v>30</v>
+        <v>149</v>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>ke sloupkobetonu</t>
+        </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>Hygiena</t>
+          <t>Spojovací materiál (blistry)</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>Papírové ručníky ZZ</t>
+          <t>Vruty do dřeva 4,5×70 a 5×90 (25 ks)</t>
         </is>
       </c>
       <c r="C189" t="n">
-        <v>45</v>
-      </c>
-      <c r="D189" t="n">
-        <v>15</v>
+        <v>89</v>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>plot, terasa</t>
+        </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>Hygiena</t>
+          <t>Spojovací materiál (blistry)</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>Kapesníky krabička 150 ks</t>
+          <t>Vruty se zápustnou hlavou TORX (sada s bitem)</t>
         </is>
       </c>
       <c r="C190" t="n">
-        <v>38</v>
-      </c>
-      <c r="D190" t="n">
-        <v>3</v>
+        <v>99</v>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>bit v balení je hlavní důvod nákupu</t>
+        </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>Hygiena</t>
+          <t>Spojovací materiál (blistry)</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>Kuchyňské utěrky 2 role</t>
+          <t>Šrouby M6/M8/M10 s maticí, 60–100 mm (sada)</t>
         </is>
       </c>
       <c r="C191" t="n">
-        <v>39</v>
+        <v>89</v>
       </c>
       <c r="D191" t="inlineStr">
         <is>
@@ -5990,364 +6070,367 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>Hubení škůdců</t>
+          <t>Spojovací materiál (blistry)</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>Pastička na myši dřevo / kov</t>
+          <t>Vratové šrouby 8×80 s maticí (10 ks)</t>
         </is>
       </c>
       <c r="C192" t="n">
-        <v>16</v>
-      </c>
-      <c r="D192" t="n">
-        <v>12</v>
+        <v>79</v>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>Hubení škůdců</t>
+          <t>Spojovací materiál (blistry)</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>Nástraha na myši Ratimor 150 g</t>
+          <t>Závitová tyč M6 a M10 1 m</t>
         </is>
       </c>
       <c r="C193" t="n">
-        <v>42</v>
-      </c>
-      <c r="D193" t="n">
-        <v>8</v>
-      </c>
-      <c r="E193" t="inlineStr">
-        <is>
-          <t>balení pro veřejnost</t>
+        <v>99</v>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>doplnit</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>Hubení škůdců</t>
+          <t>Spojovací materiál (blistry)</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>Lepová deska na myši</t>
+          <t>Trhací nýty 3,2 a 4,8 mm (50 ks)</t>
         </is>
       </c>
       <c r="C194" t="n">
-        <v>35</v>
-      </c>
-      <c r="D194" t="n">
-        <v>3</v>
+        <v>59</v>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>Hubení škůdců</t>
+          <t>Spojovací materiál (blistry)</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>Mucholapka</t>
+          <t>Sponky do sponkovačky typ G 10–12 mm</t>
         </is>
       </c>
       <c r="C195" t="n">
-        <v>7</v>
-      </c>
-      <c r="D195" t="n">
-        <v>4</v>
+        <v>59</v>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>Hubení škůdců</t>
+          <t>Spojovací materiál (blistry)</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>Feroset – lapač moučných molů</t>
+          <t>Šroub s okem a vrut s hákem (sada)</t>
         </is>
       </c>
       <c r="C196" t="n">
-        <v>16</v>
-      </c>
-      <c r="D196" t="n">
-        <v>8</v>
+        <v>45</v>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>Hubení škůdců</t>
+          <t>Ruční nářadí</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>Sprej na vosy / hmyz (Biolit)</t>
+          <t>Svinovací metr 5 m</t>
         </is>
       </c>
       <c r="C197" t="n">
-        <v>119</v>
-      </c>
-      <c r="D197" t="inlineStr">
-        <is>
-          <t>doplnit</t>
-        </is>
-      </c>
-      <c r="E197" t="inlineStr">
-        <is>
-          <t>léto</t>
-        </is>
+        <v>99</v>
+      </c>
+      <c r="D197" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>Hubení škůdců</t>
+          <t>Ruční nářadí</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>Proti mravencům (Bioformatox)</t>
+          <t>Odlamovací nůž 18 mm kovový</t>
         </is>
       </c>
       <c r="C198" t="n">
-        <v>109</v>
+        <v>89</v>
       </c>
       <c r="D198" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>Topení a zapalování</t>
+          <t>Ruční nářadí</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>Pepo pevný podpalovač 40 ks</t>
+          <t>Náhradní čepele 18 mm 10 ks</t>
         </is>
       </c>
       <c r="C199" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="D199" t="n">
-        <v>29</v>
-      </c>
-      <c r="E199" t="inlineStr">
-        <is>
-          <t>celoročně</t>
-        </is>
+        <v>12</v>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>Topení a zapalování</t>
+          <t>Ruční nářadí</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>Tekutý podpalovač 1 l</t>
+          <t>Šroubovák s bity (ráčna + 20 bitů)</t>
         </is>
       </c>
       <c r="C200" t="n">
-        <v>96</v>
-      </c>
-      <c r="D200" t="n">
-        <v>3</v>
+        <v>199</v>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>Topení a zapalování</t>
+          <t>Ruční nářadí</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>Zapalovač kuchyňský dlouhý</t>
+          <t>Kleště kombinované 180 mm</t>
         </is>
       </c>
       <c r="C201" t="n">
-        <v>37</v>
-      </c>
-      <c r="D201" t="n">
-        <v>3</v>
+        <v>149</v>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>Topení a zapalování</t>
+          <t>Ruční nářadí</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>Zapalovače turbo (2 ks)</t>
+          <t>Kladivo 300 g</t>
         </is>
       </c>
       <c r="C202" t="n">
-        <v>15</v>
-      </c>
-      <c r="D202" t="n">
-        <v>4</v>
+        <v>129</v>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>Topení a zapalování</t>
+          <t>Ruční nářadí</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>Zápalky (balení 10 krabiček)</t>
+          <t>Ocelový kartáč 5řadý</t>
         </is>
       </c>
       <c r="C203" t="n">
-        <v>25</v>
+        <v>68</v>
       </c>
       <c r="D203" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>Topení a zapalování</t>
+          <t>Ruční nářadí</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>Dřevěné uhlí 2,5 kg</t>
+          <t>Pilka na kov / pilový list</t>
         </is>
       </c>
       <c r="C204" t="n">
-        <v>112</v>
-      </c>
-      <c r="D204" t="n">
-        <v>3</v>
-      </c>
-      <c r="E204" t="inlineStr">
-        <is>
-          <t>sezónně</t>
+        <v>99</v>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>doplnit</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>Svíčky</t>
+          <t>Ruční nářadí</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>Hřbitovní patrona 120 g a 180 g</t>
+          <t>Vodováha 40 cm</t>
         </is>
       </c>
       <c r="C205" t="n">
-        <v>28</v>
-      </c>
-      <c r="D205" t="n">
-        <v>18</v>
+        <v>99</v>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>Svíčky</t>
+          <t>Ruční nářadí</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>Svíčka Theresia 4,5 dne</t>
+          <t>Sada imbus klíčů</t>
         </is>
       </c>
       <c r="C206" t="n">
-        <v>47</v>
-      </c>
-      <c r="D206" t="n">
-        <v>3</v>
+        <v>89</v>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>Svíčky</t>
+          <t>Ruční nářadí</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>Iluminační svíčky 10 ks</t>
+          <t>Zavírací nůž</t>
         </is>
       </c>
       <c r="C207" t="n">
-        <v>59</v>
+        <v>163</v>
       </c>
       <c r="D207" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>Svíčky</t>
+          <t>Ruční nářadí</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>Čajové svíčky 30 ks</t>
+          <t>Vědro stavební 12 l</t>
         </is>
       </c>
       <c r="C208" t="n">
         <v>49</v>
       </c>
-      <c r="D208" t="inlineStr">
-        <is>
-          <t>doplnit</t>
-        </is>
+      <c r="D208" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>Domácnost</t>
+          <t>Ochranné pomůcky</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>Skřipce záclonové</t>
+          <t>Pracovní rukavice vel. 8 / 9 / 10 / 11</t>
         </is>
       </c>
       <c r="C209" t="n">
-        <v>6</v>
+        <v>59</v>
       </c>
       <c r="D209" t="n">
-        <v>22</v>
+        <v>30</v>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>celá řada velikostí</t>
+        </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>Domácnost</t>
+          <t>Ochranné pomůcky</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>Háčky samolepicí</t>
+          <t>Rukavice profi 1+1</t>
         </is>
       </c>
       <c r="C210" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D210" t="n">
         <v>5</v>
@@ -6356,74 +6439,79 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>Domácnost</t>
+          <t>Ochranné pomůcky</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>Věšák nástěnný chrom</t>
+          <t>Jednorázové nitrilové rukavice (10 ks)</t>
         </is>
       </c>
       <c r="C211" t="n">
-        <v>62</v>
-      </c>
-      <c r="D211" t="n">
-        <v>10</v>
+        <v>39</v>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>Domácnost</t>
+          <t>Ochranné pomůcky</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>Kolíčky na prádlo 24 ks</t>
+          <t>Zátky do uší</t>
         </is>
       </c>
       <c r="C212" t="n">
-        <v>39</v>
-      </c>
-      <c r="D212" t="inlineStr">
-        <is>
-          <t>doplnit</t>
-        </is>
+        <v>10</v>
+      </c>
+      <c r="D212" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>Domácnost</t>
+          <t>Ochranné pomůcky</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>Prádelní šňůra 20 m</t>
+          <t>Respirátor FFP2 (2 ks)</t>
         </is>
       </c>
       <c r="C213" t="n">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="D213" t="inlineStr">
         <is>
           <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>broušení, barvy</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>Domácnost</t>
+          <t>Ochranné pomůcky</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>Provázek / polypropylenové lano 20 m</t>
+          <t>Ochranné brýle</t>
         </is>
       </c>
       <c r="C214" t="n">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="D214" t="inlineStr">
         <is>
@@ -6434,153 +6522,883 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>Domácnost</t>
+          <t>Technická chemie</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>Kroužky na klíče + rozlišovače</t>
+          <t>Ředidlo S6006 0,7 l</t>
         </is>
       </c>
       <c r="C215" t="n">
-        <v>4</v>
+        <v>85</v>
       </c>
       <c r="D215" t="n">
-        <v>46</v>
+        <v>21</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
-          <t>u pokladny</t>
+          <t>hořlavina – ověřit požární předpisy</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>Domácnost</t>
+          <t>Technická chemie</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>Visací zámek 30 / 40 mm</t>
+          <t>Ředidlo S6005 0,7 l</t>
         </is>
       </c>
       <c r="C216" t="n">
-        <v>129</v>
-      </c>
-      <c r="D216" t="inlineStr">
-        <is>
-          <t>doplnit</t>
-        </is>
+        <v>95</v>
+      </c>
+      <c r="D216" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>Domácnost</t>
+          <t>Technická chemie</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>Magnety 10 ks</t>
+          <t>Nitroředidlo C6000 0,7 l</t>
         </is>
       </c>
       <c r="C217" t="n">
-        <v>50</v>
+        <v>95</v>
       </c>
       <c r="D217" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>Sezónní stojan (rotace)</t>
+          <t>Technická chemie</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>Semena zeleniny a květin (stojan)</t>
+          <t>Líh technický 0,7 l</t>
         </is>
       </c>
       <c r="C218" t="n">
-        <v>25</v>
+        <v>98</v>
       </c>
       <c r="D218" t="n">
-        <v>153</v>
-      </c>
-      <c r="E218" t="inlineStr">
-        <is>
-          <t>únor–květen, marže 40–100 %</t>
-        </is>
+        <v>7</v>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>Sezónní stojan (rotace)</t>
+          <t>Technická chemie</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>Barvy na vejce, obtisky</t>
+          <t>Lakový benzín 0,7 l</t>
         </is>
       </c>
       <c r="C219" t="n">
-        <v>12</v>
+        <v>109</v>
       </c>
       <c r="D219" t="n">
-        <v>15</v>
-      </c>
-      <c r="E219" t="inlineStr">
-        <is>
-          <t>březen–duben</t>
-        </is>
+        <v>4</v>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>Sezónní stojan (rotace)</t>
+          <t>Technická chemie</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>Zavařovací víčka Twist, špejle, střeva</t>
+          <t>WD-40 / univerzální mazivo sprej 200 ml</t>
         </is>
       </c>
       <c r="C220" t="n">
-        <v>40</v>
-      </c>
-      <c r="D220" t="n">
-        <v>15</v>
-      </c>
-      <c r="E220" t="inlineStr">
-        <is>
-          <t>červenec–říjen</t>
+        <v>129</v>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>doplnit</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
+          <t>Technická chemie</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>Odrezovač 0,5 l</t>
+        </is>
+      </c>
+      <c r="C221" t="n">
+        <v>112</v>
+      </c>
+      <c r="D221" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>Technická chemie</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>Kyselina citronová 100 g</t>
+        </is>
+      </c>
+      <c r="C222" t="n">
+        <v>22</v>
+      </c>
+      <c r="D222" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>Technická chemie</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>Vazelína bílá</t>
+        </is>
+      </c>
+      <c r="C223" t="n">
+        <v>195</v>
+      </c>
+      <c r="D223" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>Technická chemie</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>Destilovaná voda 5 l</t>
+        </is>
+      </c>
+      <c r="C224" t="n">
+        <v>70</v>
+      </c>
+      <c r="D224" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>Technická chemie</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>Nemrznoucí směs do ostřikovačů 3 l</t>
+        </is>
+      </c>
+      <c r="C225" t="n">
+        <v>99</v>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>sezónně</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>Hygiena</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>Toaletní papír Jumbo / 8 rolí</t>
+        </is>
+      </c>
+      <c r="C226" t="n">
+        <v>39</v>
+      </c>
+      <c r="D226" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>Hygiena</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>Papírové ručníky ZZ</t>
+        </is>
+      </c>
+      <c r="C227" t="n">
+        <v>45</v>
+      </c>
+      <c r="D227" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>Hygiena</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>Kapesníky krabička 150 ks</t>
+        </is>
+      </c>
+      <c r="C228" t="n">
+        <v>38</v>
+      </c>
+      <c r="D228" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>Hygiena</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>Kuchyňské utěrky 2 role</t>
+        </is>
+      </c>
+      <c r="C229" t="n">
+        <v>39</v>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>Hubení škůdců</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>Pastička na myši dřevo / kov</t>
+        </is>
+      </c>
+      <c r="C230" t="n">
+        <v>16</v>
+      </c>
+      <c r="D230" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>Hubení škůdců</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>Nástraha na myši Ratimor 150 g</t>
+        </is>
+      </c>
+      <c r="C231" t="n">
+        <v>42</v>
+      </c>
+      <c r="D231" t="n">
+        <v>8</v>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>balení pro veřejnost</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>Hubení škůdců</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>Lepová deska na myši</t>
+        </is>
+      </c>
+      <c r="C232" t="n">
+        <v>35</v>
+      </c>
+      <c r="D232" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>Hubení škůdců</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>Mucholapka</t>
+        </is>
+      </c>
+      <c r="C233" t="n">
+        <v>7</v>
+      </c>
+      <c r="D233" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>Hubení škůdců</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>Feroset – lapač moučných molů</t>
+        </is>
+      </c>
+      <c r="C234" t="n">
+        <v>16</v>
+      </c>
+      <c r="D234" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>Hubení škůdců</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>Sprej na vosy / hmyz (Biolit)</t>
+        </is>
+      </c>
+      <c r="C235" t="n">
+        <v>119</v>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>léto</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>Hubení škůdců</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>Proti mravencům (Bioformatox)</t>
+        </is>
+      </c>
+      <c r="C236" t="n">
+        <v>109</v>
+      </c>
+      <c r="D236" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>Topení a zapalování</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>Pepo pevný podpalovač 40 ks</t>
+        </is>
+      </c>
+      <c r="C237" t="n">
+        <v>35</v>
+      </c>
+      <c r="D237" t="n">
+        <v>29</v>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>celoročně</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>Topení a zapalování</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>Tekutý podpalovač 1 l</t>
+        </is>
+      </c>
+      <c r="C238" t="n">
+        <v>96</v>
+      </c>
+      <c r="D238" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>Topení a zapalování</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>Zapalovač kuchyňský dlouhý</t>
+        </is>
+      </c>
+      <c r="C239" t="n">
+        <v>37</v>
+      </c>
+      <c r="D239" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>Topení a zapalování</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>Zapalovače turbo (2 ks)</t>
+        </is>
+      </c>
+      <c r="C240" t="n">
+        <v>15</v>
+      </c>
+      <c r="D240" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>Topení a zapalování</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>Zápalky (balení 10 krabiček)</t>
+        </is>
+      </c>
+      <c r="C241" t="n">
+        <v>25</v>
+      </c>
+      <c r="D241" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>Topení a zapalování</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>Dřevěné uhlí 2,5 kg</t>
+        </is>
+      </c>
+      <c r="C242" t="n">
+        <v>112</v>
+      </c>
+      <c r="D242" t="n">
+        <v>3</v>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>sezónně</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>Svíčky</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>Hřbitovní patrona 120 g a 180 g</t>
+        </is>
+      </c>
+      <c r="C243" t="n">
+        <v>28</v>
+      </c>
+      <c r="D243" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>Svíčky</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>Svíčka Theresia 4,5 dne</t>
+        </is>
+      </c>
+      <c r="C244" t="n">
+        <v>47</v>
+      </c>
+      <c r="D244" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>Svíčky</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>Iluminační svíčky 10 ks</t>
+        </is>
+      </c>
+      <c r="C245" t="n">
+        <v>59</v>
+      </c>
+      <c r="D245" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>Svíčky</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>Čajové svíčky 30 ks</t>
+        </is>
+      </c>
+      <c r="C246" t="n">
+        <v>49</v>
+      </c>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>Domácnost</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>Skřipce záclonové</t>
+        </is>
+      </c>
+      <c r="C247" t="n">
+        <v>6</v>
+      </c>
+      <c r="D247" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>Domácnost</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>Háčky samolepicí</t>
+        </is>
+      </c>
+      <c r="C248" t="n">
+        <v>30</v>
+      </c>
+      <c r="D248" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>Domácnost</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>Věšák nástěnný chrom</t>
+        </is>
+      </c>
+      <c r="C249" t="n">
+        <v>62</v>
+      </c>
+      <c r="D249" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>Domácnost</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>Kolíčky na prádlo 24 ks</t>
+        </is>
+      </c>
+      <c r="C250" t="n">
+        <v>39</v>
+      </c>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>Domácnost</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>Prádelní šňůra 20 m</t>
+        </is>
+      </c>
+      <c r="C251" t="n">
+        <v>49</v>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>Domácnost</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>Provázek / polypropylenové lano 20 m</t>
+        </is>
+      </c>
+      <c r="C252" t="n">
+        <v>59</v>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>Domácnost</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>Kroužky na klíče + rozlišovače</t>
+        </is>
+      </c>
+      <c r="C253" t="n">
+        <v>4</v>
+      </c>
+      <c r="D253" t="n">
+        <v>46</v>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>u pokladny</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>Domácnost</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>Visací zámek 30 / 40 mm</t>
+        </is>
+      </c>
+      <c r="C254" t="n">
+        <v>129</v>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>doplnit</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>Domácnost</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>Magnety 10 ks</t>
+        </is>
+      </c>
+      <c r="C255" t="n">
+        <v>50</v>
+      </c>
+      <c r="D255" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
           <t>Sezónní stojan (rotace)</t>
         </is>
       </c>
-      <c r="B221" t="inlineStr">
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>Semena zeleniny a květin (stojan)</t>
+        </is>
+      </c>
+      <c r="C256" t="n">
+        <v>25</v>
+      </c>
+      <c r="D256" t="n">
+        <v>153</v>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>únor–květen, marže 40–100 %</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>Sezónní stojan (rotace)</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>Barvy na vejce, obtisky</t>
+        </is>
+      </c>
+      <c r="C257" t="n">
+        <v>12</v>
+      </c>
+      <c r="D257" t="n">
+        <v>15</v>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>březen–duben</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>Sezónní stojan (rotace)</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>Zavařovací víčka Twist, špejle, střeva</t>
+        </is>
+      </c>
+      <c r="C258" t="n">
+        <v>40</v>
+      </c>
+      <c r="D258" t="n">
+        <v>15</v>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>červenec–říjen</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>Sezónní stojan (rotace)</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
         <is>
           <t>Posypová sůl 5 kg, škrabka na led</t>
         </is>
       </c>
-      <c r="C221" t="n">
+      <c r="C259" t="n">
         <v>79</v>
       </c>
-      <c r="D221" t="inlineStr">
+      <c r="D259" t="inlineStr">
         <is>
           <t>doplnit</t>
         </is>
       </c>
-      <c r="E221" t="inlineStr">
+      <c r="E259" t="inlineStr">
         <is>
           <t>listopad–únor</t>
         </is>

</xml_diff>